<commit_message>
feat: add note fields to Pour & Separate stages and update Sample plan
</commit_message>
<xml_diff>
--- a/Kế hoach sản xuất Sample.xlsx
+++ b/Kế hoach sản xuất Sample.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ortholitevietnam-my.sharepoint.com/personal/lam_dv2_ortholite_vn/Documents/PROJECT LÂM/DailyFoamingReport/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C12FF075-160F-4BB4-977C-4D56BABB08BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="8_{C12FF075-160F-4BB4-977C-4D56BABB08BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{62512D36-052B-42F4-BEC0-D335AD8826F4}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{E780E912-92A1-4ADF-95B1-638FE58CE194}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{E780E912-92A1-4ADF-95B1-638FE58CE194}"/>
   </bookViews>
   <sheets>
     <sheet name="13.5" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'13.5'!$A$2:$N$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'15.5'!$A$2:$N$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'18.5'!$A$2:$N$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'18.5'!$A$2:$N$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'20.5'!$A$2:$N$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'21.5'!$A$2:$N$19</definedName>
     <definedName name="AE" localSheetId="0">'[1]Molding-báo cáo BUn'!#REF!</definedName>
@@ -33215,7 +33215,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DFB7AE26-D39B-4A79-A937-205FFF1964B5}">
-  <sheetPr filterMode="1">
+  <sheetPr>
     <tabColor theme="4"/>
   </sheetPr>
   <dimension ref="A1:N664"/>
@@ -33580,7 +33580,7 @@
         <v>46162</v>
       </c>
     </row>
-    <row r="12" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="17"/>
       <c r="B12" s="18" t="e">
         <f>VLOOKUP(A12,'[2]master plan'!A:C,3,0)</f>
@@ -33629,7 +33629,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="17"/>
       <c r="B13" s="18" t="e">
         <f>VLOOKUP(A13,'[2]master plan'!A:C,3,0)</f>
@@ -33678,7 +33678,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="17"/>
       <c r="B14" s="18" t="e">
         <f>VLOOKUP(A14,'[2]master plan'!A:C,3,0)</f>
@@ -33727,7 +33727,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="17"/>
       <c r="B15" s="18" t="e">
         <f>VLOOKUP(A15,'[2]master plan'!A:C,3,0)</f>
@@ -33776,7 +33776,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="17"/>
       <c r="B16" s="18" t="e">
         <f>VLOOKUP(A16,'[2]master plan'!A:C,3,0)</f>
@@ -33825,7 +33825,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="17"/>
       <c r="B17" s="18" t="e">
         <f>VLOOKUP(A17,'[2]master plan'!A:C,3,0)</f>
@@ -33874,7 +33874,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="17"/>
       <c r="B18" s="18" t="e">
         <f>VLOOKUP(A18,'[2]master plan'!A:C,3,0)</f>
@@ -33923,7 +33923,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="17"/>
       <c r="B19" s="18" t="e">
         <f>VLOOKUP(A19,'[2]master plan'!A:C,3,0)</f>
@@ -33972,7 +33972,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="17"/>
       <c r="B20" s="18" t="e">
         <f>VLOOKUP(A20,'[2]master plan'!A:C,3,0)</f>
@@ -34534,17 +34534,7 @@
   <protectedRanges>
     <protectedRange algorithmName="SHA-512" hashValue="e1FOu1UlwA7reaiyQlEGzbU6dAFPyHPlKfgo6VzFBBobawyOfUsh2c/+wjC8bICpcXVPmRerMGA9+qKsw5p7Iw==" saltValue="UD2tVZrxqZTGI3vDzMBrHw==" spinCount="100000" sqref="E12:E20 E3:E11" name="Range1_1"/>
   </protectedRanges>
-  <autoFilter ref="A2:N21" xr:uid="{E2BC4C4A-3703-4A99-A30B-53817C3A378F}">
-    <filterColumn colId="1">
-      <filters blank="1">
-        <filter val="RPRO-260513-0945"/>
-        <filter val="RPRO-260513-0946"/>
-        <filter val="RPRO-260513-0947"/>
-        <filter val="RPRO-260513-0949"/>
-        <filter val="RPRO-260513-0950"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A2:N21" xr:uid="{E2BC4C4A-3703-4A99-A30B-53817C3A378F}"/>
   <mergeCells count="1">
     <mergeCell ref="D1:F1"/>
   </mergeCells>
@@ -34581,7 +34571,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38F5428D-F8E8-4268-960E-0C7709324729}">
-  <sheetPr filterMode="1">
+  <sheetPr>
     <tabColor theme="4"/>
   </sheetPr>
   <dimension ref="A1:N667"/>
@@ -34610,7 +34600,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46163.878920370371</v>
+        <v>46163.886088888888</v>
       </c>
       <c r="D1" s="62" t="s">
         <v>1</v>
@@ -35147,7 +35137,7 @@
         <v>46164</v>
       </c>
     </row>
-    <row r="18" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="17"/>
       <c r="B18" s="18" t="e">
         <f>VLOOKUP(A18,'[2]master plan'!A:C,3,0)</f>
@@ -35196,7 +35186,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="17"/>
       <c r="B19" s="18" t="e">
         <f>VLOOKUP(A19,'[2]master plan'!A:C,3,0)</f>
@@ -35245,7 +35235,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="17"/>
       <c r="B20" s="18" t="e">
         <f>VLOOKUP(A20,'[2]master plan'!A:C,3,0)</f>
@@ -35294,7 +35284,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="17"/>
       <c r="B21" s="18" t="e">
         <f>VLOOKUP(A21,'[2]master plan'!A:C,3,0)</f>
@@ -35343,7 +35333,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="17"/>
       <c r="B22" s="18" t="e">
         <f>VLOOKUP(A22,'[2]master plan'!A:C,3,0)</f>
@@ -35392,7 +35382,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="17"/>
       <c r="B23" s="18" t="e">
         <f>VLOOKUP(A23,'[2]master plan'!A:C,3,0)</f>
@@ -35954,21 +35944,7 @@
   <protectedRanges>
     <protectedRange algorithmName="SHA-512" hashValue="e1FOu1UlwA7reaiyQlEGzbU6dAFPyHPlKfgo6VzFBBobawyOfUsh2c/+wjC8bICpcXVPmRerMGA9+qKsw5p7Iw==" saltValue="UD2tVZrxqZTGI3vDzMBrHw==" spinCount="100000" sqref="E3:E23" name="Range1_1"/>
   </protectedRanges>
-  <autoFilter ref="A2:N24" xr:uid="{E2BC4C4A-3703-4A99-A30B-53817C3A378F}">
-    <filterColumn colId="1">
-      <filters blank="1">
-        <filter val="RPRO-260515-0272"/>
-        <filter val="RPRO-260515-0273"/>
-        <filter val="RPRO-260515-0274"/>
-        <filter val="RPRO-260515-0275"/>
-        <filter val="RPRO-260515-0276"/>
-        <filter val="RPRO-260515-0277"/>
-        <filter val="RPRO-260515-0278"/>
-        <filter val="RPRO-260515-0279"/>
-        <filter val="RPRO-260515-0280"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A2:N24" xr:uid="{E2BC4C4A-3703-4A99-A30B-53817C3A378F}"/>
   <mergeCells count="1">
     <mergeCell ref="D1:F1"/>
   </mergeCells>
@@ -36034,7 +36010,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46163.878920370371</v>
+        <v>46163.886088888888</v>
       </c>
       <c r="D1" s="62" t="s">
         <v>1</v>
@@ -37414,7 +37390,7 @@
   <protectedRanges>
     <protectedRange algorithmName="SHA-512" hashValue="e1FOu1UlwA7reaiyQlEGzbU6dAFPyHPlKfgo6VzFBBobawyOfUsh2c/+wjC8bICpcXVPmRerMGA9+qKsw5p7Iw==" saltValue="UD2tVZrxqZTGI3vDzMBrHw==" spinCount="100000" sqref="E3:E28" name="Range1_1"/>
   </protectedRanges>
-  <autoFilter ref="A2:N29" xr:uid="{E2BC4C4A-3703-4A99-A30B-53817C3A378F}"/>
+  <autoFilter ref="A2:N3" xr:uid="{C37AD070-2916-43CC-A604-A8704404E33C}"/>
   <mergeCells count="1">
     <mergeCell ref="D1:F1"/>
   </mergeCells>
@@ -37480,7 +37456,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46163.878920370371</v>
+        <v>46163.886088888888</v>
       </c>
       <c r="D1" s="62" t="s">
         <v>1</v>
@@ -38869,7 +38845,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB7B6BC1-AB47-4E1B-BA30-0BF2D008E387}">
-  <sheetPr filterMode="1">
+  <sheetPr>
     <tabColor theme="4"/>
   </sheetPr>
   <dimension ref="A1:N662"/>
@@ -38883,8 +38859,7 @@
     <col min="6" max="6" width="19.1796875" style="54" customWidth="1"/>
     <col min="7" max="7" width="19" style="54" customWidth="1"/>
     <col min="8" max="8" width="17.1796875" style="55" customWidth="1"/>
-    <col min="9" max="9" width="20.1796875" style="53" customWidth="1"/>
-    <col min="10" max="10" width="20.1796875" style="53" hidden="1" customWidth="1"/>
+    <col min="9" max="10" width="20.1796875" style="53" customWidth="1"/>
     <col min="11" max="11" width="25.7265625" style="53" customWidth="1"/>
     <col min="12" max="12" width="21.453125" style="61" customWidth="1"/>
     <col min="13" max="13" width="22" style="57" customWidth="1"/>
@@ -38898,7 +38873,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46163.878920370371</v>
+        <v>46163.886088888888</v>
       </c>
       <c r="D1" s="62" t="s">
         <v>1</v>
@@ -39061,7 +39036,7 @@
         <v>46167</v>
       </c>
     </row>
-    <row r="6" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="17"/>
       <c r="B6" s="18" t="e">
         <f>VLOOKUP(A6,'[2]master plan'!A:C,3,0)</f>
@@ -39110,7 +39085,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="17"/>
       <c r="B7" s="18" t="e">
         <f>VLOOKUP(A7,'[2]master plan'!A:C,3,0)</f>
@@ -39159,7 +39134,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="17"/>
       <c r="B8" s="18" t="e">
         <f>VLOOKUP(A8,'[2]master plan'!A:C,3,0)</f>
@@ -39208,7 +39183,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="17"/>
       <c r="B9" s="18" t="e">
         <f>VLOOKUP(A9,'[2]master plan'!A:C,3,0)</f>
@@ -39257,7 +39232,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="17"/>
       <c r="B10" s="18" t="e">
         <f>VLOOKUP(A10,'[2]master plan'!A:C,3,0)</f>
@@ -39306,7 +39281,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="17"/>
       <c r="B11" s="18" t="e">
         <f>VLOOKUP(A11,'[2]master plan'!A:C,3,0)</f>
@@ -39355,7 +39330,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="17"/>
       <c r="B12" s="18" t="e">
         <f>VLOOKUP(A12,'[2]master plan'!A:C,3,0)</f>
@@ -39404,7 +39379,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="17"/>
       <c r="B13" s="18" t="e">
         <f>VLOOKUP(A13,'[2]master plan'!A:C,3,0)</f>
@@ -39453,7 +39428,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="17"/>
       <c r="B14" s="18" t="e">
         <f>VLOOKUP(A14,'[2]master plan'!A:C,3,0)</f>
@@ -39502,7 +39477,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="17"/>
       <c r="B15" s="18" t="e">
         <f>VLOOKUP(A15,'[2]master plan'!A:C,3,0)</f>
@@ -39551,7 +39526,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="17"/>
       <c r="B16" s="18" t="e">
         <f>VLOOKUP(A16,'[2]master plan'!A:C,3,0)</f>
@@ -39600,7 +39575,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="17"/>
       <c r="B17" s="18" t="e">
         <f>VLOOKUP(A17,'[2]master plan'!A:C,3,0)</f>
@@ -39649,7 +39624,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="17"/>
       <c r="B18" s="18" t="e">
         <f>VLOOKUP(A18,'[2]master plan'!A:C,3,0)</f>
@@ -40211,14 +40186,7 @@
   <protectedRanges>
     <protectedRange algorithmName="SHA-512" hashValue="e1FOu1UlwA7reaiyQlEGzbU6dAFPyHPlKfgo6VzFBBobawyOfUsh2c/+wjC8bICpcXVPmRerMGA9+qKsw5p7Iw==" saltValue="UD2tVZrxqZTGI3vDzMBrHw==" spinCount="100000" sqref="E3:E18" name="Range1_1"/>
   </protectedRanges>
-  <autoFilter ref="A2:N19" xr:uid="{E2BC4C4A-3703-4A99-A30B-53817C3A378F}">
-    <filterColumn colId="1">
-      <filters blank="1">
-        <filter val="RPRO-260521-0669"/>
-        <filter val="RPRO-260521-0670"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A2:N19" xr:uid="{E2BC4C4A-3703-4A99-A30B-53817C3A378F}"/>
   <mergeCells count="1">
     <mergeCell ref="D1:F1"/>
   </mergeCells>

</xml_diff>

<commit_message>
fix: tinh do day bun trung binh theo ngay thay vi tung don
</commit_message>
<xml_diff>
--- a/Kế hoach sản xuất Sample.xlsx
+++ b/Kế hoach sản xuất Sample.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ortholitevietnam-my.sharepoint.com/personal/lam_dv2_ortholite_vn/Documents/PROJECT LÂM/DailyFoamingReport/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="8_{C12FF075-160F-4BB4-977C-4D56BABB08BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{62512D36-052B-42F4-BEC0-D335AD8826F4}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="8_{C12FF075-160F-4BB4-977C-4D56BABB08BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D762CD4A-EFE7-44D7-9ED4-B9E5074D5C65}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{E780E912-92A1-4ADF-95B1-638FE58CE194}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{E780E912-92A1-4ADF-95B1-638FE58CE194}"/>
   </bookViews>
   <sheets>
     <sheet name="13.5" sheetId="1" r:id="rId1"/>
@@ -171,7 +171,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="247">
   <si>
     <t>Release Date</t>
   </si>
@@ -641,9 +641,6 @@
     <t>SSO-2605-00716</t>
   </si>
   <si>
-    <t>OV-0435</t>
-  </si>
-  <si>
     <t>S-2026-05-47</t>
   </si>
   <si>
@@ -677,9 +674,6 @@
     <t>SSO-2605-00651</t>
   </si>
   <si>
-    <t>OE-0111A</t>
-  </si>
-  <si>
     <t>S-2026-05-49</t>
   </si>
   <si>
@@ -693,9 +687,6 @@
   </si>
   <si>
     <t>OrthoLite Regular GREY/17-1501TPX Flat Sheet 0.11D 5-10 Asker C 1.1M 2M 3.5mm</t>
-  </si>
-  <si>
-    <t>OV-0272</t>
   </si>
   <si>
     <t>S-2026-05-50</t>
@@ -719,9 +710,6 @@
     <t>SSO-2605-00721</t>
   </si>
   <si>
-    <t>OV-0112</t>
-  </si>
-  <si>
     <t>S-2026-05-51</t>
   </si>
   <si>
@@ -735,9 +723,6 @@
   </si>
   <si>
     <t>SSO-2605-00722</t>
-  </si>
-  <si>
-    <t>OV-0085</t>
   </si>
   <si>
     <t>S-2026-05-53</t>
@@ -864,9 +849,6 @@
   </si>
   <si>
     <t>OrthoLite Regular-Nike SEEDPEARL/12-0703TPX Flat Sheet 0.11D 25+/-4 Asker C 1.1M 1.7M 2mm</t>
-  </si>
-  <si>
-    <t>DIE CUT</t>
   </si>
   <si>
     <t>S-2026-05-63</t>
@@ -1005,6 +987,9 @@
   </si>
   <si>
     <t>SSO-2605-01133   - URGENT (5-28)</t>
+  </si>
+  <si>
+    <t>OK</t>
   </si>
 </sst>
 </file>
@@ -1539,9 +1524,6 @@
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="21" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1586,6 +1568,9 @@
     </xf>
     <xf numFmtId="14" fontId="25" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2117,8 +2102,8 @@
       <sheetName val="form 2 (11)"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
+      <sheetData sheetId="0" refreshError="1"/>
+      <sheetData sheetId="1" refreshError="1"/>
       <sheetData sheetId="2">
         <row r="1">
           <cell r="C1" t="str">
@@ -32488,7 +32473,7 @@
             <v xml:space="preserve">PUR2605210001S  </v>
           </cell>
           <cell r="E447" t="str">
-            <v/>
+            <v>BDB-000058</v>
           </cell>
           <cell r="F447" t="str">
             <v>PVN-001319</v>
@@ -32506,7 +32491,7 @@
             <v>0</v>
           </cell>
           <cell r="K447">
-            <v>0</v>
+            <v>50</v>
           </cell>
           <cell r="L447" t="str">
             <v>ADIDAS</v>
@@ -32535,14 +32520,14 @@
           <cell r="T447">
             <v>7</v>
           </cell>
-          <cell r="U447" t="str">
-            <v/>
+          <cell r="U447">
+            <v>5</v>
           </cell>
           <cell r="V447">
-            <v>0</v>
+            <v>3.5709999999999999E-2</v>
           </cell>
           <cell r="W447">
-            <v>0</v>
+            <v>2</v>
           </cell>
         </row>
         <row r="448">
@@ -32556,7 +32541,7 @@
             <v xml:space="preserve">PUR2605210002S   </v>
           </cell>
           <cell r="E448" t="str">
-            <v/>
+            <v>BDB-000076</v>
           </cell>
           <cell r="F448" t="str">
             <v>PVN-003742</v>
@@ -32574,7 +32559,7 @@
             <v>0</v>
           </cell>
           <cell r="K448">
-            <v>0</v>
+            <v>30</v>
           </cell>
           <cell r="L448" t="str">
             <v>ADIDAS</v>
@@ -32603,14 +32588,14 @@
           <cell r="T448">
             <v>7</v>
           </cell>
-          <cell r="U448" t="str">
-            <v/>
+          <cell r="U448">
+            <v>5</v>
           </cell>
           <cell r="V448">
-            <v>0</v>
+            <v>3.5709999999999999E-2</v>
           </cell>
           <cell r="W448">
-            <v>0</v>
+            <v>2</v>
           </cell>
         </row>
         <row r="449">
@@ -32814,105 +32799,111 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13"/>
-      <sheetData sheetId="14"/>
-      <sheetData sheetId="15"/>
-      <sheetData sheetId="16"/>
-      <sheetData sheetId="17"/>
-      <sheetData sheetId="18"/>
-      <sheetData sheetId="19"/>
-      <sheetData sheetId="20"/>
-      <sheetData sheetId="21"/>
-      <sheetData sheetId="22"/>
-      <sheetData sheetId="23"/>
-      <sheetData sheetId="24"/>
-      <sheetData sheetId="25"/>
-      <sheetData sheetId="26"/>
-      <sheetData sheetId="27"/>
-      <sheetData sheetId="28"/>
-      <sheetData sheetId="29"/>
-      <sheetData sheetId="30"/>
-      <sheetData sheetId="31"/>
-      <sheetData sheetId="32"/>
-      <sheetData sheetId="33"/>
-      <sheetData sheetId="34"/>
-      <sheetData sheetId="35"/>
-      <sheetData sheetId="36"/>
-      <sheetData sheetId="37"/>
-      <sheetData sheetId="38"/>
-      <sheetData sheetId="39"/>
-      <sheetData sheetId="40"/>
-      <sheetData sheetId="41"/>
-      <sheetData sheetId="42"/>
-      <sheetData sheetId="43"/>
-      <sheetData sheetId="44"/>
-      <sheetData sheetId="45"/>
-      <sheetData sheetId="46"/>
-      <sheetData sheetId="47"/>
-      <sheetData sheetId="48"/>
-      <sheetData sheetId="49"/>
-      <sheetData sheetId="50"/>
-      <sheetData sheetId="51"/>
-      <sheetData sheetId="52"/>
-      <sheetData sheetId="53"/>
-      <sheetData sheetId="54"/>
-      <sheetData sheetId="55"/>
-      <sheetData sheetId="56"/>
-      <sheetData sheetId="57"/>
-      <sheetData sheetId="58"/>
-      <sheetData sheetId="59"/>
-      <sheetData sheetId="60"/>
-      <sheetData sheetId="61"/>
-      <sheetData sheetId="62"/>
-      <sheetData sheetId="63"/>
-      <sheetData sheetId="64"/>
-      <sheetData sheetId="65"/>
-      <sheetData sheetId="66"/>
-      <sheetData sheetId="67"/>
-      <sheetData sheetId="68"/>
-      <sheetData sheetId="69"/>
-      <sheetData sheetId="70"/>
-      <sheetData sheetId="71"/>
-      <sheetData sheetId="72"/>
-      <sheetData sheetId="73"/>
-      <sheetData sheetId="74"/>
-      <sheetData sheetId="75"/>
-      <sheetData sheetId="76"/>
-      <sheetData sheetId="77"/>
-      <sheetData sheetId="78"/>
-      <sheetData sheetId="79"/>
-      <sheetData sheetId="80"/>
-      <sheetData sheetId="81"/>
-      <sheetData sheetId="82"/>
-      <sheetData sheetId="83"/>
-      <sheetData sheetId="84"/>
-      <sheetData sheetId="85"/>
-      <sheetData sheetId="86"/>
-      <sheetData sheetId="87"/>
-      <sheetData sheetId="88"/>
+      <sheetData sheetId="3" refreshError="1"/>
+      <sheetData sheetId="4" refreshError="1"/>
+      <sheetData sheetId="5" refreshError="1"/>
+      <sheetData sheetId="6" refreshError="1"/>
+      <sheetData sheetId="7" refreshError="1"/>
+      <sheetData sheetId="8" refreshError="1"/>
+      <sheetData sheetId="9" refreshError="1"/>
+      <sheetData sheetId="10" refreshError="1"/>
+      <sheetData sheetId="11" refreshError="1"/>
+      <sheetData sheetId="12" refreshError="1"/>
+      <sheetData sheetId="13" refreshError="1"/>
+      <sheetData sheetId="14" refreshError="1"/>
+      <sheetData sheetId="15" refreshError="1"/>
+      <sheetData sheetId="16" refreshError="1"/>
+      <sheetData sheetId="17" refreshError="1"/>
+      <sheetData sheetId="18" refreshError="1"/>
+      <sheetData sheetId="19" refreshError="1"/>
+      <sheetData sheetId="20" refreshError="1"/>
+      <sheetData sheetId="21" refreshError="1"/>
+      <sheetData sheetId="22" refreshError="1"/>
+      <sheetData sheetId="23" refreshError="1"/>
+      <sheetData sheetId="24" refreshError="1"/>
+      <sheetData sheetId="25" refreshError="1"/>
+      <sheetData sheetId="26" refreshError="1"/>
+      <sheetData sheetId="27" refreshError="1"/>
+      <sheetData sheetId="28" refreshError="1"/>
+      <sheetData sheetId="29" refreshError="1"/>
+      <sheetData sheetId="30" refreshError="1"/>
+      <sheetData sheetId="31" refreshError="1"/>
+      <sheetData sheetId="32" refreshError="1"/>
+      <sheetData sheetId="33" refreshError="1"/>
+      <sheetData sheetId="34" refreshError="1"/>
+      <sheetData sheetId="35" refreshError="1"/>
+      <sheetData sheetId="36" refreshError="1"/>
+      <sheetData sheetId="37" refreshError="1"/>
+      <sheetData sheetId="38" refreshError="1"/>
+      <sheetData sheetId="39" refreshError="1"/>
+      <sheetData sheetId="40" refreshError="1"/>
+      <sheetData sheetId="41" refreshError="1"/>
+      <sheetData sheetId="42" refreshError="1"/>
+      <sheetData sheetId="43" refreshError="1"/>
+      <sheetData sheetId="44" refreshError="1"/>
+      <sheetData sheetId="45" refreshError="1"/>
+      <sheetData sheetId="46" refreshError="1"/>
+      <sheetData sheetId="47" refreshError="1"/>
+      <sheetData sheetId="48" refreshError="1"/>
+      <sheetData sheetId="49" refreshError="1"/>
+      <sheetData sheetId="50" refreshError="1"/>
+      <sheetData sheetId="51" refreshError="1"/>
+      <sheetData sheetId="52" refreshError="1"/>
+      <sheetData sheetId="53" refreshError="1"/>
+      <sheetData sheetId="54" refreshError="1"/>
+      <sheetData sheetId="55" refreshError="1"/>
+      <sheetData sheetId="56" refreshError="1"/>
+      <sheetData sheetId="57" refreshError="1"/>
+      <sheetData sheetId="58" refreshError="1"/>
+      <sheetData sheetId="59" refreshError="1"/>
+      <sheetData sheetId="60" refreshError="1"/>
+      <sheetData sheetId="61" refreshError="1"/>
+      <sheetData sheetId="62" refreshError="1"/>
+      <sheetData sheetId="63" refreshError="1"/>
+      <sheetData sheetId="64" refreshError="1"/>
+      <sheetData sheetId="65" refreshError="1"/>
+      <sheetData sheetId="66" refreshError="1"/>
+      <sheetData sheetId="67" refreshError="1"/>
+      <sheetData sheetId="68" refreshError="1"/>
+      <sheetData sheetId="69" refreshError="1"/>
+      <sheetData sheetId="70" refreshError="1"/>
+      <sheetData sheetId="71" refreshError="1"/>
+      <sheetData sheetId="72" refreshError="1"/>
+      <sheetData sheetId="73" refreshError="1"/>
+      <sheetData sheetId="74" refreshError="1"/>
+      <sheetData sheetId="75" refreshError="1"/>
+      <sheetData sheetId="76" refreshError="1"/>
+      <sheetData sheetId="77" refreshError="1"/>
+      <sheetData sheetId="78" refreshError="1"/>
+      <sheetData sheetId="79" refreshError="1"/>
+      <sheetData sheetId="80" refreshError="1"/>
+      <sheetData sheetId="81" refreshError="1"/>
+      <sheetData sheetId="82" refreshError="1"/>
+      <sheetData sheetId="83" refreshError="1"/>
+      <sheetData sheetId="84" refreshError="1"/>
+      <sheetData sheetId="85" refreshError="1"/>
+      <sheetData sheetId="86" refreshError="1"/>
+      <sheetData sheetId="87" refreshError="1"/>
+      <sheetData sheetId="88" refreshError="1"/>
       <sheetData sheetId="89"/>
-      <sheetData sheetId="90"/>
-      <sheetData sheetId="91"/>
-      <sheetData sheetId="92"/>
-      <sheetData sheetId="93"/>
-      <sheetData sheetId="94"/>
-      <sheetData sheetId="95"/>
+      <sheetData sheetId="90" refreshError="1"/>
+      <sheetData sheetId="91">
+        <row r="1">
+          <cell r="F1" t="str">
+            <v>No_Item</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="92" refreshError="1"/>
+      <sheetData sheetId="93" refreshError="1"/>
+      <sheetData sheetId="94" refreshError="1"/>
+      <sheetData sheetId="95" refreshError="1"/>
       <sheetData sheetId="96"/>
-      <sheetData sheetId="97"/>
-      <sheetData sheetId="98"/>
+      <sheetData sheetId="97" refreshError="1"/>
+      <sheetData sheetId="98" refreshError="1"/>
       <sheetData sheetId="99"/>
-      <sheetData sheetId="100"/>
-      <sheetData sheetId="101"/>
+      <sheetData sheetId="100" refreshError="1"/>
+      <sheetData sheetId="101" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -33245,11 +33236,11 @@
       <c r="B1" s="1">
         <v>46155.681657291665</v>
       </c>
-      <c r="D1" s="62" t="s">
+      <c r="D1" s="77" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
+      <c r="E1" s="77"/>
+      <c r="F1" s="77"/>
       <c r="G1" s="3"/>
       <c r="H1" s="4"/>
       <c r="I1" s="5"/>
@@ -34600,13 +34591,13 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46163.886088888888</v>
-      </c>
-      <c r="D1" s="62" t="s">
+        <v>46164.418156597225</v>
+      </c>
+      <c r="D1" s="77" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
+      <c r="E1" s="77"/>
+      <c r="F1" s="77"/>
       <c r="G1" s="3"/>
       <c r="H1" s="4"/>
       <c r="I1" s="5"/>
@@ -34708,19 +34699,19 @@
       </c>
     </row>
     <row r="4" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="63"/>
-      <c r="B4" s="64"/>
-      <c r="C4" s="65"/>
-      <c r="D4" s="66"/>
-      <c r="E4" s="67"/>
-      <c r="F4" s="68"/>
-      <c r="G4" s="69"/>
-      <c r="H4" s="70"/>
-      <c r="I4" s="71"/>
+      <c r="A4" s="62"/>
+      <c r="B4" s="63"/>
+      <c r="C4" s="64"/>
+      <c r="D4" s="65"/>
+      <c r="E4" s="66"/>
+      <c r="F4" s="67"/>
+      <c r="G4" s="68"/>
+      <c r="H4" s="69"/>
+      <c r="I4" s="70"/>
       <c r="J4" s="25"/>
-      <c r="K4" s="71"/>
-      <c r="L4" s="72"/>
-      <c r="M4" s="73"/>
+      <c r="K4" s="70"/>
+      <c r="L4" s="71"/>
+      <c r="M4" s="72"/>
       <c r="N4" s="28"/>
     </row>
     <row r="5" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
@@ -34848,19 +34839,19 @@
       </c>
     </row>
     <row r="8" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="63"/>
-      <c r="B8" s="64"/>
-      <c r="C8" s="65"/>
-      <c r="D8" s="66"/>
-      <c r="E8" s="67"/>
-      <c r="F8" s="68"/>
-      <c r="G8" s="69"/>
-      <c r="H8" s="70"/>
-      <c r="I8" s="71"/>
+      <c r="A8" s="62"/>
+      <c r="B8" s="63"/>
+      <c r="C8" s="64"/>
+      <c r="D8" s="65"/>
+      <c r="E8" s="66"/>
+      <c r="F8" s="67"/>
+      <c r="G8" s="68"/>
+      <c r="H8" s="69"/>
+      <c r="I8" s="70"/>
       <c r="J8" s="25"/>
-      <c r="K8" s="71"/>
-      <c r="L8" s="72"/>
-      <c r="M8" s="73"/>
+      <c r="K8" s="70"/>
+      <c r="L8" s="71"/>
+      <c r="M8" s="72"/>
       <c r="N8" s="28"/>
     </row>
     <row r="9" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
@@ -34906,19 +34897,19 @@
       </c>
     </row>
     <row r="10" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="63"/>
-      <c r="B10" s="64"/>
-      <c r="C10" s="65"/>
-      <c r="D10" s="66"/>
-      <c r="E10" s="67"/>
-      <c r="F10" s="68"/>
-      <c r="G10" s="69"/>
-      <c r="H10" s="70"/>
-      <c r="I10" s="71"/>
+      <c r="A10" s="62"/>
+      <c r="B10" s="63"/>
+      <c r="C10" s="64"/>
+      <c r="D10" s="65"/>
+      <c r="E10" s="66"/>
+      <c r="F10" s="67"/>
+      <c r="G10" s="68"/>
+      <c r="H10" s="69"/>
+      <c r="I10" s="70"/>
       <c r="J10" s="25"/>
-      <c r="K10" s="71"/>
-      <c r="L10" s="72"/>
-      <c r="M10" s="73"/>
+      <c r="K10" s="70"/>
+      <c r="L10" s="71"/>
+      <c r="M10" s="72"/>
       <c r="N10" s="28"/>
     </row>
     <row r="11" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
@@ -34964,19 +34955,19 @@
       </c>
     </row>
     <row r="12" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="63"/>
-      <c r="B12" s="64"/>
-      <c r="C12" s="65"/>
-      <c r="D12" s="66"/>
-      <c r="E12" s="67"/>
-      <c r="F12" s="68"/>
-      <c r="G12" s="69"/>
-      <c r="H12" s="70"/>
-      <c r="I12" s="71"/>
+      <c r="A12" s="62"/>
+      <c r="B12" s="63"/>
+      <c r="C12" s="64"/>
+      <c r="D12" s="65"/>
+      <c r="E12" s="66"/>
+      <c r="F12" s="67"/>
+      <c r="G12" s="68"/>
+      <c r="H12" s="69"/>
+      <c r="I12" s="70"/>
       <c r="J12" s="25"/>
-      <c r="K12" s="71"/>
-      <c r="L12" s="72"/>
-      <c r="M12" s="73"/>
+      <c r="K12" s="70"/>
+      <c r="L12" s="71"/>
+      <c r="M12" s="72"/>
       <c r="N12" s="28"/>
     </row>
     <row r="13" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
@@ -35022,19 +35013,19 @@
       </c>
     </row>
     <row r="14" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="63"/>
-      <c r="B14" s="64"/>
-      <c r="C14" s="65"/>
-      <c r="D14" s="66"/>
-      <c r="E14" s="67"/>
-      <c r="F14" s="68"/>
-      <c r="G14" s="69"/>
-      <c r="H14" s="70"/>
-      <c r="I14" s="71"/>
+      <c r="A14" s="62"/>
+      <c r="B14" s="63"/>
+      <c r="C14" s="64"/>
+      <c r="D14" s="65"/>
+      <c r="E14" s="66"/>
+      <c r="F14" s="67"/>
+      <c r="G14" s="68"/>
+      <c r="H14" s="69"/>
+      <c r="I14" s="70"/>
       <c r="J14" s="25"/>
-      <c r="K14" s="71"/>
-      <c r="L14" s="72"/>
-      <c r="M14" s="73"/>
+      <c r="K14" s="70"/>
+      <c r="L14" s="71"/>
+      <c r="M14" s="72"/>
       <c r="N14" s="28"/>
     </row>
     <row r="15" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
@@ -35080,19 +35071,19 @@
       </c>
     </row>
     <row r="16" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="63"/>
-      <c r="B16" s="64"/>
-      <c r="C16" s="65"/>
-      <c r="D16" s="66"/>
-      <c r="E16" s="67"/>
-      <c r="F16" s="68"/>
-      <c r="G16" s="69"/>
-      <c r="H16" s="70"/>
-      <c r="I16" s="71"/>
+      <c r="A16" s="62"/>
+      <c r="B16" s="63"/>
+      <c r="C16" s="64"/>
+      <c r="D16" s="65"/>
+      <c r="E16" s="66"/>
+      <c r="F16" s="67"/>
+      <c r="G16" s="68"/>
+      <c r="H16" s="69"/>
+      <c r="I16" s="70"/>
       <c r="J16" s="25"/>
-      <c r="K16" s="71"/>
-      <c r="L16" s="72"/>
-      <c r="M16" s="74"/>
+      <c r="K16" s="70"/>
+      <c r="L16" s="71"/>
+      <c r="M16" s="73"/>
       <c r="N16" s="28"/>
     </row>
     <row r="17" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
@@ -36010,13 +36001,13 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46163.886088888888</v>
-      </c>
-      <c r="D1" s="62" t="s">
+        <v>46164.418156597225</v>
+      </c>
+      <c r="D1" s="77" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
+      <c r="E1" s="77"/>
+      <c r="F1" s="77"/>
       <c r="G1" s="3"/>
       <c r="H1" s="4"/>
       <c r="I1" s="5"/>
@@ -36105,12 +36096,12 @@
         <v>114</v>
       </c>
       <c r="K3" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="L3" s="75">
+        <v>246</v>
+      </c>
+      <c r="L3" s="74">
         <v>0</v>
       </c>
-      <c r="M3" s="76" t="s">
+      <c r="M3" s="75" t="s">
         <v>115</v>
       </c>
       <c r="N3" s="28">
@@ -36118,20 +36109,22 @@
       </c>
     </row>
     <row r="4" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="63"/>
-      <c r="B4" s="64"/>
-      <c r="C4" s="65"/>
-      <c r="D4" s="66"/>
-      <c r="E4" s="67"/>
-      <c r="F4" s="68"/>
-      <c r="G4" s="69"/>
-      <c r="H4" s="70"/>
-      <c r="I4" s="71"/>
+      <c r="A4" s="62"/>
+      <c r="B4" s="63"/>
+      <c r="C4" s="64"/>
+      <c r="D4" s="65"/>
+      <c r="E4" s="66"/>
+      <c r="F4" s="67"/>
+      <c r="G4" s="68"/>
+      <c r="H4" s="69"/>
+      <c r="I4" s="70"/>
       <c r="J4" s="25"/>
-      <c r="K4" s="71"/>
-      <c r="L4" s="71"/>
-      <c r="M4" s="71"/>
-      <c r="N4" s="77"/>
+      <c r="K4" s="25" t="s">
+        <v>246</v>
+      </c>
+      <c r="L4" s="70"/>
+      <c r="M4" s="70"/>
+      <c r="N4" s="76"/>
     </row>
     <row r="5" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="17" t="s">
@@ -36165,7 +36158,7 @@
         <v>121</v>
       </c>
       <c r="K5" s="25" t="s">
-        <v>59</v>
+        <v>246</v>
       </c>
       <c r="L5" s="26">
         <v>1</v>
@@ -36178,20 +36171,22 @@
       </c>
     </row>
     <row r="6" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="63"/>
-      <c r="B6" s="64"/>
-      <c r="C6" s="65"/>
-      <c r="D6" s="66"/>
-      <c r="E6" s="67"/>
-      <c r="F6" s="68"/>
-      <c r="G6" s="69"/>
-      <c r="H6" s="70"/>
-      <c r="I6" s="71"/>
+      <c r="A6" s="62"/>
+      <c r="B6" s="63"/>
+      <c r="C6" s="64"/>
+      <c r="D6" s="65"/>
+      <c r="E6" s="66"/>
+      <c r="F6" s="67"/>
+      <c r="G6" s="68"/>
+      <c r="H6" s="69"/>
+      <c r="I6" s="70"/>
       <c r="J6" s="25"/>
-      <c r="K6" s="71"/>
-      <c r="L6" s="72"/>
-      <c r="M6" s="73"/>
-      <c r="N6" s="77"/>
+      <c r="K6" s="25" t="s">
+        <v>246</v>
+      </c>
+      <c r="L6" s="71"/>
+      <c r="M6" s="72"/>
+      <c r="N6" s="76"/>
     </row>
     <row r="7" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="17" t="s">
@@ -36225,7 +36220,7 @@
         <v>129</v>
       </c>
       <c r="K7" s="25" t="s">
-        <v>130</v>
+        <v>246</v>
       </c>
       <c r="L7" s="26">
         <v>2</v>
@@ -36236,36 +36231,38 @@
       </c>
     </row>
     <row r="8" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="63"/>
-      <c r="B8" s="64"/>
-      <c r="C8" s="65"/>
-      <c r="D8" s="66"/>
-      <c r="E8" s="67"/>
-      <c r="F8" s="68"/>
-      <c r="G8" s="69"/>
-      <c r="H8" s="70"/>
-      <c r="I8" s="71"/>
+      <c r="A8" s="62"/>
+      <c r="B8" s="63"/>
+      <c r="C8" s="64"/>
+      <c r="D8" s="65"/>
+      <c r="E8" s="66"/>
+      <c r="F8" s="67"/>
+      <c r="G8" s="68"/>
+      <c r="H8" s="69"/>
+      <c r="I8" s="70"/>
       <c r="J8" s="25"/>
-      <c r="K8" s="71"/>
-      <c r="L8" s="72"/>
-      <c r="M8" s="73"/>
-      <c r="N8" s="77"/>
+      <c r="K8" s="25" t="s">
+        <v>246</v>
+      </c>
+      <c r="L8" s="71"/>
+      <c r="M8" s="72"/>
+      <c r="N8" s="76"/>
     </row>
     <row r="9" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="17" t="s">
+        <v>130</v>
+      </c>
+      <c r="B9" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="C9" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="D9" s="20" t="s">
         <v>133</v>
       </c>
-      <c r="D9" s="20" t="s">
+      <c r="E9" s="21" t="s">
         <v>134</v>
-      </c>
-      <c r="E9" s="21" t="s">
-        <v>135</v>
       </c>
       <c r="F9" s="22">
         <v>30</v>
@@ -36283,7 +36280,7 @@
         <v>129</v>
       </c>
       <c r="K9" s="25" t="s">
-        <v>130</v>
+        <v>246</v>
       </c>
       <c r="L9" s="26">
         <v>3</v>
@@ -36295,19 +36292,19 @@
     </row>
     <row r="10" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="17" t="s">
+        <v>135</v>
+      </c>
+      <c r="B10" s="18" t="s">
         <v>136</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="C10" s="19" t="s">
+        <v>132</v>
+      </c>
+      <c r="D10" s="20" t="s">
         <v>137</v>
       </c>
-      <c r="C10" s="19" t="s">
-        <v>133</v>
-      </c>
-      <c r="D10" s="20" t="s">
+      <c r="E10" s="21" t="s">
         <v>138</v>
-      </c>
-      <c r="E10" s="21" t="s">
-        <v>139</v>
       </c>
       <c r="F10" s="22">
         <v>30</v>
@@ -36319,13 +36316,13 @@
         <v>1</v>
       </c>
       <c r="I10" s="25" t="s">
+        <v>139</v>
+      </c>
+      <c r="J10" s="25" t="s">
         <v>140</v>
       </c>
-      <c r="J10" s="25" t="s">
-        <v>141</v>
-      </c>
       <c r="K10" s="25" t="s">
-        <v>142</v>
+        <v>246</v>
       </c>
       <c r="L10" s="26"/>
       <c r="M10" s="27"/>
@@ -36334,36 +36331,38 @@
       </c>
     </row>
     <row r="11" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="63"/>
-      <c r="B11" s="64"/>
-      <c r="C11" s="65"/>
-      <c r="D11" s="66"/>
-      <c r="E11" s="67"/>
-      <c r="F11" s="68"/>
-      <c r="G11" s="69"/>
-      <c r="H11" s="70"/>
-      <c r="I11" s="71"/>
+      <c r="A11" s="62"/>
+      <c r="B11" s="63"/>
+      <c r="C11" s="64"/>
+      <c r="D11" s="65"/>
+      <c r="E11" s="66"/>
+      <c r="F11" s="67"/>
+      <c r="G11" s="68"/>
+      <c r="H11" s="69"/>
+      <c r="I11" s="70"/>
       <c r="J11" s="25"/>
-      <c r="K11" s="71"/>
-      <c r="L11" s="72"/>
-      <c r="M11" s="73"/>
-      <c r="N11" s="77"/>
+      <c r="K11" s="25" t="s">
+        <v>246</v>
+      </c>
+      <c r="L11" s="71"/>
+      <c r="M11" s="72"/>
+      <c r="N11" s="76"/>
     </row>
     <row r="12" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="17" t="s">
+        <v>141</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>142</v>
+      </c>
+      <c r="C12" s="19" t="s">
         <v>143</v>
       </c>
-      <c r="B12" s="18" t="s">
+      <c r="D12" s="20" t="s">
         <v>144</v>
       </c>
-      <c r="C12" s="19" t="s">
+      <c r="E12" s="21" t="s">
         <v>145</v>
-      </c>
-      <c r="D12" s="20" t="s">
-        <v>146</v>
-      </c>
-      <c r="E12" s="21" t="s">
-        <v>147</v>
       </c>
       <c r="F12" s="22">
         <v>30</v>
@@ -36381,7 +36380,7 @@
         <v>43</v>
       </c>
       <c r="K12" s="25" t="s">
-        <v>148</v>
+        <v>246</v>
       </c>
       <c r="L12" s="26">
         <v>1</v>
@@ -36392,36 +36391,38 @@
       </c>
     </row>
     <row r="13" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="63"/>
-      <c r="B13" s="64"/>
-      <c r="C13" s="65"/>
-      <c r="D13" s="66"/>
-      <c r="E13" s="67"/>
-      <c r="F13" s="68"/>
-      <c r="G13" s="69"/>
-      <c r="H13" s="70"/>
-      <c r="I13" s="71"/>
+      <c r="A13" s="62"/>
+      <c r="B13" s="63"/>
+      <c r="C13" s="64"/>
+      <c r="D13" s="65"/>
+      <c r="E13" s="66"/>
+      <c r="F13" s="67"/>
+      <c r="G13" s="68"/>
+      <c r="H13" s="69"/>
+      <c r="I13" s="70"/>
       <c r="J13" s="25"/>
-      <c r="K13" s="71"/>
-      <c r="L13" s="72"/>
-      <c r="M13" s="73"/>
-      <c r="N13" s="77"/>
+      <c r="K13" s="25" t="s">
+        <v>246</v>
+      </c>
+      <c r="L13" s="71"/>
+      <c r="M13" s="72"/>
+      <c r="N13" s="76"/>
     </row>
     <row r="14" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="17" t="s">
+        <v>146</v>
+      </c>
+      <c r="B14" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="C14" s="19" t="s">
+        <v>148</v>
+      </c>
+      <c r="D14" s="20" t="s">
         <v>149</v>
       </c>
-      <c r="B14" s="18" t="s">
+      <c r="E14" s="21" t="s">
         <v>150</v>
-      </c>
-      <c r="C14" s="19" t="s">
-        <v>151</v>
-      </c>
-      <c r="D14" s="20" t="s">
-        <v>152</v>
-      </c>
-      <c r="E14" s="21" t="s">
-        <v>153</v>
       </c>
       <c r="F14" s="22">
         <v>40</v>
@@ -36433,13 +36434,13 @@
         <v>2</v>
       </c>
       <c r="I14" s="25" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="J14" s="25" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="K14" s="25" t="s">
-        <v>156</v>
+        <v>246</v>
       </c>
       <c r="L14" s="26">
         <v>3</v>
@@ -36451,19 +36452,19 @@
     </row>
     <row r="15" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="17" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="D15" s="20" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="E15" s="21" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="F15" s="22">
         <v>20</v>
@@ -36475,13 +36476,13 @@
         <v>1</v>
       </c>
       <c r="I15" s="25" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="J15" s="25" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="K15" s="25" t="s">
-        <v>162</v>
+        <v>246</v>
       </c>
       <c r="L15" s="26"/>
       <c r="M15" s="40"/>
@@ -36490,27 +36491,29 @@
       </c>
     </row>
     <row r="16" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="63"/>
-      <c r="B16" s="64"/>
-      <c r="C16" s="65"/>
-      <c r="D16" s="66"/>
-      <c r="E16" s="67"/>
-      <c r="F16" s="68"/>
-      <c r="G16" s="69"/>
-      <c r="H16" s="70"/>
-      <c r="I16" s="71"/>
+      <c r="A16" s="62"/>
+      <c r="B16" s="63"/>
+      <c r="C16" s="64"/>
+      <c r="D16" s="65"/>
+      <c r="E16" s="66"/>
+      <c r="F16" s="67"/>
+      <c r="G16" s="68"/>
+      <c r="H16" s="69"/>
+      <c r="I16" s="70"/>
       <c r="J16" s="25"/>
-      <c r="K16" s="71"/>
-      <c r="L16" s="72"/>
-      <c r="M16" s="74"/>
-      <c r="N16" s="77"/>
+      <c r="K16" s="25" t="s">
+        <v>246</v>
+      </c>
+      <c r="L16" s="71"/>
+      <c r="M16" s="73"/>
+      <c r="N16" s="76"/>
     </row>
     <row r="17" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="17" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="C17" s="19" t="s">
         <v>63</v>
@@ -36519,7 +36522,7 @@
         <v>71</v>
       </c>
       <c r="E17" s="21" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="F17" s="22">
         <v>150</v>
@@ -36534,10 +36537,10 @@
         <v>57</v>
       </c>
       <c r="J17" s="25" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="K17" s="25" t="s">
-        <v>167</v>
+        <v>246</v>
       </c>
       <c r="L17" s="26">
         <v>9</v>
@@ -36549,10 +36552,10 @@
     </row>
     <row r="18" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="17" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="C18" s="19" t="s">
         <v>63</v>
@@ -36576,10 +36579,10 @@
         <v>57</v>
       </c>
       <c r="J18" s="25" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="K18" s="25" t="s">
-        <v>67</v>
+        <v>246</v>
       </c>
       <c r="L18" s="26"/>
       <c r="M18" s="40"/>
@@ -36588,36 +36591,38 @@
       </c>
     </row>
     <row r="19" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="63"/>
-      <c r="B19" s="64"/>
-      <c r="C19" s="65"/>
-      <c r="D19" s="66"/>
-      <c r="E19" s="67"/>
-      <c r="F19" s="68"/>
-      <c r="G19" s="69"/>
-      <c r="H19" s="70"/>
-      <c r="I19" s="71"/>
+      <c r="A19" s="62"/>
+      <c r="B19" s="63"/>
+      <c r="C19" s="64"/>
+      <c r="D19" s="65"/>
+      <c r="E19" s="66"/>
+      <c r="F19" s="67"/>
+      <c r="G19" s="68"/>
+      <c r="H19" s="69"/>
+      <c r="I19" s="70"/>
       <c r="J19" s="25"/>
-      <c r="K19" s="71"/>
-      <c r="L19" s="72"/>
-      <c r="M19" s="74"/>
-      <c r="N19" s="77"/>
+      <c r="K19" s="25" t="s">
+        <v>246</v>
+      </c>
+      <c r="L19" s="71"/>
+      <c r="M19" s="73"/>
+      <c r="N19" s="76"/>
     </row>
     <row r="20" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="17" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="B20" s="18" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="C20" s="19" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="D20" s="20" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="E20" s="21" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="F20" s="22">
         <v>50</v>
@@ -36635,7 +36640,7 @@
         <v>27</v>
       </c>
       <c r="K20" s="25" t="s">
-        <v>28</v>
+        <v>246</v>
       </c>
       <c r="L20" s="26">
         <v>5</v>
@@ -36646,36 +36651,38 @@
       </c>
     </row>
     <row r="21" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="63"/>
-      <c r="B21" s="64"/>
-      <c r="C21" s="65"/>
-      <c r="D21" s="66"/>
-      <c r="E21" s="67"/>
-      <c r="F21" s="68"/>
-      <c r="G21" s="69"/>
-      <c r="H21" s="70"/>
-      <c r="I21" s="71"/>
+      <c r="A21" s="62"/>
+      <c r="B21" s="63"/>
+      <c r="C21" s="64"/>
+      <c r="D21" s="65"/>
+      <c r="E21" s="66"/>
+      <c r="F21" s="67"/>
+      <c r="G21" s="68"/>
+      <c r="H21" s="69"/>
+      <c r="I21" s="70"/>
       <c r="J21" s="25"/>
-      <c r="K21" s="71"/>
-      <c r="L21" s="72"/>
-      <c r="M21" s="74"/>
-      <c r="N21" s="77"/>
+      <c r="K21" s="25" t="s">
+        <v>246</v>
+      </c>
+      <c r="L21" s="71"/>
+      <c r="M21" s="73"/>
+      <c r="N21" s="76"/>
     </row>
     <row r="22" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="17" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="B22" s="18" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="C22" s="19" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="D22" s="20" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="E22" s="21" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="F22" s="22">
         <v>50</v>
@@ -36693,7 +36700,7 @@
         <v>27</v>
       </c>
       <c r="K22" s="25" t="s">
-        <v>28</v>
+        <v>246</v>
       </c>
       <c r="L22" s="26">
         <v>5</v>
@@ -36704,27 +36711,29 @@
       </c>
     </row>
     <row r="23" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="63"/>
-      <c r="B23" s="64"/>
-      <c r="C23" s="65"/>
-      <c r="D23" s="66"/>
-      <c r="E23" s="67"/>
-      <c r="F23" s="68"/>
-      <c r="G23" s="69"/>
-      <c r="H23" s="70"/>
-      <c r="I23" s="71"/>
+      <c r="A23" s="62"/>
+      <c r="B23" s="63"/>
+      <c r="C23" s="64"/>
+      <c r="D23" s="65"/>
+      <c r="E23" s="66"/>
+      <c r="F23" s="67"/>
+      <c r="G23" s="68"/>
+      <c r="H23" s="69"/>
+      <c r="I23" s="70"/>
       <c r="J23" s="25"/>
-      <c r="K23" s="71"/>
-      <c r="L23" s="72"/>
-      <c r="M23" s="73"/>
-      <c r="N23" s="77"/>
+      <c r="K23" s="25" t="s">
+        <v>246</v>
+      </c>
+      <c r="L23" s="71"/>
+      <c r="M23" s="72"/>
+      <c r="N23" s="76"/>
     </row>
     <row r="24" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="17" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="B24" s="18" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="C24" s="19" t="s">
         <v>30</v>
@@ -36751,7 +36760,7 @@
         <v>27</v>
       </c>
       <c r="K24" s="25" t="s">
-        <v>28</v>
+        <v>246</v>
       </c>
       <c r="L24" s="26">
         <v>2</v>
@@ -36762,27 +36771,29 @@
       </c>
     </row>
     <row r="25" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="63"/>
-      <c r="B25" s="64"/>
-      <c r="C25" s="65"/>
-      <c r="D25" s="66"/>
-      <c r="E25" s="67"/>
-      <c r="F25" s="68"/>
-      <c r="G25" s="69"/>
-      <c r="H25" s="70"/>
-      <c r="I25" s="71"/>
+      <c r="A25" s="62"/>
+      <c r="B25" s="63"/>
+      <c r="C25" s="64"/>
+      <c r="D25" s="65"/>
+      <c r="E25" s="66"/>
+      <c r="F25" s="67"/>
+      <c r="G25" s="68"/>
+      <c r="H25" s="69"/>
+      <c r="I25" s="70"/>
       <c r="J25" s="25"/>
-      <c r="K25" s="71"/>
-      <c r="L25" s="72"/>
-      <c r="M25" s="74"/>
-      <c r="N25" s="77"/>
+      <c r="K25" s="25" t="s">
+        <v>246</v>
+      </c>
+      <c r="L25" s="71"/>
+      <c r="M25" s="73"/>
+      <c r="N25" s="76"/>
     </row>
     <row r="26" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="17" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="B26" s="18" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="C26" s="19" t="s">
         <v>35</v>
@@ -36809,7 +36820,7 @@
         <v>27</v>
       </c>
       <c r="K26" s="25" t="s">
-        <v>28</v>
+        <v>246</v>
       </c>
       <c r="L26" s="26">
         <v>2</v>
@@ -36820,36 +36831,38 @@
       </c>
     </row>
     <row r="27" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="63"/>
-      <c r="B27" s="64"/>
-      <c r="C27" s="65"/>
-      <c r="D27" s="66"/>
-      <c r="E27" s="67"/>
-      <c r="F27" s="68"/>
-      <c r="G27" s="69"/>
-      <c r="H27" s="70"/>
-      <c r="I27" s="71"/>
+      <c r="A27" s="62"/>
+      <c r="B27" s="63"/>
+      <c r="C27" s="64"/>
+      <c r="D27" s="65"/>
+      <c r="E27" s="66"/>
+      <c r="F27" s="67"/>
+      <c r="G27" s="68"/>
+      <c r="H27" s="69"/>
+      <c r="I27" s="70"/>
       <c r="J27" s="25"/>
-      <c r="K27" s="71"/>
-      <c r="L27" s="72"/>
-      <c r="M27" s="74"/>
-      <c r="N27" s="77"/>
+      <c r="K27" s="25" t="s">
+        <v>246</v>
+      </c>
+      <c r="L27" s="71"/>
+      <c r="M27" s="73"/>
+      <c r="N27" s="76"/>
     </row>
     <row r="28" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="17" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="B28" s="18" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="C28" s="19" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="D28" s="20" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="E28" s="21" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="F28" s="22">
         <v>40</v>
@@ -36867,7 +36880,7 @@
         <v>27</v>
       </c>
       <c r="K28" s="25" t="s">
-        <v>28</v>
+        <v>246</v>
       </c>
       <c r="L28" s="26">
         <v>2</v>
@@ -37456,13 +37469,13 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46163.886088888888</v>
-      </c>
-      <c r="D1" s="62" t="s">
+        <v>46164.418156481479</v>
+      </c>
+      <c r="D1" s="77" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
+      <c r="E1" s="77"/>
+      <c r="F1" s="77"/>
       <c r="G1" s="3"/>
       <c r="H1" s="4"/>
       <c r="I1" s="5"/>
@@ -37521,19 +37534,19 @@
     </row>
     <row r="3" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="17" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="C3" s="19" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="D3" s="20" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="E3" s="21" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="F3" s="22">
         <v>70</v>
@@ -37548,10 +37561,10 @@
         <v>57</v>
       </c>
       <c r="J3" s="25" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="K3" s="25" t="s">
-        <v>167</v>
+        <v>246</v>
       </c>
       <c r="L3" s="26">
         <v>2</v>
@@ -37562,36 +37575,38 @@
       </c>
     </row>
     <row r="4" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="63"/>
-      <c r="B4" s="64"/>
-      <c r="C4" s="65"/>
-      <c r="D4" s="66"/>
-      <c r="E4" s="67"/>
-      <c r="F4" s="68"/>
-      <c r="G4" s="69"/>
-      <c r="H4" s="70"/>
-      <c r="I4" s="71"/>
-      <c r="J4" s="71"/>
-      <c r="K4" s="71"/>
-      <c r="L4" s="72"/>
-      <c r="M4" s="73"/>
+      <c r="A4" s="62"/>
+      <c r="B4" s="63"/>
+      <c r="C4" s="64"/>
+      <c r="D4" s="65"/>
+      <c r="E4" s="66"/>
+      <c r="F4" s="67"/>
+      <c r="G4" s="68"/>
+      <c r="H4" s="69"/>
+      <c r="I4" s="70"/>
+      <c r="J4" s="70"/>
+      <c r="K4" s="25" t="s">
+        <v>246</v>
+      </c>
+      <c r="L4" s="71"/>
+      <c r="M4" s="72"/>
       <c r="N4" s="28"/>
     </row>
     <row r="5" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="17" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="C5" s="19" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="F5" s="22">
         <v>40</v>
@@ -37603,13 +37618,13 @@
         <v>2</v>
       </c>
       <c r="I5" s="25" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="J5" s="25" t="s">
         <v>27</v>
       </c>
       <c r="K5" s="25" t="s">
-        <v>28</v>
+        <v>246</v>
       </c>
       <c r="L5" s="26">
         <v>2</v>
@@ -37620,36 +37635,38 @@
       </c>
     </row>
     <row r="6" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="63"/>
-      <c r="B6" s="64"/>
-      <c r="C6" s="65"/>
-      <c r="D6" s="66"/>
-      <c r="E6" s="67"/>
-      <c r="F6" s="68"/>
-      <c r="G6" s="69"/>
-      <c r="H6" s="70"/>
-      <c r="I6" s="71"/>
-      <c r="J6" s="71"/>
-      <c r="K6" s="71"/>
-      <c r="L6" s="72"/>
-      <c r="M6" s="73"/>
+      <c r="A6" s="62"/>
+      <c r="B6" s="63"/>
+      <c r="C6" s="64"/>
+      <c r="D6" s="65"/>
+      <c r="E6" s="66"/>
+      <c r="F6" s="67"/>
+      <c r="G6" s="68"/>
+      <c r="H6" s="69"/>
+      <c r="I6" s="70"/>
+      <c r="J6" s="70"/>
+      <c r="K6" s="25" t="s">
+        <v>246</v>
+      </c>
+      <c r="L6" s="71"/>
+      <c r="M6" s="72"/>
       <c r="N6" s="28"/>
     </row>
     <row r="7" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="17" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="D7" s="20" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="F7" s="22">
         <v>40</v>
@@ -37661,13 +37678,13 @@
         <v>1</v>
       </c>
       <c r="I7" s="25" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="J7" s="25" t="s">
         <v>27</v>
       </c>
       <c r="K7" s="25" t="s">
-        <v>205</v>
+        <v>246</v>
       </c>
       <c r="L7" s="26">
         <v>1</v>
@@ -37678,36 +37695,38 @@
       </c>
     </row>
     <row r="8" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="63"/>
-      <c r="B8" s="64"/>
-      <c r="C8" s="65"/>
-      <c r="D8" s="66"/>
-      <c r="E8" s="67"/>
-      <c r="F8" s="68"/>
-      <c r="G8" s="69"/>
-      <c r="H8" s="70"/>
-      <c r="I8" s="71"/>
-      <c r="J8" s="71"/>
-      <c r="K8" s="71"/>
-      <c r="L8" s="72"/>
-      <c r="M8" s="73"/>
+      <c r="A8" s="62"/>
+      <c r="B8" s="63"/>
+      <c r="C8" s="64"/>
+      <c r="D8" s="65"/>
+      <c r="E8" s="66"/>
+      <c r="F8" s="67"/>
+      <c r="G8" s="68"/>
+      <c r="H8" s="69"/>
+      <c r="I8" s="70"/>
+      <c r="J8" s="70"/>
+      <c r="K8" s="25" t="s">
+        <v>246</v>
+      </c>
+      <c r="L8" s="71"/>
+      <c r="M8" s="72"/>
       <c r="N8" s="28"/>
     </row>
     <row r="9" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="17" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="D9" s="20" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="F9" s="22">
         <v>40</v>
@@ -37719,13 +37738,13 @@
         <v>2</v>
       </c>
       <c r="I9" s="25" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="J9" s="25" t="s">
         <v>27</v>
       </c>
       <c r="K9" s="25" t="s">
-        <v>205</v>
+        <v>246</v>
       </c>
       <c r="L9" s="26">
         <v>2</v>
@@ -37736,36 +37755,38 @@
       </c>
     </row>
     <row r="10" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="63"/>
-      <c r="B10" s="64"/>
-      <c r="C10" s="65"/>
-      <c r="D10" s="66"/>
-      <c r="E10" s="67"/>
-      <c r="F10" s="68"/>
-      <c r="G10" s="69"/>
-      <c r="H10" s="70"/>
-      <c r="I10" s="71"/>
-      <c r="J10" s="71"/>
-      <c r="K10" s="71"/>
-      <c r="L10" s="72"/>
-      <c r="M10" s="73"/>
+      <c r="A10" s="62"/>
+      <c r="B10" s="63"/>
+      <c r="C10" s="64"/>
+      <c r="D10" s="65"/>
+      <c r="E10" s="66"/>
+      <c r="F10" s="67"/>
+      <c r="G10" s="68"/>
+      <c r="H10" s="69"/>
+      <c r="I10" s="70"/>
+      <c r="J10" s="70"/>
+      <c r="K10" s="25" t="s">
+        <v>246</v>
+      </c>
+      <c r="L10" s="71"/>
+      <c r="M10" s="72"/>
       <c r="N10" s="28"/>
     </row>
     <row r="11" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="17" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="D11" s="20" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="F11" s="22">
         <v>30</v>
@@ -37777,13 +37798,13 @@
         <v>2</v>
       </c>
       <c r="I11" s="25" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="J11" s="25" t="s">
         <v>27</v>
       </c>
       <c r="K11" s="25" t="s">
-        <v>205</v>
+        <v>246</v>
       </c>
       <c r="L11" s="26">
         <v>2</v>
@@ -37794,36 +37815,38 @@
       </c>
     </row>
     <row r="12" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="63"/>
-      <c r="B12" s="64"/>
-      <c r="C12" s="65"/>
-      <c r="D12" s="66"/>
-      <c r="E12" s="67"/>
-      <c r="F12" s="68"/>
-      <c r="G12" s="69"/>
-      <c r="H12" s="70"/>
-      <c r="I12" s="71"/>
-      <c r="J12" s="71"/>
-      <c r="K12" s="71"/>
-      <c r="L12" s="72"/>
-      <c r="M12" s="73"/>
+      <c r="A12" s="62"/>
+      <c r="B12" s="63"/>
+      <c r="C12" s="64"/>
+      <c r="D12" s="65"/>
+      <c r="E12" s="66"/>
+      <c r="F12" s="67"/>
+      <c r="G12" s="68"/>
+      <c r="H12" s="69"/>
+      <c r="I12" s="70"/>
+      <c r="J12" s="70"/>
+      <c r="K12" s="25" t="s">
+        <v>246</v>
+      </c>
+      <c r="L12" s="71"/>
+      <c r="M12" s="72"/>
       <c r="N12" s="28"/>
     </row>
     <row r="13" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="17" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="D13" s="20" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="E13" s="21" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="F13" s="22">
         <v>50</v>
@@ -37835,13 +37858,13 @@
         <v>2</v>
       </c>
       <c r="I13" s="25" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="J13" s="25" t="s">
         <v>27</v>
       </c>
       <c r="K13" s="25" t="s">
-        <v>28</v>
+        <v>246</v>
       </c>
       <c r="L13" s="26">
         <v>2</v>
@@ -37852,36 +37875,38 @@
       </c>
     </row>
     <row r="14" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="63"/>
-      <c r="B14" s="64"/>
-      <c r="C14" s="65"/>
-      <c r="D14" s="66"/>
-      <c r="E14" s="67"/>
-      <c r="F14" s="68"/>
-      <c r="G14" s="69"/>
-      <c r="H14" s="70"/>
-      <c r="I14" s="71"/>
-      <c r="J14" s="71"/>
-      <c r="K14" s="71"/>
-      <c r="L14" s="72"/>
-      <c r="M14" s="73"/>
+      <c r="A14" s="62"/>
+      <c r="B14" s="63"/>
+      <c r="C14" s="64"/>
+      <c r="D14" s="65"/>
+      <c r="E14" s="66"/>
+      <c r="F14" s="67"/>
+      <c r="G14" s="68"/>
+      <c r="H14" s="69"/>
+      <c r="I14" s="70"/>
+      <c r="J14" s="70"/>
+      <c r="K14" s="25" t="s">
+        <v>246</v>
+      </c>
+      <c r="L14" s="71"/>
+      <c r="M14" s="72"/>
       <c r="N14" s="28"/>
     </row>
     <row r="15" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="17" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="C15" s="19" t="s">
         <v>54</v>
       </c>
       <c r="D15" s="20" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="E15" s="21" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="F15" s="22">
         <v>30</v>
@@ -37899,7 +37924,7 @@
         <v>27</v>
       </c>
       <c r="K15" s="25" t="s">
-        <v>78</v>
+        <v>246</v>
       </c>
       <c r="L15" s="26">
         <v>6</v>
@@ -37911,19 +37936,19 @@
     </row>
     <row r="16" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="17" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="C16" s="19" t="s">
         <v>54</v>
       </c>
       <c r="D16" s="20" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="E16" s="21" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="F16" s="22">
         <v>80</v>
@@ -37941,7 +37966,7 @@
         <v>27</v>
       </c>
       <c r="K16" s="25" t="s">
-        <v>28</v>
+        <v>246</v>
       </c>
       <c r="L16" s="26"/>
       <c r="M16" s="27"/>
@@ -37951,19 +37976,19 @@
     </row>
     <row r="17" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="17" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="C17" s="19" t="s">
         <v>54</v>
       </c>
       <c r="D17" s="20" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="E17" s="21" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="F17" s="22">
         <v>20</v>
@@ -37981,7 +38006,7 @@
         <v>27</v>
       </c>
       <c r="K17" s="25" t="s">
-        <v>74</v>
+        <v>246</v>
       </c>
       <c r="L17" s="26"/>
       <c r="M17" s="27"/>
@@ -37990,36 +38015,38 @@
       </c>
     </row>
     <row r="18" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="63"/>
-      <c r="B18" s="64"/>
-      <c r="C18" s="65"/>
-      <c r="D18" s="66"/>
-      <c r="E18" s="67"/>
-      <c r="F18" s="68"/>
-      <c r="G18" s="69"/>
-      <c r="H18" s="70"/>
-      <c r="I18" s="71"/>
-      <c r="J18" s="71"/>
-      <c r="K18" s="71"/>
-      <c r="L18" s="72"/>
-      <c r="M18" s="73"/>
+      <c r="A18" s="62"/>
+      <c r="B18" s="63"/>
+      <c r="C18" s="64"/>
+      <c r="D18" s="65"/>
+      <c r="E18" s="66"/>
+      <c r="F18" s="67"/>
+      <c r="G18" s="68"/>
+      <c r="H18" s="69"/>
+      <c r="I18" s="70"/>
+      <c r="J18" s="70"/>
+      <c r="K18" s="25" t="s">
+        <v>246</v>
+      </c>
+      <c r="L18" s="71"/>
+      <c r="M18" s="72"/>
       <c r="N18" s="28"/>
     </row>
     <row r="19" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="17" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="C19" s="19" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="D19" s="20" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="E19" s="21" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="F19" s="22">
         <v>30</v>
@@ -38037,7 +38064,7 @@
         <v>27</v>
       </c>
       <c r="K19" s="25" t="s">
-        <v>28</v>
+        <v>246</v>
       </c>
       <c r="L19" s="26">
         <v>2</v>
@@ -38048,36 +38075,38 @@
       </c>
     </row>
     <row r="20" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="63"/>
-      <c r="B20" s="64"/>
-      <c r="C20" s="65"/>
-      <c r="D20" s="66"/>
-      <c r="E20" s="67"/>
-      <c r="F20" s="68"/>
-      <c r="G20" s="69"/>
-      <c r="H20" s="70"/>
-      <c r="I20" s="71"/>
-      <c r="J20" s="71"/>
-      <c r="K20" s="71"/>
-      <c r="L20" s="72"/>
-      <c r="M20" s="73"/>
+      <c r="A20" s="62"/>
+      <c r="B20" s="63"/>
+      <c r="C20" s="64"/>
+      <c r="D20" s="65"/>
+      <c r="E20" s="66"/>
+      <c r="F20" s="67"/>
+      <c r="G20" s="68"/>
+      <c r="H20" s="69"/>
+      <c r="I20" s="70"/>
+      <c r="J20" s="70"/>
+      <c r="K20" s="25" t="s">
+        <v>246</v>
+      </c>
+      <c r="L20" s="71"/>
+      <c r="M20" s="72"/>
       <c r="N20" s="28"/>
     </row>
     <row r="21" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="17" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="C21" s="19" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="D21" s="20" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="E21" s="21" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="F21" s="22">
         <v>20</v>
@@ -38095,7 +38124,7 @@
         <v>27</v>
       </c>
       <c r="K21" s="25" t="s">
-        <v>28</v>
+        <v>246</v>
       </c>
       <c r="L21" s="26">
         <v>1</v>
@@ -38140,7 +38169,7 @@
       <c r="L22" s="26"/>
       <c r="M22" s="27"/>
       <c r="N22" s="28" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
     </row>
     <row r="23" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
@@ -38178,7 +38207,7 @@
       <c r="L23" s="26"/>
       <c r="M23" s="40"/>
       <c r="N23" s="28" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
     </row>
     <row r="24" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
@@ -38863,7 +38892,7 @@
     <col min="11" max="11" width="25.7265625" style="53" customWidth="1"/>
     <col min="12" max="12" width="21.453125" style="61" customWidth="1"/>
     <col min="13" max="13" width="22" style="57" customWidth="1"/>
-    <col min="14" max="14" width="21.7265625" style="58" customWidth="1"/>
+    <col min="14" max="14" width="39.36328125" style="58" bestFit="1" customWidth="1"/>
     <col min="15" max="16384" width="9.1796875" style="2"/>
   </cols>
   <sheetData>
@@ -38873,13 +38902,13 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46163.886088888888</v>
-      </c>
-      <c r="D1" s="62" t="s">
+        <v>46164.418156250002</v>
+      </c>
+      <c r="D1" s="77" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="62"/>
-      <c r="F1" s="62"/>
+      <c r="E1" s="77"/>
+      <c r="F1" s="77"/>
       <c r="G1" s="3"/>
       <c r="H1" s="4"/>
       <c r="I1" s="5"/>
@@ -38938,19 +38967,19 @@
     </row>
     <row r="3" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="17" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="B3" s="18" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="C3" s="19" t="s">
         <v>105</v>
       </c>
       <c r="D3" s="20" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="E3" s="21" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="F3" s="22">
         <v>50</v>
@@ -38965,10 +38994,10 @@
         <v>57</v>
       </c>
       <c r="J3" s="25" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
       <c r="K3" s="25" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="L3" s="26">
         <v>2</v>
@@ -38979,36 +39008,36 @@
       </c>
     </row>
     <row r="4" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="63"/>
-      <c r="B4" s="64"/>
-      <c r="C4" s="65"/>
-      <c r="D4" s="66"/>
-      <c r="E4" s="67"/>
-      <c r="F4" s="68"/>
-      <c r="G4" s="69"/>
-      <c r="H4" s="70"/>
-      <c r="I4" s="71"/>
+      <c r="A4" s="62"/>
+      <c r="B4" s="63"/>
+      <c r="C4" s="64"/>
+      <c r="D4" s="65"/>
+      <c r="E4" s="66"/>
+      <c r="F4" s="67"/>
+      <c r="G4" s="68"/>
+      <c r="H4" s="69"/>
+      <c r="I4" s="70"/>
       <c r="J4" s="25"/>
-      <c r="K4" s="71"/>
-      <c r="L4" s="72"/>
-      <c r="M4" s="73"/>
+      <c r="K4" s="70"/>
+      <c r="L4" s="71"/>
+      <c r="M4" s="72"/>
       <c r="N4" s="28"/>
     </row>
     <row r="5" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="17" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="C5" s="19" t="s">
         <v>39</v>
       </c>
       <c r="D5" s="20" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="E5" s="21" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="F5" s="22">
         <v>30</v>
@@ -39023,10 +39052,10 @@
         <v>57</v>
       </c>
       <c r="J5" s="25" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="K5" s="25" t="s">
-        <v>167</v>
+        <v>246</v>
       </c>
       <c r="L5" s="26">
         <v>2</v>

</xml_diff>

<commit_message>
feat: update sample production plans for BCN 1.6 and 1.6 sheets
</commit_message>
<xml_diff>
--- a/Kế hoach sản xuất Sample.xlsx
+++ b/Kế hoach sản xuất Sample.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ortholitevietnam-my.sharepoint.com/personal/lam_dv2_ortholite_vn/Documents/PROJECT LÂM/DailyFoamingReport/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="48" documentId="8_{C12FF075-160F-4BB4-977C-4D56BABB08BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{08481B9F-BFF0-4955-8A0E-BE6A8A15391F}"/>
+  <xr:revisionPtr revIDLastSave="49" documentId="8_{C12FF075-160F-4BB4-977C-4D56BABB08BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9EC64ABE-46D3-4F48-8D3B-04C5A1BCF438}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="6" xr2:uid="{E780E912-92A1-4ADF-95B1-638FE58CE194}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="8" xr2:uid="{E780E912-92A1-4ADF-95B1-638FE58CE194}"/>
   </bookViews>
   <sheets>
     <sheet name="13.5" sheetId="1" r:id="rId1"/>
@@ -21,12 +21,14 @@
     <sheet name="25.5" sheetId="6" r:id="rId6"/>
     <sheet name="27.5" sheetId="7" r:id="rId7"/>
     <sheet name="29.5 - L2" sheetId="8" r:id="rId8"/>
+    <sheet name="1.6" sheetId="9" r:id="rId9"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId9"/>
     <externalReference r:id="rId10"/>
+    <externalReference r:id="rId11"/>
   </externalReferences>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'1.6'!$A$2:$N$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'13.5'!$A$2:$N$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'15.5'!$A$2:$N$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'18.5'!$A$2:$N$3</definedName>
@@ -35,6 +37,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'25.5'!$A$2:$N$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'27.5'!$A$2:$N$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'29.5 - L2'!$A$2:$N$25</definedName>
+    <definedName name="AE" localSheetId="8">'[1]Molding-báo cáo BUn'!#REF!</definedName>
     <definedName name="AE" localSheetId="0">'[1]Molding-báo cáo BUn'!#REF!</definedName>
     <definedName name="AE" localSheetId="1">'[1]Molding-báo cáo BUn'!#REF!</definedName>
     <definedName name="AE" localSheetId="2">'[1]Molding-báo cáo BUn'!#REF!</definedName>
@@ -43,6 +46,7 @@
     <definedName name="AE" localSheetId="5">'[1]Molding-báo cáo BUn'!#REF!</definedName>
     <definedName name="AE" localSheetId="6">'[1]Molding-báo cáo BUn'!#REF!</definedName>
     <definedName name="AE" localSheetId="7">'[1]Molding-báo cáo BUn'!#REF!</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="8">'1.6'!$A$1:$N$21</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'13.5'!$A$1:$N$21</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'15.5'!$A$1:$N$24</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'18.5'!$A$1:$N$29</definedName>
@@ -51,6 +55,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="5">'25.5'!$A$1:$N$22</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="6">'27.5'!$A$1:$N$22</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="7">'29.5 - L2'!$A$1:$N$25</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="8">'1.6'!$1:$2</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'13.5'!$1:$2</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'15.5'!$1:$2</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'18.5'!$1:$2</definedName>
@@ -59,6 +64,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'25.5'!$1:$2</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'27.5'!$1:$2</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'29.5 - L2'!$1:$2</definedName>
+    <definedName name="Z_1811EAD5_BD80_4EFF_9596_8EF0EFF4AD2A_.wvu.FilterData" localSheetId="8" hidden="1">'1.6'!$A$2:$N$2</definedName>
     <definedName name="Z_1811EAD5_BD80_4EFF_9596_8EF0EFF4AD2A_.wvu.FilterData" localSheetId="0" hidden="1">'13.5'!$A$2:$N$2</definedName>
     <definedName name="Z_1811EAD5_BD80_4EFF_9596_8EF0EFF4AD2A_.wvu.FilterData" localSheetId="1" hidden="1">'15.5'!$A$2:$N$2</definedName>
     <definedName name="Z_1811EAD5_BD80_4EFF_9596_8EF0EFF4AD2A_.wvu.FilterData" localSheetId="2" hidden="1">'18.5'!$A$2:$N$2</definedName>
@@ -67,6 +73,7 @@
     <definedName name="Z_1811EAD5_BD80_4EFF_9596_8EF0EFF4AD2A_.wvu.FilterData" localSheetId="5" hidden="1">'25.5'!$A$2:$N$2</definedName>
     <definedName name="Z_1811EAD5_BD80_4EFF_9596_8EF0EFF4AD2A_.wvu.FilterData" localSheetId="6" hidden="1">'27.5'!$A$2:$N$2</definedName>
     <definedName name="Z_1811EAD5_BD80_4EFF_9596_8EF0EFF4AD2A_.wvu.FilterData" localSheetId="7" hidden="1">'29.5 - L2'!$A$2:$N$2</definedName>
+    <definedName name="Z_1811EAD5_BD80_4EFF_9596_8EF0EFF4AD2A_.wvu.PrintTitles" localSheetId="8" hidden="1">'1.6'!$1:$2</definedName>
     <definedName name="Z_1811EAD5_BD80_4EFF_9596_8EF0EFF4AD2A_.wvu.PrintTitles" localSheetId="0" hidden="1">'13.5'!$1:$2</definedName>
     <definedName name="Z_1811EAD5_BD80_4EFF_9596_8EF0EFF4AD2A_.wvu.PrintTitles" localSheetId="1" hidden="1">'15.5'!$1:$2</definedName>
     <definedName name="Z_1811EAD5_BD80_4EFF_9596_8EF0EFF4AD2A_.wvu.PrintTitles" localSheetId="2" hidden="1">'18.5'!$1:$2</definedName>
@@ -75,6 +82,7 @@
     <definedName name="Z_1811EAD5_BD80_4EFF_9596_8EF0EFF4AD2A_.wvu.PrintTitles" localSheetId="5" hidden="1">'25.5'!$1:$2</definedName>
     <definedName name="Z_1811EAD5_BD80_4EFF_9596_8EF0EFF4AD2A_.wvu.PrintTitles" localSheetId="6" hidden="1">'27.5'!$1:$2</definedName>
     <definedName name="Z_1811EAD5_BD80_4EFF_9596_8EF0EFF4AD2A_.wvu.PrintTitles" localSheetId="7" hidden="1">'29.5 - L2'!$1:$2</definedName>
+    <definedName name="Z_18A7E0A3_1642_489C_8130_3CC9FF80B04E_.wvu.FilterData" localSheetId="8" hidden="1">'1.6'!$B$2:$M$2</definedName>
     <definedName name="Z_18A7E0A3_1642_489C_8130_3CC9FF80B04E_.wvu.FilterData" localSheetId="0" hidden="1">'13.5'!$B$2:$M$2</definedName>
     <definedName name="Z_18A7E0A3_1642_489C_8130_3CC9FF80B04E_.wvu.FilterData" localSheetId="1" hidden="1">'15.5'!$B$2:$M$2</definedName>
     <definedName name="Z_18A7E0A3_1642_489C_8130_3CC9FF80B04E_.wvu.FilterData" localSheetId="2" hidden="1">'18.5'!$B$2:$M$2</definedName>
@@ -83,6 +91,7 @@
     <definedName name="Z_18A7E0A3_1642_489C_8130_3CC9FF80B04E_.wvu.FilterData" localSheetId="5" hidden="1">'25.5'!$B$2:$M$2</definedName>
     <definedName name="Z_18A7E0A3_1642_489C_8130_3CC9FF80B04E_.wvu.FilterData" localSheetId="6" hidden="1">'27.5'!$B$2:$M$2</definedName>
     <definedName name="Z_18A7E0A3_1642_489C_8130_3CC9FF80B04E_.wvu.FilterData" localSheetId="7" hidden="1">'29.5 - L2'!$B$2:$M$2</definedName>
+    <definedName name="Z_2653C0F9_59B0_4DB3_BD8D_CACC833527F0_.wvu.FilterData" localSheetId="8" hidden="1">'1.6'!$A$2:$N$2</definedName>
     <definedName name="Z_2653C0F9_59B0_4DB3_BD8D_CACC833527F0_.wvu.FilterData" localSheetId="0" hidden="1">'13.5'!$A$2:$N$2</definedName>
     <definedName name="Z_2653C0F9_59B0_4DB3_BD8D_CACC833527F0_.wvu.FilterData" localSheetId="1" hidden="1">'15.5'!$A$2:$N$2</definedName>
     <definedName name="Z_2653C0F9_59B0_4DB3_BD8D_CACC833527F0_.wvu.FilterData" localSheetId="2" hidden="1">'18.5'!$A$2:$N$2</definedName>
@@ -91,6 +100,7 @@
     <definedName name="Z_2653C0F9_59B0_4DB3_BD8D_CACC833527F0_.wvu.FilterData" localSheetId="5" hidden="1">'25.5'!$A$2:$N$2</definedName>
     <definedName name="Z_2653C0F9_59B0_4DB3_BD8D_CACC833527F0_.wvu.FilterData" localSheetId="6" hidden="1">'27.5'!$A$2:$N$2</definedName>
     <definedName name="Z_2653C0F9_59B0_4DB3_BD8D_CACC833527F0_.wvu.FilterData" localSheetId="7" hidden="1">'29.5 - L2'!$A$2:$N$2</definedName>
+    <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.FilterData" localSheetId="8" hidden="1">'1.6'!$A$2:$N$2</definedName>
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.FilterData" localSheetId="0" hidden="1">'13.5'!$A$2:$N$2</definedName>
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.FilterData" localSheetId="1" hidden="1">'15.5'!$A$2:$N$2</definedName>
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.FilterData" localSheetId="2" hidden="1">'18.5'!$A$2:$N$2</definedName>
@@ -99,6 +109,7 @@
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.FilterData" localSheetId="5" hidden="1">'25.5'!$A$2:$N$2</definedName>
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.FilterData" localSheetId="6" hidden="1">'27.5'!$A$2:$N$2</definedName>
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.FilterData" localSheetId="7" hidden="1">'29.5 - L2'!$A$2:$N$2</definedName>
+    <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.PrintTitles" localSheetId="8" hidden="1">'1.6'!$1:$2</definedName>
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.PrintTitles" localSheetId="0" hidden="1">'13.5'!$1:$2</definedName>
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.PrintTitles" localSheetId="1" hidden="1">'15.5'!$1:$2</definedName>
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.PrintTitles" localSheetId="2" hidden="1">'18.5'!$1:$2</definedName>
@@ -107,6 +118,7 @@
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.PrintTitles" localSheetId="5" hidden="1">'25.5'!$1:$2</definedName>
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.PrintTitles" localSheetId="6" hidden="1">'27.5'!$1:$2</definedName>
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.PrintTitles" localSheetId="7" hidden="1">'29.5 - L2'!$1:$2</definedName>
+    <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.Rows" localSheetId="8" hidden="1">'1.6'!#REF!</definedName>
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.Rows" localSheetId="0" hidden="1">'13.5'!#REF!</definedName>
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.Rows" localSheetId="1" hidden="1">'15.5'!#REF!</definedName>
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.Rows" localSheetId="2" hidden="1">'18.5'!#REF!</definedName>
@@ -115,6 +127,7 @@
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.Rows" localSheetId="5" hidden="1">'25.5'!#REF!</definedName>
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.Rows" localSheetId="6" hidden="1">'27.5'!#REF!</definedName>
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.Rows" localSheetId="7" hidden="1">'29.5 - L2'!#REF!</definedName>
+    <definedName name="Z_314949E3_0D3B_4560_AE70_4D3C4970782A_.wvu.FilterData" localSheetId="8" hidden="1">'1.6'!$B$2:$M$2</definedName>
     <definedName name="Z_314949E3_0D3B_4560_AE70_4D3C4970782A_.wvu.FilterData" localSheetId="0" hidden="1">'13.5'!$B$2:$M$2</definedName>
     <definedName name="Z_314949E3_0D3B_4560_AE70_4D3C4970782A_.wvu.FilterData" localSheetId="1" hidden="1">'15.5'!$B$2:$M$2</definedName>
     <definedName name="Z_314949E3_0D3B_4560_AE70_4D3C4970782A_.wvu.FilterData" localSheetId="2" hidden="1">'18.5'!$B$2:$M$2</definedName>
@@ -123,6 +136,7 @@
     <definedName name="Z_314949E3_0D3B_4560_AE70_4D3C4970782A_.wvu.FilterData" localSheetId="5" hidden="1">'25.5'!$B$2:$M$2</definedName>
     <definedName name="Z_314949E3_0D3B_4560_AE70_4D3C4970782A_.wvu.FilterData" localSheetId="6" hidden="1">'27.5'!$B$2:$M$2</definedName>
     <definedName name="Z_314949E3_0D3B_4560_AE70_4D3C4970782A_.wvu.FilterData" localSheetId="7" hidden="1">'29.5 - L2'!$B$2:$M$2</definedName>
+    <definedName name="Z_318C8B1E_0627_4DC9_8089_60901FDA475B_.wvu.FilterData" localSheetId="8" hidden="1">'1.6'!$B$2:$N$2</definedName>
     <definedName name="Z_318C8B1E_0627_4DC9_8089_60901FDA475B_.wvu.FilterData" localSheetId="0" hidden="1">'13.5'!$B$2:$N$2</definedName>
     <definedName name="Z_318C8B1E_0627_4DC9_8089_60901FDA475B_.wvu.FilterData" localSheetId="1" hidden="1">'15.5'!$B$2:$N$2</definedName>
     <definedName name="Z_318C8B1E_0627_4DC9_8089_60901FDA475B_.wvu.FilterData" localSheetId="2" hidden="1">'18.5'!$B$2:$N$2</definedName>
@@ -131,6 +145,7 @@
     <definedName name="Z_318C8B1E_0627_4DC9_8089_60901FDA475B_.wvu.FilterData" localSheetId="5" hidden="1">'25.5'!$B$2:$N$2</definedName>
     <definedName name="Z_318C8B1E_0627_4DC9_8089_60901FDA475B_.wvu.FilterData" localSheetId="6" hidden="1">'27.5'!$B$2:$N$2</definedName>
     <definedName name="Z_318C8B1E_0627_4DC9_8089_60901FDA475B_.wvu.FilterData" localSheetId="7" hidden="1">'29.5 - L2'!$B$2:$N$2</definedName>
+    <definedName name="Z_318C8B1E_0627_4DC9_8089_60901FDA475B_.wvu.PrintTitles" localSheetId="8" hidden="1">'1.6'!$1:$2</definedName>
     <definedName name="Z_318C8B1E_0627_4DC9_8089_60901FDA475B_.wvu.PrintTitles" localSheetId="0" hidden="1">'13.5'!$1:$2</definedName>
     <definedName name="Z_318C8B1E_0627_4DC9_8089_60901FDA475B_.wvu.PrintTitles" localSheetId="1" hidden="1">'15.5'!$1:$2</definedName>
     <definedName name="Z_318C8B1E_0627_4DC9_8089_60901FDA475B_.wvu.PrintTitles" localSheetId="2" hidden="1">'18.5'!$1:$2</definedName>
@@ -139,6 +154,7 @@
     <definedName name="Z_318C8B1E_0627_4DC9_8089_60901FDA475B_.wvu.PrintTitles" localSheetId="5" hidden="1">'25.5'!$1:$2</definedName>
     <definedName name="Z_318C8B1E_0627_4DC9_8089_60901FDA475B_.wvu.PrintTitles" localSheetId="6" hidden="1">'27.5'!$1:$2</definedName>
     <definedName name="Z_318C8B1E_0627_4DC9_8089_60901FDA475B_.wvu.PrintTitles" localSheetId="7" hidden="1">'29.5 - L2'!$1:$2</definedName>
+    <definedName name="Z_323B6797_06D8_47A1_B001_797373BE57F2_.wvu.FilterData" localSheetId="8" hidden="1">'1.6'!$B$2:$M$2</definedName>
     <definedName name="Z_323B6797_06D8_47A1_B001_797373BE57F2_.wvu.FilterData" localSheetId="0" hidden="1">'13.5'!$B$2:$M$2</definedName>
     <definedName name="Z_323B6797_06D8_47A1_B001_797373BE57F2_.wvu.FilterData" localSheetId="1" hidden="1">'15.5'!$B$2:$M$2</definedName>
     <definedName name="Z_323B6797_06D8_47A1_B001_797373BE57F2_.wvu.FilterData" localSheetId="2" hidden="1">'18.5'!$B$2:$M$2</definedName>
@@ -147,6 +163,7 @@
     <definedName name="Z_323B6797_06D8_47A1_B001_797373BE57F2_.wvu.FilterData" localSheetId="5" hidden="1">'25.5'!$B$2:$M$2</definedName>
     <definedName name="Z_323B6797_06D8_47A1_B001_797373BE57F2_.wvu.FilterData" localSheetId="6" hidden="1">'27.5'!$B$2:$M$2</definedName>
     <definedName name="Z_323B6797_06D8_47A1_B001_797373BE57F2_.wvu.FilterData" localSheetId="7" hidden="1">'29.5 - L2'!$B$2:$M$2</definedName>
+    <definedName name="Z_6A9DC2EA_1959_4EB9_A839_907E58591C36_.wvu.FilterData" localSheetId="8" hidden="1">'1.6'!$B$2:$M$2</definedName>
     <definedName name="Z_6A9DC2EA_1959_4EB9_A839_907E58591C36_.wvu.FilterData" localSheetId="0" hidden="1">'13.5'!$B$2:$M$2</definedName>
     <definedName name="Z_6A9DC2EA_1959_4EB9_A839_907E58591C36_.wvu.FilterData" localSheetId="1" hidden="1">'15.5'!$B$2:$M$2</definedName>
     <definedName name="Z_6A9DC2EA_1959_4EB9_A839_907E58591C36_.wvu.FilterData" localSheetId="2" hidden="1">'18.5'!$B$2:$M$2</definedName>
@@ -155,6 +172,7 @@
     <definedName name="Z_6A9DC2EA_1959_4EB9_A839_907E58591C36_.wvu.FilterData" localSheetId="5" hidden="1">'25.5'!$B$2:$M$2</definedName>
     <definedName name="Z_6A9DC2EA_1959_4EB9_A839_907E58591C36_.wvu.FilterData" localSheetId="6" hidden="1">'27.5'!$B$2:$M$2</definedName>
     <definedName name="Z_6A9DC2EA_1959_4EB9_A839_907E58591C36_.wvu.FilterData" localSheetId="7" hidden="1">'29.5 - L2'!$B$2:$M$2</definedName>
+    <definedName name="Z_866BE165_7CE2_41D4_AD4C_D79698D432B1_.wvu.FilterData" localSheetId="8" hidden="1">'1.6'!$B$2:$M$2</definedName>
     <definedName name="Z_866BE165_7CE2_41D4_AD4C_D79698D432B1_.wvu.FilterData" localSheetId="0" hidden="1">'13.5'!$B$2:$M$2</definedName>
     <definedName name="Z_866BE165_7CE2_41D4_AD4C_D79698D432B1_.wvu.FilterData" localSheetId="1" hidden="1">'15.5'!$B$2:$M$2</definedName>
     <definedName name="Z_866BE165_7CE2_41D4_AD4C_D79698D432B1_.wvu.FilterData" localSheetId="2" hidden="1">'18.5'!$B$2:$M$2</definedName>
@@ -163,6 +181,7 @@
     <definedName name="Z_866BE165_7CE2_41D4_AD4C_D79698D432B1_.wvu.FilterData" localSheetId="5" hidden="1">'25.5'!$B$2:$M$2</definedName>
     <definedName name="Z_866BE165_7CE2_41D4_AD4C_D79698D432B1_.wvu.FilterData" localSheetId="6" hidden="1">'27.5'!$B$2:$M$2</definedName>
     <definedName name="Z_866BE165_7CE2_41D4_AD4C_D79698D432B1_.wvu.FilterData" localSheetId="7" hidden="1">'29.5 - L2'!$B$2:$M$2</definedName>
+    <definedName name="Z_866CB300_9BE2_4E49_BCB4_72634A7939D7_.wvu.FilterData" localSheetId="8" hidden="1">'1.6'!$B$2:$N$2</definedName>
     <definedName name="Z_866CB300_9BE2_4E49_BCB4_72634A7939D7_.wvu.FilterData" localSheetId="0" hidden="1">'13.5'!$B$2:$N$2</definedName>
     <definedName name="Z_866CB300_9BE2_4E49_BCB4_72634A7939D7_.wvu.FilterData" localSheetId="1" hidden="1">'15.5'!$B$2:$N$2</definedName>
     <definedName name="Z_866CB300_9BE2_4E49_BCB4_72634A7939D7_.wvu.FilterData" localSheetId="2" hidden="1">'18.5'!$B$2:$N$2</definedName>
@@ -171,6 +190,7 @@
     <definedName name="Z_866CB300_9BE2_4E49_BCB4_72634A7939D7_.wvu.FilterData" localSheetId="5" hidden="1">'25.5'!$B$2:$N$2</definedName>
     <definedName name="Z_866CB300_9BE2_4E49_BCB4_72634A7939D7_.wvu.FilterData" localSheetId="6" hidden="1">'27.5'!$B$2:$N$2</definedName>
     <definedName name="Z_866CB300_9BE2_4E49_BCB4_72634A7939D7_.wvu.FilterData" localSheetId="7" hidden="1">'29.5 - L2'!$B$2:$N$2</definedName>
+    <definedName name="Z_8CF255E0_B8BB_4016_A366_4FCF106965CF_.wvu.FilterData" localSheetId="8" hidden="1">'1.6'!$A$2:$N$2</definedName>
     <definedName name="Z_8CF255E0_B8BB_4016_A366_4FCF106965CF_.wvu.FilterData" localSheetId="0" hidden="1">'13.5'!$A$2:$N$2</definedName>
     <definedName name="Z_8CF255E0_B8BB_4016_A366_4FCF106965CF_.wvu.FilterData" localSheetId="1" hidden="1">'15.5'!$A$2:$N$2</definedName>
     <definedName name="Z_8CF255E0_B8BB_4016_A366_4FCF106965CF_.wvu.FilterData" localSheetId="2" hidden="1">'18.5'!$A$2:$N$2</definedName>
@@ -179,6 +199,7 @@
     <definedName name="Z_8CF255E0_B8BB_4016_A366_4FCF106965CF_.wvu.FilterData" localSheetId="5" hidden="1">'25.5'!$A$2:$N$2</definedName>
     <definedName name="Z_8CF255E0_B8BB_4016_A366_4FCF106965CF_.wvu.FilterData" localSheetId="6" hidden="1">'27.5'!$A$2:$N$2</definedName>
     <definedName name="Z_8CF255E0_B8BB_4016_A366_4FCF106965CF_.wvu.FilterData" localSheetId="7" hidden="1">'29.5 - L2'!$A$2:$N$2</definedName>
+    <definedName name="Z_A4A1FC39_A54C_43AC_9912_8824EB6833F5_.wvu.FilterData" localSheetId="8" hidden="1">'1.6'!$A$2:$N$2</definedName>
     <definedName name="Z_A4A1FC39_A54C_43AC_9912_8824EB6833F5_.wvu.FilterData" localSheetId="0" hidden="1">'13.5'!$A$2:$N$2</definedName>
     <definedName name="Z_A4A1FC39_A54C_43AC_9912_8824EB6833F5_.wvu.FilterData" localSheetId="1" hidden="1">'15.5'!$A$2:$N$2</definedName>
     <definedName name="Z_A4A1FC39_A54C_43AC_9912_8824EB6833F5_.wvu.FilterData" localSheetId="2" hidden="1">'18.5'!$A$2:$N$2</definedName>
@@ -187,6 +208,7 @@
     <definedName name="Z_A4A1FC39_A54C_43AC_9912_8824EB6833F5_.wvu.FilterData" localSheetId="5" hidden="1">'25.5'!$A$2:$N$2</definedName>
     <definedName name="Z_A4A1FC39_A54C_43AC_9912_8824EB6833F5_.wvu.FilterData" localSheetId="6" hidden="1">'27.5'!$A$2:$N$2</definedName>
     <definedName name="Z_A4A1FC39_A54C_43AC_9912_8824EB6833F5_.wvu.FilterData" localSheetId="7" hidden="1">'29.5 - L2'!$A$2:$N$2</definedName>
+    <definedName name="Z_AF6B2EAC_2950_4809_A605_2107D254FC8D_.wvu.FilterData" localSheetId="8" hidden="1">'1.6'!$B$2:$N$2</definedName>
     <definedName name="Z_AF6B2EAC_2950_4809_A605_2107D254FC8D_.wvu.FilterData" localSheetId="0" hidden="1">'13.5'!$B$2:$N$2</definedName>
     <definedName name="Z_AF6B2EAC_2950_4809_A605_2107D254FC8D_.wvu.FilterData" localSheetId="1" hidden="1">'15.5'!$B$2:$N$2</definedName>
     <definedName name="Z_AF6B2EAC_2950_4809_A605_2107D254FC8D_.wvu.FilterData" localSheetId="2" hidden="1">'18.5'!$B$2:$N$2</definedName>
@@ -195,6 +217,7 @@
     <definedName name="Z_AF6B2EAC_2950_4809_A605_2107D254FC8D_.wvu.FilterData" localSheetId="5" hidden="1">'25.5'!$B$2:$N$2</definedName>
     <definedName name="Z_AF6B2EAC_2950_4809_A605_2107D254FC8D_.wvu.FilterData" localSheetId="6" hidden="1">'27.5'!$B$2:$N$2</definedName>
     <definedName name="Z_AF6B2EAC_2950_4809_A605_2107D254FC8D_.wvu.FilterData" localSheetId="7" hidden="1">'29.5 - L2'!$B$2:$N$2</definedName>
+    <definedName name="Z_AF6B2EAC_2950_4809_A605_2107D254FC8D_.wvu.PrintTitles" localSheetId="8" hidden="1">'1.6'!$1:$2</definedName>
     <definedName name="Z_AF6B2EAC_2950_4809_A605_2107D254FC8D_.wvu.PrintTitles" localSheetId="0" hidden="1">'13.5'!$1:$2</definedName>
     <definedName name="Z_AF6B2EAC_2950_4809_A605_2107D254FC8D_.wvu.PrintTitles" localSheetId="1" hidden="1">'15.5'!$1:$2</definedName>
     <definedName name="Z_AF6B2EAC_2950_4809_A605_2107D254FC8D_.wvu.PrintTitles" localSheetId="2" hidden="1">'18.5'!$1:$2</definedName>
@@ -203,6 +226,7 @@
     <definedName name="Z_AF6B2EAC_2950_4809_A605_2107D254FC8D_.wvu.PrintTitles" localSheetId="5" hidden="1">'25.5'!$1:$2</definedName>
     <definedName name="Z_AF6B2EAC_2950_4809_A605_2107D254FC8D_.wvu.PrintTitles" localSheetId="6" hidden="1">'27.5'!$1:$2</definedName>
     <definedName name="Z_AF6B2EAC_2950_4809_A605_2107D254FC8D_.wvu.PrintTitles" localSheetId="7" hidden="1">'29.5 - L2'!$1:$2</definedName>
+    <definedName name="Z_CA92E8A2_92C9_4575_A139_6FE5DA69269F_.wvu.FilterData" localSheetId="8" hidden="1">'1.6'!$B$2:$M$2</definedName>
     <definedName name="Z_CA92E8A2_92C9_4575_A139_6FE5DA69269F_.wvu.FilterData" localSheetId="0" hidden="1">'13.5'!$B$2:$M$2</definedName>
     <definedName name="Z_CA92E8A2_92C9_4575_A139_6FE5DA69269F_.wvu.FilterData" localSheetId="1" hidden="1">'15.5'!$B$2:$M$2</definedName>
     <definedName name="Z_CA92E8A2_92C9_4575_A139_6FE5DA69269F_.wvu.FilterData" localSheetId="2" hidden="1">'18.5'!$B$2:$M$2</definedName>
@@ -211,6 +235,7 @@
     <definedName name="Z_CA92E8A2_92C9_4575_A139_6FE5DA69269F_.wvu.FilterData" localSheetId="5" hidden="1">'25.5'!$B$2:$M$2</definedName>
     <definedName name="Z_CA92E8A2_92C9_4575_A139_6FE5DA69269F_.wvu.FilterData" localSheetId="6" hidden="1">'27.5'!$B$2:$M$2</definedName>
     <definedName name="Z_CA92E8A2_92C9_4575_A139_6FE5DA69269F_.wvu.FilterData" localSheetId="7" hidden="1">'29.5 - L2'!$B$2:$M$2</definedName>
+    <definedName name="Z_DF644A2B_B913_48D6_B430_E57F3B482B79_.wvu.FilterData" localSheetId="8" hidden="1">'1.6'!$A$2:$N$2</definedName>
     <definedName name="Z_DF644A2B_B913_48D6_B430_E57F3B482B79_.wvu.FilterData" localSheetId="0" hidden="1">'13.5'!$A$2:$N$2</definedName>
     <definedName name="Z_DF644A2B_B913_48D6_B430_E57F3B482B79_.wvu.FilterData" localSheetId="1" hidden="1">'15.5'!$A$2:$N$2</definedName>
     <definedName name="Z_DF644A2B_B913_48D6_B430_E57F3B482B79_.wvu.FilterData" localSheetId="2" hidden="1">'18.5'!$A$2:$N$2</definedName>
@@ -219,6 +244,7 @@
     <definedName name="Z_DF644A2B_B913_48D6_B430_E57F3B482B79_.wvu.FilterData" localSheetId="5" hidden="1">'25.5'!$A$2:$N$2</definedName>
     <definedName name="Z_DF644A2B_B913_48D6_B430_E57F3B482B79_.wvu.FilterData" localSheetId="6" hidden="1">'27.5'!$A$2:$N$2</definedName>
     <definedName name="Z_DF644A2B_B913_48D6_B430_E57F3B482B79_.wvu.FilterData" localSheetId="7" hidden="1">'29.5 - L2'!$A$2:$N$2</definedName>
+    <definedName name="Z_DF644A2B_B913_48D6_B430_E57F3B482B79_.wvu.PrintTitles" localSheetId="8" hidden="1">'1.6'!$1:$2</definedName>
     <definedName name="Z_DF644A2B_B913_48D6_B430_E57F3B482B79_.wvu.PrintTitles" localSheetId="0" hidden="1">'13.5'!$1:$2</definedName>
     <definedName name="Z_DF644A2B_B913_48D6_B430_E57F3B482B79_.wvu.PrintTitles" localSheetId="1" hidden="1">'15.5'!$1:$2</definedName>
     <definedName name="Z_DF644A2B_B913_48D6_B430_E57F3B482B79_.wvu.PrintTitles" localSheetId="2" hidden="1">'18.5'!$1:$2</definedName>
@@ -249,7 +275,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="729" uniqueCount="355">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="786" uniqueCount="378">
   <si>
     <t>Release Date</t>
   </si>
@@ -1393,6 +1419,75 @@
   <si>
     <t>OrthoLite Regular NEUTRAL GRAY/17-4402TPX Flat Sheet 0.15D 45+/-4 Asker C 1.1M 1.7M 9.8mm</t>
   </si>
+  <si>
+    <t>S-2026-05-102</t>
+  </si>
+  <si>
+    <t>RPRO-260601-0847</t>
+  </si>
+  <si>
+    <t>S-2026-05-103</t>
+  </si>
+  <si>
+    <t>RPRO-260601-0848</t>
+  </si>
+  <si>
+    <t>PVN-002973</t>
+  </si>
+  <si>
+    <t>UltraLite-Hybrid OrthoLite SEEDPEARL/12-0703TPX Hybrid Flat Sheet 0.085D 25+/-4 Asker C 1.1M 2M 4.5mm</t>
+  </si>
+  <si>
+    <t>S-2026-05-104</t>
+  </si>
+  <si>
+    <t>RPRO-260601-0849</t>
+  </si>
+  <si>
+    <t>PVN-002465</t>
+  </si>
+  <si>
+    <t>OrthoLite Regular-Hybrid SEEDPEARL/12-0703TPX Hybrid Flat Sheet 0.11D 25+/-4 Asker C 1.1M 2M 5mm</t>
+  </si>
+  <si>
+    <t>S-2026-05-105</t>
+  </si>
+  <si>
+    <t>RPRO-260601-0850</t>
+  </si>
+  <si>
+    <t>PVN-003630</t>
+  </si>
+  <si>
+    <t>OrthoLite Ultra GREEN/16-5932TPX Flat Sheet 0.085D 25+/-4 Asker C 1.1M 2M 2mm</t>
+  </si>
+  <si>
+    <t>UNDER ARMOUR</t>
+  </si>
+  <si>
+    <t>SSO-2606-00021    - URGENT (6-8)</t>
+  </si>
+  <si>
+    <t>S-2026-05-106</t>
+  </si>
+  <si>
+    <t>RPRO-260601-0851</t>
+  </si>
+  <si>
+    <t>BDB-000180</t>
+  </si>
+  <si>
+    <t>PVN-003236</t>
+  </si>
+  <si>
+    <t>OrthoLite Eco LT-Hybrid-Converse SEEDPEARL/12-0703TPX Hybrid Flat Sheet 0.13D 25+/-4 Asker C 1.1M 2M 5mm</t>
+  </si>
+  <si>
+    <t>CONVERSE</t>
+  </si>
+  <si>
+    <t>Die cut</t>
+  </si>
 </sst>
 </file>
 
@@ -1993,7 +2088,77 @@
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="64">
+  <dxfs count="71">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2794,6 +2959,7 @@
       <sheetName val="12.5"/>
       <sheetName val="13.5"/>
       <sheetName val="15.5"/>
+      <sheetName val="BCN 1.6"/>
       <sheetName val="18.5"/>
       <sheetName val="20.5"/>
       <sheetName val="21.5"/>
@@ -2801,13 +2967,15 @@
       <sheetName val="25.5"/>
       <sheetName val="27.5"/>
       <sheetName val="29.5"/>
-      <sheetName val="form 2 (14)"/>
+      <sheetName val="29.5 - L2"/>
+      <sheetName val="1.6"/>
+      <sheetName val="form 2 (16)"/>
       <sheetName val="In đơn"/>
       <sheetName val="Production BOM"/>
       <sheetName val="Items"/>
       <sheetName val="mm Pu"/>
       <sheetName val="master plan (2)"/>
-      <sheetName val="29.5 - L2"/>
+      <sheetName val="form 2 (14)"/>
       <sheetName val="form 2 (15)"/>
       <sheetName val="MỚI (2)"/>
       <sheetName val="Sheet1"/>
@@ -34345,10 +34513,10 @@
             <v>100</v>
           </cell>
           <cell r="J462">
-            <v>0</v>
+            <v>100</v>
           </cell>
           <cell r="K462">
-            <v>100</v>
+            <v>0</v>
           </cell>
           <cell r="L462" t="str">
             <v>ADIDAS</v>
@@ -34416,10 +34584,10 @@
             <v>100</v>
           </cell>
           <cell r="J463">
-            <v>0</v>
+            <v>100</v>
           </cell>
           <cell r="K463">
-            <v>100</v>
+            <v>0</v>
           </cell>
           <cell r="L463" t="str">
             <v>ADIDAS</v>
@@ -34724,7 +34892,7 @@
             <v>46176</v>
           </cell>
           <cell r="R467">
-            <v>46173</v>
+            <v>46172</v>
           </cell>
           <cell r="S467">
             <v>6</v>
@@ -34824,7 +34992,7 @@
             <v>PUR2605280001S</v>
           </cell>
           <cell r="E469" t="str">
-            <v/>
+            <v>BDB-000058</v>
           </cell>
           <cell r="F469" t="str">
             <v>PVN-001277</v>
@@ -34842,7 +35010,7 @@
             <v>0</v>
           </cell>
           <cell r="K469">
-            <v>0</v>
+            <v>50</v>
           </cell>
           <cell r="L469" t="str">
             <v>ADIDAS</v>
@@ -34871,14 +35039,14 @@
           <cell r="T469">
             <v>7</v>
           </cell>
-          <cell r="U469" t="str">
-            <v/>
+          <cell r="U469">
+            <v>4</v>
           </cell>
           <cell r="V469">
-            <v>0</v>
+            <v>2.8570000000000002E-2</v>
           </cell>
           <cell r="W469">
-            <v>0</v>
+            <v>2</v>
           </cell>
         </row>
         <row r="470">
@@ -34895,7 +35063,7 @@
             <v>PUR2600502900001S</v>
           </cell>
           <cell r="E470" t="str">
-            <v/>
+            <v>BDB-000123</v>
           </cell>
           <cell r="F470" t="str">
             <v>PVN-003815</v>
@@ -34913,7 +35081,7 @@
             <v>0</v>
           </cell>
           <cell r="K470">
-            <v>0</v>
+            <v>30</v>
           </cell>
           <cell r="L470" t="str">
             <v>FOOTJOY</v>
@@ -34942,14 +35110,14 @@
           <cell r="T470">
             <v>6</v>
           </cell>
-          <cell r="U470" t="str">
-            <v/>
+          <cell r="U470">
+            <v>6</v>
           </cell>
           <cell r="V470">
-            <v>0</v>
+            <v>4.3479999999999998E-2</v>
           </cell>
           <cell r="W470">
-            <v>0</v>
+            <v>2</v>
           </cell>
         </row>
         <row r="471">
@@ -34966,7 +35134,7 @@
             <v>PUR2600502900001S</v>
           </cell>
           <cell r="E471" t="str">
-            <v/>
+            <v>BDB-000314</v>
           </cell>
           <cell r="F471" t="str">
             <v>PVN-004066</v>
@@ -34984,7 +35152,7 @@
             <v>0</v>
           </cell>
           <cell r="K471">
-            <v>0</v>
+            <v>30</v>
           </cell>
           <cell r="L471" t="str">
             <v>FOOTJOY</v>
@@ -35013,14 +35181,14 @@
           <cell r="T471">
             <v>7</v>
           </cell>
-          <cell r="U471" t="str">
-            <v/>
+          <cell r="U471">
+            <v>9.5</v>
           </cell>
           <cell r="V471">
-            <v>0</v>
+            <v>7.1429999999999993E-2</v>
           </cell>
           <cell r="W471">
-            <v>0</v>
+            <v>3</v>
           </cell>
         </row>
         <row r="472">
@@ -35037,7 +35205,7 @@
             <v>PUR2600502900001S</v>
           </cell>
           <cell r="E472" t="str">
-            <v/>
+            <v>BDB-000382</v>
           </cell>
           <cell r="F472" t="str">
             <v>PVN-004363</v>
@@ -35055,7 +35223,7 @@
             <v>0</v>
           </cell>
           <cell r="K472">
-            <v>0</v>
+            <v>20</v>
           </cell>
           <cell r="L472" t="str">
             <v>FOOTJOY</v>
@@ -35084,14 +35252,14 @@
           <cell r="T472">
             <v>7</v>
           </cell>
-          <cell r="U472" t="str">
-            <v/>
+          <cell r="U472">
+            <v>9.5</v>
           </cell>
           <cell r="V472">
-            <v>0</v>
+            <v>6.6669999999999993E-2</v>
           </cell>
           <cell r="W472">
-            <v>0</v>
+            <v>2</v>
           </cell>
         </row>
         <row r="473">
@@ -35108,7 +35276,7 @@
             <v>PUR2600502900001S</v>
           </cell>
           <cell r="E473" t="str">
-            <v/>
+            <v>BDB-000387</v>
           </cell>
           <cell r="F473" t="str">
             <v>PVN-004385</v>
@@ -35126,7 +35294,7 @@
             <v>0</v>
           </cell>
           <cell r="K473">
-            <v>0</v>
+            <v>20</v>
           </cell>
           <cell r="L473" t="str">
             <v>FOOTJOY</v>
@@ -35155,14 +35323,14 @@
           <cell r="T473">
             <v>7</v>
           </cell>
-          <cell r="U473" t="str">
-            <v/>
+          <cell r="U473">
+            <v>9.5</v>
           </cell>
           <cell r="V473">
-            <v>0</v>
+            <v>6.6669999999999993E-2</v>
           </cell>
           <cell r="W473">
-            <v>0</v>
+            <v>2</v>
           </cell>
         </row>
         <row r="474">
@@ -35179,7 +35347,7 @@
             <v>PUR2600502900001S</v>
           </cell>
           <cell r="E474" t="str">
-            <v/>
+            <v>BDB-000378</v>
           </cell>
           <cell r="F474" t="str">
             <v>PVN-004336</v>
@@ -35197,7 +35365,7 @@
             <v>0</v>
           </cell>
           <cell r="K474">
-            <v>0</v>
+            <v>20</v>
           </cell>
           <cell r="L474" t="str">
             <v>FOOTJOY</v>
@@ -35226,14 +35394,14 @@
           <cell r="T474">
             <v>7</v>
           </cell>
-          <cell r="U474" t="str">
-            <v/>
+          <cell r="U474">
+            <v>9.8000000000000007</v>
           </cell>
           <cell r="V474">
-            <v>0</v>
+            <v>7.1429999999999993E-2</v>
           </cell>
           <cell r="W474">
-            <v>0</v>
+            <v>2</v>
           </cell>
         </row>
         <row r="475">
@@ -35250,7 +35418,7 @@
             <v>PUR2600502900001S</v>
           </cell>
           <cell r="E475" t="str">
-            <v/>
+            <v>BDB-000291</v>
           </cell>
           <cell r="F475" t="str">
             <v>PVN-004250</v>
@@ -35268,7 +35436,7 @@
             <v>0</v>
           </cell>
           <cell r="K475">
-            <v>0</v>
+            <v>30</v>
           </cell>
           <cell r="L475" t="str">
             <v>FOOTJOY</v>
@@ -35297,14 +35465,14 @@
           <cell r="T475">
             <v>7</v>
           </cell>
-          <cell r="U475" t="str">
-            <v/>
+          <cell r="U475">
+            <v>9.8000000000000007</v>
           </cell>
           <cell r="V475">
-            <v>0</v>
+            <v>7.1429999999999993E-2</v>
           </cell>
           <cell r="W475">
-            <v>0</v>
+            <v>3</v>
           </cell>
         </row>
         <row r="476">
@@ -35321,7 +35489,7 @@
             <v>PUR2600502900001S</v>
           </cell>
           <cell r="E476" t="str">
-            <v/>
+            <v>BDB-000051</v>
           </cell>
           <cell r="F476" t="str">
             <v>PVN-003324</v>
@@ -35339,7 +35507,7 @@
             <v>0</v>
           </cell>
           <cell r="K476">
-            <v>0</v>
+            <v>10</v>
           </cell>
           <cell r="L476" t="str">
             <v>FOOTJOY</v>
@@ -35368,25 +35536,71 @@
           <cell r="T476">
             <v>6</v>
           </cell>
-          <cell r="U476" t="str">
-            <v/>
+          <cell r="U476">
+            <v>7.5</v>
           </cell>
           <cell r="V476">
-            <v>0</v>
+            <v>5.5559999999999998E-2</v>
           </cell>
           <cell r="W476">
-            <v>0</v>
+            <v>1</v>
           </cell>
         </row>
         <row r="477">
+          <cell r="A477" t="str">
+            <v>S-2026-05-101</v>
+          </cell>
+          <cell r="D477" t="str">
+            <v>PUR-202606010001S</v>
+          </cell>
           <cell r="E477" t="str">
             <v/>
           </cell>
+          <cell r="F477" t="str">
+            <v>PVN-004433</v>
+          </cell>
+          <cell r="G477" t="str">
+            <v>OrthoLite X-30-Hybrid BROWN SUGAR/17-1134TPX Hybrid Flat Sheet 0.13D 25+/-4 Asker C 1.1M 2M 15mm</v>
+          </cell>
+          <cell r="H477">
+            <v>10</v>
+          </cell>
+          <cell r="I477">
+            <v>10</v>
+          </cell>
           <cell r="J477">
             <v>0</v>
           </cell>
           <cell r="K477">
             <v>0</v>
+          </cell>
+          <cell r="L477" t="str">
+            <v>ASICS</v>
+          </cell>
+          <cell r="M477" t="str">
+            <v>Sample</v>
+          </cell>
+          <cell r="N477" t="str">
+            <v xml:space="preserve">DIE-CUT
+URGENT </v>
+          </cell>
+          <cell r="O477" t="str">
+            <v>Sample</v>
+          </cell>
+          <cell r="P477">
+            <v>46174</v>
+          </cell>
+          <cell r="Q477">
+            <v>46181</v>
+          </cell>
+          <cell r="R477">
+            <v>46178</v>
+          </cell>
+          <cell r="S477">
+            <v>6</v>
+          </cell>
+          <cell r="T477">
+            <v>7</v>
           </cell>
           <cell r="U477" t="str">
             <v/>
@@ -35399,14 +35613,62 @@
           </cell>
         </row>
         <row r="478">
+          <cell r="A478" t="str">
+            <v>S-2026-05-102</v>
+          </cell>
+          <cell r="C478" t="str">
+            <v>RPRO-260601-0847</v>
+          </cell>
+          <cell r="D478" t="str">
+            <v>PUR-202606010001S</v>
+          </cell>
           <cell r="E478" t="str">
             <v/>
           </cell>
+          <cell r="F478" t="str">
+            <v>PVN-003298</v>
+          </cell>
+          <cell r="G478" t="str">
+            <v>OrthoLite Ultra-Hybrid SEEDPEARL/12-0703TPX Hybrid 0.085D 25+/-4 Asker C 1.1M 2M 4mm</v>
+          </cell>
+          <cell r="H478">
+            <v>100</v>
+          </cell>
+          <cell r="I478">
+            <v>100</v>
+          </cell>
           <cell r="J478">
             <v>0</v>
           </cell>
           <cell r="K478">
             <v>0</v>
+          </cell>
+          <cell r="L478" t="str">
+            <v>SALOMON</v>
+          </cell>
+          <cell r="M478" t="str">
+            <v>Sample</v>
+          </cell>
+          <cell r="N478" t="str">
+            <v>FL SHEET</v>
+          </cell>
+          <cell r="O478" t="str">
+            <v>Sample</v>
+          </cell>
+          <cell r="P478">
+            <v>46174</v>
+          </cell>
+          <cell r="Q478">
+            <v>46181</v>
+          </cell>
+          <cell r="R478">
+            <v>46178</v>
+          </cell>
+          <cell r="S478">
+            <v>6</v>
+          </cell>
+          <cell r="T478">
+            <v>7</v>
           </cell>
           <cell r="U478" t="str">
             <v/>
@@ -35419,14 +35681,62 @@
           </cell>
         </row>
         <row r="479">
+          <cell r="A479" t="str">
+            <v>S-2026-05-103</v>
+          </cell>
+          <cell r="C479" t="str">
+            <v>RPRO-260601-0848</v>
+          </cell>
+          <cell r="D479" t="str">
+            <v>PUR-202606010001S</v>
+          </cell>
           <cell r="E479" t="str">
             <v/>
           </cell>
+          <cell r="F479" t="str">
+            <v>PVN-002973</v>
+          </cell>
+          <cell r="G479" t="str">
+            <v>UltraLite-Hybrid OrthoLite SEEDPEARL/12-0703TPX Hybrid Flat Sheet 0.085D 25+/-4 Asker C 1.1M 2M 4.5mm</v>
+          </cell>
+          <cell r="H479">
+            <v>30</v>
+          </cell>
+          <cell r="I479">
+            <v>30</v>
+          </cell>
           <cell r="J479">
             <v>0</v>
           </cell>
           <cell r="K479">
             <v>0</v>
+          </cell>
+          <cell r="L479" t="str">
+            <v>SALOMON</v>
+          </cell>
+          <cell r="M479" t="str">
+            <v>Sample</v>
+          </cell>
+          <cell r="N479" t="str">
+            <v>MOLDED</v>
+          </cell>
+          <cell r="O479" t="str">
+            <v>Sample</v>
+          </cell>
+          <cell r="P479">
+            <v>46174</v>
+          </cell>
+          <cell r="Q479">
+            <v>46181</v>
+          </cell>
+          <cell r="R479">
+            <v>46178</v>
+          </cell>
+          <cell r="S479">
+            <v>6</v>
+          </cell>
+          <cell r="T479">
+            <v>7</v>
           </cell>
           <cell r="U479" t="str">
             <v/>
@@ -35439,14 +35749,62 @@
           </cell>
         </row>
         <row r="480">
+          <cell r="A480" t="str">
+            <v>S-2026-05-104</v>
+          </cell>
+          <cell r="C480" t="str">
+            <v>RPRO-260601-0849</v>
+          </cell>
+          <cell r="D480" t="str">
+            <v>PUR-202606010001S</v>
+          </cell>
           <cell r="E480" t="str">
             <v/>
           </cell>
+          <cell r="F480" t="str">
+            <v>PVN-002465</v>
+          </cell>
+          <cell r="G480" t="str">
+            <v>OrthoLite Regular-Hybrid SEEDPEARL/12-0703TPX Hybrid Flat Sheet 0.11D 25+/-4 Asker C 1.1M 2M 5mm</v>
+          </cell>
+          <cell r="H480">
+            <v>50</v>
+          </cell>
+          <cell r="I480">
+            <v>50</v>
+          </cell>
           <cell r="J480">
             <v>0</v>
           </cell>
           <cell r="K480">
             <v>0</v>
+          </cell>
+          <cell r="L480" t="str">
+            <v>ASICS</v>
+          </cell>
+          <cell r="M480" t="str">
+            <v>Sample</v>
+          </cell>
+          <cell r="N480" t="str">
+            <v>DIE-CUT</v>
+          </cell>
+          <cell r="O480" t="str">
+            <v>Sample</v>
+          </cell>
+          <cell r="P480">
+            <v>46174</v>
+          </cell>
+          <cell r="Q480">
+            <v>46181</v>
+          </cell>
+          <cell r="R480">
+            <v>46178</v>
+          </cell>
+          <cell r="S480">
+            <v>6</v>
+          </cell>
+          <cell r="T480">
+            <v>7</v>
           </cell>
           <cell r="U480" t="str">
             <v/>
@@ -35459,14 +35817,62 @@
           </cell>
         </row>
         <row r="481">
+          <cell r="A481" t="str">
+            <v>S-2026-05-105</v>
+          </cell>
+          <cell r="C481" t="str">
+            <v>RPRO-260601-0850</v>
+          </cell>
+          <cell r="D481" t="str">
+            <v xml:space="preserve">PUR-202606010001S </v>
+          </cell>
           <cell r="E481" t="str">
             <v/>
           </cell>
+          <cell r="F481" t="str">
+            <v>PVN-003630</v>
+          </cell>
+          <cell r="G481" t="str">
+            <v>OrthoLite Ultra GREEN/16-5932TPX Flat Sheet 0.085D 25+/-4 Asker C 1.1M 2M 2mm</v>
+          </cell>
+          <cell r="H481">
+            <v>30</v>
+          </cell>
+          <cell r="I481">
+            <v>30</v>
+          </cell>
           <cell r="J481">
             <v>0</v>
           </cell>
           <cell r="K481">
             <v>0</v>
+          </cell>
+          <cell r="L481" t="str">
+            <v>UNDER ARMOUR</v>
+          </cell>
+          <cell r="M481" t="str">
+            <v>SSO-2606-00021    - URGENT (6-8)</v>
+          </cell>
+          <cell r="N481" t="str">
+            <v>Flat sheet</v>
+          </cell>
+          <cell r="O481" t="str">
+            <v>Sample</v>
+          </cell>
+          <cell r="P481">
+            <v>46174</v>
+          </cell>
+          <cell r="Q481">
+            <v>46181</v>
+          </cell>
+          <cell r="R481">
+            <v>46178</v>
+          </cell>
+          <cell r="S481">
+            <v>6</v>
+          </cell>
+          <cell r="T481">
+            <v>7</v>
           </cell>
           <cell r="U481" t="str">
             <v/>
@@ -35479,14 +35885,62 @@
           </cell>
         </row>
         <row r="482">
+          <cell r="A482" t="str">
+            <v>S-2026-05-106</v>
+          </cell>
+          <cell r="C482" t="str">
+            <v>RPRO-260601-0851</v>
+          </cell>
+          <cell r="D482" t="str">
+            <v xml:space="preserve">PUR-202606010001S </v>
+          </cell>
           <cell r="E482" t="str">
             <v/>
           </cell>
+          <cell r="F482" t="str">
+            <v>PVN-003236</v>
+          </cell>
+          <cell r="G482" t="str">
+            <v>OrthoLite Eco LT-Hybrid-Converse SEEDPEARL/12-0703TPX Hybrid Flat Sheet 0.13D 25+/-4 Asker C 1.1M 2M 5mm</v>
+          </cell>
+          <cell r="H482">
+            <v>50</v>
+          </cell>
+          <cell r="I482">
+            <v>50</v>
+          </cell>
           <cell r="J482">
             <v>0</v>
           </cell>
           <cell r="K482">
             <v>0</v>
+          </cell>
+          <cell r="L482" t="str">
+            <v>CONVERSE</v>
+          </cell>
+          <cell r="M482" t="str">
+            <v>Sample</v>
+          </cell>
+          <cell r="N482" t="str">
+            <v>Die cut</v>
+          </cell>
+          <cell r="O482" t="str">
+            <v>Sample</v>
+          </cell>
+          <cell r="P482">
+            <v>46174</v>
+          </cell>
+          <cell r="Q482">
+            <v>46181</v>
+          </cell>
+          <cell r="R482">
+            <v>46178</v>
+          </cell>
+          <cell r="S482">
+            <v>6</v>
+          </cell>
+          <cell r="T482">
+            <v>7</v>
           </cell>
           <cell r="U482" t="str">
             <v/>
@@ -35831,24 +36285,24 @@
       <sheetData sheetId="87" refreshError="1"/>
       <sheetData sheetId="88" refreshError="1"/>
       <sheetData sheetId="89" refreshError="1"/>
-      <sheetData sheetId="90" refreshError="1"/>
+      <sheetData sheetId="90"/>
       <sheetData sheetId="91" refreshError="1"/>
       <sheetData sheetId="92" refreshError="1"/>
       <sheetData sheetId="93" refreshError="1"/>
       <sheetData sheetId="94" refreshError="1"/>
       <sheetData sheetId="95" refreshError="1"/>
       <sheetData sheetId="96" refreshError="1"/>
-      <sheetData sheetId="97"/>
-      <sheetData sheetId="98" refreshError="1"/>
-      <sheetData sheetId="99" refreshError="1"/>
-      <sheetData sheetId="100" refreshError="1"/>
+      <sheetData sheetId="97" refreshError="1"/>
+      <sheetData sheetId="98"/>
+      <sheetData sheetId="99"/>
+      <sheetData sheetId="100"/>
       <sheetData sheetId="101" refreshError="1"/>
       <sheetData sheetId="102" refreshError="1"/>
-      <sheetData sheetId="103"/>
-      <sheetData sheetId="104"/>
+      <sheetData sheetId="103" refreshError="1"/>
+      <sheetData sheetId="104" refreshError="1"/>
       <sheetData sheetId="105" refreshError="1"/>
-      <sheetData sheetId="106" refreshError="1"/>
-      <sheetData sheetId="107" refreshError="1"/>
+      <sheetData sheetId="106"/>
+      <sheetData sheetId="107"/>
       <sheetData sheetId="108" refreshError="1"/>
       <sheetData sheetId="109" refreshError="1"/>
       <sheetData sheetId="110" refreshError="1"/>
@@ -36018,6 +36472,9 @@
       <sheetData sheetId="274" refreshError="1"/>
       <sheetData sheetId="275" refreshError="1"/>
       <sheetData sheetId="276" refreshError="1"/>
+      <sheetData sheetId="277" refreshError="1"/>
+      <sheetData sheetId="278" refreshError="1"/>
+      <sheetData sheetId="279" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -37644,23 +38101,23 @@
     <mergeCell ref="D1:F1"/>
   </mergeCells>
   <conditionalFormatting sqref="A2">
-    <cfRule type="duplicateValues" dxfId="63" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="70" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:A20">
-    <cfRule type="duplicateValues" dxfId="62" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="69" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A23:A1048576">
-    <cfRule type="duplicateValues" dxfId="61" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="68" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="60" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="59" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="67" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="66" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:M2">
-    <cfRule type="duplicateValues" dxfId="58" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="65" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1">
-    <cfRule type="duplicateValues" dxfId="57" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="64" priority="5"/>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.18" right="0.17" top="0.5" bottom="0" header="0.17" footer="0.17"/>
@@ -37705,7 +38162,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46172.903662268516</v>
+        <v>46174.661814930558</v>
       </c>
       <c r="D1" s="80" t="s">
         <v>1</v>
@@ -39054,23 +39511,23 @@
     <mergeCell ref="D1:F1"/>
   </mergeCells>
   <conditionalFormatting sqref="A2">
-    <cfRule type="duplicateValues" dxfId="56" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="63" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:A23">
-    <cfRule type="duplicateValues" dxfId="55" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="62" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A26:A1048576">
-    <cfRule type="duplicateValues" dxfId="54" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="61" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="53" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="52" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="60" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="59" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:M2">
-    <cfRule type="duplicateValues" dxfId="51" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="58" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1">
-    <cfRule type="duplicateValues" dxfId="50" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="57" priority="3"/>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.18" right="0.17" top="0.5" bottom="0" header="0.17" footer="0.17"/>
@@ -39115,7 +39572,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46172.903662268516</v>
+        <v>46174.661814930558</v>
       </c>
       <c r="D1" s="80" t="s">
         <v>1</v>
@@ -40522,23 +40979,23 @@
     <mergeCell ref="D1:F1"/>
   </mergeCells>
   <conditionalFormatting sqref="A2">
-    <cfRule type="duplicateValues" dxfId="49" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="56" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:A28">
-    <cfRule type="duplicateValues" dxfId="48" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="55" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A31:A1048576">
-    <cfRule type="duplicateValues" dxfId="47" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="54" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="46" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="45" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="53" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="52" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:M2">
-    <cfRule type="duplicateValues" dxfId="44" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="51" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1">
-    <cfRule type="duplicateValues" dxfId="43" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="50" priority="3"/>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.18" right="0.17" top="0.5" bottom="0" header="0.17" footer="0.17"/>
@@ -40583,7 +41040,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46172.903662268516</v>
+        <v>46174.661814930558</v>
       </c>
       <c r="D1" s="80" t="s">
         <v>1</v>
@@ -41956,23 +42413,23 @@
     <mergeCell ref="D1:F1"/>
   </mergeCells>
   <conditionalFormatting sqref="A2">
-    <cfRule type="duplicateValues" dxfId="42" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="49" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:A25">
-    <cfRule type="duplicateValues" dxfId="41" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="48" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A28:A1048576">
-    <cfRule type="duplicateValues" dxfId="40" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="47" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="39" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="38" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="46" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="45" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:M2">
-    <cfRule type="duplicateValues" dxfId="37" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="44" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1">
-    <cfRule type="duplicateValues" dxfId="36" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="43" priority="3"/>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.18" right="0.17" top="0.5" bottom="0" header="0.17" footer="0.17"/>
@@ -42016,7 +42473,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46172.903662268516</v>
+        <v>46174.661814930558</v>
       </c>
       <c r="D1" s="80" t="s">
         <v>1</v>
@@ -43231,39 +43688,39 @@
     <mergeCell ref="D7:F7"/>
   </mergeCells>
   <conditionalFormatting sqref="A2">
-    <cfRule type="duplicateValues" dxfId="35" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:A6 A14:A18">
-    <cfRule type="duplicateValues" dxfId="34" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A8">
-    <cfRule type="duplicateValues" dxfId="33" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A9:A13">
-    <cfRule type="duplicateValues" dxfId="32" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="39" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A21:A1048576">
-    <cfRule type="duplicateValues" dxfId="31" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C6 C14:C1048576">
-    <cfRule type="duplicateValues" dxfId="30" priority="7"/>
-    <cfRule type="duplicateValues" dxfId="29" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C7:C13">
-    <cfRule type="duplicateValues" dxfId="28" priority="2"/>
-    <cfRule type="duplicateValues" dxfId="27" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I8:L8">
-    <cfRule type="duplicateValues" dxfId="26" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:M2">
-    <cfRule type="duplicateValues" dxfId="25" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="M7">
-    <cfRule type="duplicateValues" dxfId="24" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1">
-    <cfRule type="duplicateValues" dxfId="23" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="9"/>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.18" right="0.17" top="0.5" bottom="0" header="0.17" footer="0.17"/>
@@ -43308,7 +43765,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46172.903662268516</v>
+        <v>46174.661814930558</v>
       </c>
       <c r="D1" s="80" t="s">
         <v>1</v>
@@ -44633,26 +45090,26 @@
     <mergeCell ref="D1:F1"/>
   </mergeCells>
   <conditionalFormatting sqref="A2">
-    <cfRule type="duplicateValues" dxfId="22" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:A15">
-    <cfRule type="duplicateValues" dxfId="21" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A16:A21">
-    <cfRule type="duplicateValues" dxfId="20" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A24:A1048576">
-    <cfRule type="duplicateValues" dxfId="19" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="18" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="17" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:M2">
-    <cfRule type="duplicateValues" dxfId="16" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1">
-    <cfRule type="duplicateValues" dxfId="15" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="3"/>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.18" right="0.17" top="0.5" bottom="0" header="0.17" footer="0.17"/>
@@ -44698,7 +45155,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46172.903662268516</v>
+        <v>46174.661814930558</v>
       </c>
       <c r="D1" s="80" t="s">
         <v>1</v>
@@ -46053,23 +46510,23 @@
     <mergeCell ref="D1:F1"/>
   </mergeCells>
   <conditionalFormatting sqref="A2">
-    <cfRule type="duplicateValues" dxfId="14" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:A21">
-    <cfRule type="duplicateValues" dxfId="13" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A24:A1048576">
-    <cfRule type="duplicateValues" dxfId="12" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="11" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="10" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:M2">
-    <cfRule type="duplicateValues" dxfId="9" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1">
-    <cfRule type="duplicateValues" dxfId="8" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="3"/>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.18" right="0.17" top="0.5" bottom="0" header="0.17" footer="0.17"/>
@@ -46114,7 +46571,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46172.903662268516</v>
+        <v>46174.661814930558</v>
       </c>
       <c r="D1" s="80" t="s">
         <v>1</v>
@@ -47515,24 +47972,24 @@
     <mergeCell ref="D1:F1"/>
   </mergeCells>
   <conditionalFormatting sqref="A2">
-    <cfRule type="duplicateValues" dxfId="7" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:A24">
-    <cfRule type="duplicateValues" dxfId="6" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A27:A1048576">
-    <cfRule type="duplicateValues" dxfId="5" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="4" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="2"/>
-    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:M2">
-    <cfRule type="duplicateValues" dxfId="1" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1">
-    <cfRule type="duplicateValues" dxfId="0" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="4"/>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.18" right="0.17" top="0.5" bottom="0" header="0.17" footer="0.17"/>
@@ -47544,4 +48001,1403 @@
     <brk id="25" max="15" man="1"/>
   </rowBreaks>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E0C7FDD-C476-4FE6-B890-05884597F111}">
+  <sheetPr filterMode="1">
+    <tabColor theme="4"/>
+  </sheetPr>
+  <dimension ref="A1:N664"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="74.25" customHeight="1" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="30.26953125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="41.453125" style="52" customWidth="1"/>
+    <col min="3" max="3" width="26.81640625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="28.81640625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="175.54296875" style="53" customWidth="1"/>
+    <col min="6" max="6" width="19.1796875" style="54" customWidth="1"/>
+    <col min="7" max="7" width="19" style="54" customWidth="1"/>
+    <col min="8" max="8" width="17.1796875" style="55" customWidth="1"/>
+    <col min="9" max="9" width="20.1796875" style="53" customWidth="1"/>
+    <col min="10" max="10" width="20.1796875" style="53" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="33.54296875" style="53" customWidth="1"/>
+    <col min="12" max="12" width="21.453125" style="61" customWidth="1"/>
+    <col min="13" max="13" width="22" style="57" customWidth="1"/>
+    <col min="14" max="14" width="28.1796875" style="58" customWidth="1"/>
+    <col min="15" max="15" width="22.26953125" style="2" bestFit="1" customWidth="1"/>
+    <col min="16" max="16384" width="9.1796875" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" ht="128.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <f ca="1">NOW()</f>
+        <v>46174.661814930558</v>
+      </c>
+      <c r="D1" s="80" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="80"/>
+      <c r="F1" s="80"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="5"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="7"/>
+      <c r="L1" s="8">
+        <f>SUBTOTAL(9,L2:L1048576)</f>
+        <v>9</v>
+      </c>
+      <c r="M1" s="7"/>
+      <c r="N1" s="9"/>
+    </row>
+    <row r="2" spans="1:14" s="16" customFormat="1" ht="132.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="I2" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="J2" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="K2" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="L2" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="M2" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="N2" s="15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="17" t="s">
+        <v>355</v>
+      </c>
+      <c r="B3" s="18" t="s">
+        <v>356</v>
+      </c>
+      <c r="C3" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="D3" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="E3" s="21" t="s">
+        <v>72</v>
+      </c>
+      <c r="F3" s="22">
+        <v>100</v>
+      </c>
+      <c r="G3" s="23">
+        <v>3</v>
+      </c>
+      <c r="H3" s="24">
+        <v>3</v>
+      </c>
+      <c r="I3" s="25" t="s">
+        <v>73</v>
+      </c>
+      <c r="J3" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="K3" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="L3" s="26">
+        <v>4</v>
+      </c>
+      <c r="M3" s="27"/>
+      <c r="N3" s="28">
+        <v>46178</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="17" t="s">
+        <v>357</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>358</v>
+      </c>
+      <c r="C4" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="D4" s="20" t="s">
+        <v>359</v>
+      </c>
+      <c r="E4" s="21" t="s">
+        <v>360</v>
+      </c>
+      <c r="F4" s="22">
+        <v>30</v>
+      </c>
+      <c r="G4" s="23">
+        <v>1</v>
+      </c>
+      <c r="H4" s="24">
+        <v>1</v>
+      </c>
+      <c r="I4" s="25" t="s">
+        <v>73</v>
+      </c>
+      <c r="J4" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="K4" s="25" t="s">
+        <v>28</v>
+      </c>
+      <c r="L4" s="26"/>
+      <c r="M4" s="27"/>
+      <c r="N4" s="28">
+        <v>46178</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="62"/>
+      <c r="B5" s="63"/>
+      <c r="C5" s="64"/>
+      <c r="D5" s="65"/>
+      <c r="E5" s="66"/>
+      <c r="F5" s="67"/>
+      <c r="G5" s="68"/>
+      <c r="H5" s="69"/>
+      <c r="I5" s="70"/>
+      <c r="J5" s="70"/>
+      <c r="K5" s="70"/>
+      <c r="L5" s="71"/>
+      <c r="M5" s="72"/>
+      <c r="N5" s="28"/>
+    </row>
+    <row r="6" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="17" t="s">
+        <v>361</v>
+      </c>
+      <c r="B6" s="18" t="s">
+        <v>362</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="D6" s="20" t="s">
+        <v>363</v>
+      </c>
+      <c r="E6" s="21" t="s">
+        <v>364</v>
+      </c>
+      <c r="F6" s="22">
+        <v>50</v>
+      </c>
+      <c r="G6" s="23">
+        <v>2</v>
+      </c>
+      <c r="H6" s="24">
+        <v>2</v>
+      </c>
+      <c r="I6" s="25" t="s">
+        <v>77</v>
+      </c>
+      <c r="J6" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="K6" s="25" t="s">
+        <v>78</v>
+      </c>
+      <c r="L6" s="26">
+        <v>2</v>
+      </c>
+      <c r="M6" s="40"/>
+      <c r="N6" s="28">
+        <v>46178</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="62"/>
+      <c r="B7" s="63"/>
+      <c r="C7" s="64"/>
+      <c r="D7" s="65"/>
+      <c r="E7" s="66"/>
+      <c r="F7" s="67"/>
+      <c r="G7" s="68"/>
+      <c r="H7" s="69"/>
+      <c r="I7" s="70"/>
+      <c r="J7" s="70"/>
+      <c r="K7" s="70"/>
+      <c r="L7" s="71"/>
+      <c r="M7" s="73"/>
+      <c r="N7" s="28"/>
+    </row>
+    <row r="8" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="17" t="s">
+        <v>365</v>
+      </c>
+      <c r="B8" s="18" t="s">
+        <v>366</v>
+      </c>
+      <c r="C8" s="19" t="s">
+        <v>105</v>
+      </c>
+      <c r="D8" s="20" t="s">
+        <v>367</v>
+      </c>
+      <c r="E8" s="21" t="s">
+        <v>368</v>
+      </c>
+      <c r="F8" s="22">
+        <v>30</v>
+      </c>
+      <c r="G8" s="23">
+        <v>1</v>
+      </c>
+      <c r="H8" s="24">
+        <v>1</v>
+      </c>
+      <c r="I8" s="25" t="s">
+        <v>369</v>
+      </c>
+      <c r="J8" s="25" t="s">
+        <v>370</v>
+      </c>
+      <c r="K8" s="25" t="s">
+        <v>67</v>
+      </c>
+      <c r="L8" s="26">
+        <v>1</v>
+      </c>
+      <c r="M8" s="27"/>
+      <c r="N8" s="28">
+        <v>46178</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="62"/>
+      <c r="B9" s="63"/>
+      <c r="C9" s="64"/>
+      <c r="D9" s="65"/>
+      <c r="E9" s="66"/>
+      <c r="F9" s="67"/>
+      <c r="G9" s="68"/>
+      <c r="H9" s="69"/>
+      <c r="I9" s="70"/>
+      <c r="J9" s="70"/>
+      <c r="K9" s="70"/>
+      <c r="L9" s="71"/>
+      <c r="M9" s="72"/>
+      <c r="N9" s="28"/>
+    </row>
+    <row r="10" spans="1:14" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="17" t="s">
+        <v>371</v>
+      </c>
+      <c r="B10" s="18" t="s">
+        <v>372</v>
+      </c>
+      <c r="C10" s="19" t="s">
+        <v>373</v>
+      </c>
+      <c r="D10" s="20" t="s">
+        <v>374</v>
+      </c>
+      <c r="E10" s="21" t="s">
+        <v>375</v>
+      </c>
+      <c r="F10" s="22">
+        <v>50</v>
+      </c>
+      <c r="G10" s="23">
+        <v>2</v>
+      </c>
+      <c r="H10" s="24">
+        <v>2</v>
+      </c>
+      <c r="I10" s="25" t="s">
+        <v>376</v>
+      </c>
+      <c r="J10" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="K10" s="25" t="s">
+        <v>377</v>
+      </c>
+      <c r="L10" s="26">
+        <v>2</v>
+      </c>
+      <c r="M10" s="27"/>
+      <c r="N10" s="28">
+        <v>46178</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="17"/>
+      <c r="B11" s="18" t="e">
+        <f>VLOOKUP(A11,'[2]master plan'!A:C,3,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C11" s="19" t="e">
+        <f>VLOOKUP($A11,'[2]master plan'!$A:$N,5,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D11" s="20" t="e">
+        <f>VLOOKUP($A11,'[2]master plan'!$A:$N,6,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E11" s="21" t="e">
+        <f>VLOOKUP(A11,'[2]master plan'!A:G,7,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F11" s="22" t="e">
+        <f>VLOOKUP(A11,'[2]master plan'!A:H,8,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="G11" s="23" t="e">
+        <f>VLOOKUP(A11,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H11" s="24" t="e">
+        <f>VLOOKUP(A11,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="I11" s="25" t="e">
+        <f>VLOOKUP($A11,'[2]master plan'!$A:$N,12,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="J11" s="25" t="e">
+        <f>VLOOKUP($A11,'[2]master plan'!$A:$N,13,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="K11" s="25" t="e">
+        <f>VLOOKUP($A11,'[2]master plan'!$A:$N,14,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="L11" s="26"/>
+      <c r="M11" s="27"/>
+      <c r="N11" s="28" t="str">
+        <f>_xlfn.IFNA(VLOOKUP(A11,'[2]master plan'!A:R,18,0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="17"/>
+      <c r="B12" s="18" t="e">
+        <f>VLOOKUP(A12,'[2]master plan'!A:C,3,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C12" s="19" t="e">
+        <f>VLOOKUP($A12,'[2]master plan'!$A:$N,5,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D12" s="20" t="e">
+        <f>VLOOKUP($A12,'[2]master plan'!$A:$N,6,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E12" s="21" t="e">
+        <f>VLOOKUP(A12,'[2]master plan'!A:G,7,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F12" s="22" t="e">
+        <f>VLOOKUP(A12,'[2]master plan'!A:H,8,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="G12" s="23" t="e">
+        <f>VLOOKUP(A12,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H12" s="24" t="e">
+        <f>VLOOKUP(A12,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="I12" s="25" t="e">
+        <f>VLOOKUP($A12,'[2]master plan'!$A:$N,12,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="J12" s="25" t="e">
+        <f>VLOOKUP($A12,'[2]master plan'!$A:$N,13,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="K12" s="25" t="e">
+        <f>VLOOKUP($A12,'[2]master plan'!$A:$N,14,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="L12" s="26"/>
+      <c r="M12" s="40"/>
+      <c r="N12" s="28" t="str">
+        <f>_xlfn.IFNA(VLOOKUP(A12,'[2]master plan'!A:R,18,0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="17"/>
+      <c r="B13" s="18" t="e">
+        <f>VLOOKUP(A13,'[2]master plan'!A:C,3,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C13" s="19" t="e">
+        <f>VLOOKUP($A13,'[2]master plan'!$A:$N,5,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D13" s="20" t="e">
+        <f>VLOOKUP($A13,'[2]master plan'!$A:$N,6,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E13" s="21" t="e">
+        <f>VLOOKUP(A13,'[2]master plan'!A:G,7,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F13" s="22" t="e">
+        <f>VLOOKUP(A13,'[2]master plan'!A:H,8,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="G13" s="23" t="e">
+        <f>VLOOKUP(A13,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H13" s="24" t="e">
+        <f>VLOOKUP(A13,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="I13" s="25" t="e">
+        <f>VLOOKUP($A13,'[2]master plan'!$A:$N,12,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="J13" s="25" t="e">
+        <f>VLOOKUP($A13,'[2]master plan'!$A:$N,13,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="K13" s="25" t="e">
+        <f>VLOOKUP($A13,'[2]master plan'!$A:$N,14,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="L13" s="26"/>
+      <c r="M13" s="27"/>
+      <c r="N13" s="28" t="str">
+        <f>_xlfn.IFNA(VLOOKUP(A13,'[2]master plan'!A:R,18,0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="17"/>
+      <c r="B14" s="18" t="e">
+        <f>VLOOKUP(A14,'[2]master plan'!A:C,3,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C14" s="19" t="e">
+        <f>VLOOKUP($A14,'[2]master plan'!$A:$N,5,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D14" s="20" t="e">
+        <f>VLOOKUP($A14,'[2]master plan'!$A:$N,6,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E14" s="21" t="e">
+        <f>VLOOKUP(A14,'[2]master plan'!A:G,7,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F14" s="22" t="e">
+        <f>VLOOKUP(A14,'[2]master plan'!A:H,8,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="G14" s="23" t="e">
+        <f>VLOOKUP(A14,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H14" s="24" t="e">
+        <f>VLOOKUP(A14,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="I14" s="25" t="e">
+        <f>VLOOKUP($A14,'[2]master plan'!$A:$N,12,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="J14" s="25" t="e">
+        <f>VLOOKUP($A14,'[2]master plan'!$A:$N,13,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="K14" s="25" t="e">
+        <f>VLOOKUP($A14,'[2]master plan'!$A:$N,14,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="L14" s="26"/>
+      <c r="M14" s="27"/>
+      <c r="N14" s="28" t="str">
+        <f>_xlfn.IFNA(VLOOKUP(A14,'[2]master plan'!A:R,18,0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="17"/>
+      <c r="B15" s="18" t="e">
+        <f>VLOOKUP(A15,'[2]master plan'!A:C,3,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C15" s="19" t="e">
+        <f>VLOOKUP($A15,'[2]master plan'!$A:$N,5,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D15" s="20" t="e">
+        <f>VLOOKUP($A15,'[2]master plan'!$A:$N,6,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E15" s="21" t="e">
+        <f>VLOOKUP(A15,'[2]master plan'!A:G,7,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F15" s="22" t="e">
+        <f>VLOOKUP(A15,'[2]master plan'!A:H,8,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="G15" s="23" t="e">
+        <f>VLOOKUP(A15,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H15" s="24" t="e">
+        <f>VLOOKUP(A15,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="I15" s="25" t="e">
+        <f>VLOOKUP($A15,'[2]master plan'!$A:$N,12,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="J15" s="25" t="e">
+        <f>VLOOKUP($A15,'[2]master plan'!$A:$N,13,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="K15" s="25" t="e">
+        <f>VLOOKUP($A15,'[2]master plan'!$A:$N,14,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="L15" s="26"/>
+      <c r="M15" s="40"/>
+      <c r="N15" s="28" t="str">
+        <f>_xlfn.IFNA(VLOOKUP(A15,'[2]master plan'!A:R,18,0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="17"/>
+      <c r="B16" s="18" t="e">
+        <f>VLOOKUP(A16,'[2]master plan'!A:C,3,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C16" s="19" t="e">
+        <f>VLOOKUP($A16,'[2]master plan'!$A:$N,5,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D16" s="20" t="e">
+        <f>VLOOKUP($A16,'[2]master plan'!$A:$N,6,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E16" s="21" t="e">
+        <f>VLOOKUP(A16,'[2]master plan'!A:G,7,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F16" s="22" t="e">
+        <f>VLOOKUP(A16,'[2]master plan'!A:H,8,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="G16" s="23" t="e">
+        <f>VLOOKUP(A16,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H16" s="24" t="e">
+        <f>VLOOKUP(A16,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="I16" s="25" t="e">
+        <f>VLOOKUP($A16,'[2]master plan'!$A:$N,12,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="J16" s="25" t="e">
+        <f>VLOOKUP($A16,'[2]master plan'!$A:$N,13,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="K16" s="25" t="e">
+        <f>VLOOKUP($A16,'[2]master plan'!$A:$N,14,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="L16" s="26"/>
+      <c r="M16" s="40"/>
+      <c r="N16" s="28" t="str">
+        <f>_xlfn.IFNA(VLOOKUP(A16,'[2]master plan'!A:R,18,0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="17"/>
+      <c r="B17" s="18" t="e">
+        <f>VLOOKUP(A17,'[2]master plan'!A:C,3,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C17" s="19" t="e">
+        <f>VLOOKUP($A17,'[2]master plan'!$A:$N,5,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D17" s="20" t="e">
+        <f>VLOOKUP($A17,'[2]master plan'!$A:$N,6,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E17" s="21" t="e">
+        <f>VLOOKUP(A17,'[2]master plan'!A:G,7,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F17" s="22" t="e">
+        <f>VLOOKUP(A17,'[2]master plan'!A:H,8,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="G17" s="23" t="e">
+        <f>VLOOKUP(A17,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H17" s="24" t="e">
+        <f>VLOOKUP(A17,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="I17" s="25" t="e">
+        <f>VLOOKUP($A17,'[2]master plan'!$A:$N,12,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="J17" s="25" t="e">
+        <f>VLOOKUP($A17,'[2]master plan'!$A:$N,13,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="K17" s="25" t="e">
+        <f>VLOOKUP($A17,'[2]master plan'!$A:$N,14,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="L17" s="26"/>
+      <c r="M17" s="27"/>
+      <c r="N17" s="28" t="str">
+        <f>_xlfn.IFNA(VLOOKUP(A17,'[2]master plan'!A:R,18,0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="17"/>
+      <c r="B18" s="18" t="e">
+        <f>VLOOKUP(A18,'[2]master plan'!A:C,3,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C18" s="19" t="e">
+        <f>VLOOKUP($A18,'[2]master plan'!$A:$N,5,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D18" s="20" t="e">
+        <f>VLOOKUP($A18,'[2]master plan'!$A:$N,6,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E18" s="21" t="e">
+        <f>VLOOKUP(A18,'[2]master plan'!A:G,7,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F18" s="22" t="e">
+        <f>VLOOKUP(A18,'[2]master plan'!A:H,8,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="G18" s="23" t="e">
+        <f>VLOOKUP(A18,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H18" s="24" t="e">
+        <f>VLOOKUP(A18,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="I18" s="25" t="e">
+        <f>VLOOKUP($A18,'[2]master plan'!$A:$N,12,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="J18" s="25" t="e">
+        <f>VLOOKUP($A18,'[2]master plan'!$A:$N,13,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="K18" s="25" t="e">
+        <f>VLOOKUP($A18,'[2]master plan'!$A:$N,14,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="L18" s="26"/>
+      <c r="M18" s="40"/>
+      <c r="N18" s="28" t="str">
+        <f>_xlfn.IFNA(VLOOKUP(A18,'[2]master plan'!A:R,18,0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="17"/>
+      <c r="B19" s="18" t="e">
+        <f>VLOOKUP(A19,'[2]master plan'!A:C,3,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C19" s="19" t="e">
+        <f>VLOOKUP($A19,'[2]master plan'!$A:$N,5,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D19" s="20" t="e">
+        <f>VLOOKUP($A19,'[2]master plan'!$A:$N,6,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E19" s="21" t="e">
+        <f>VLOOKUP(A19,'[2]master plan'!A:G,7,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F19" s="22" t="e">
+        <f>VLOOKUP(A19,'[2]master plan'!A:H,8,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="G19" s="23" t="e">
+        <f>VLOOKUP(A19,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H19" s="24" t="e">
+        <f>VLOOKUP(A19,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="I19" s="25" t="e">
+        <f>VLOOKUP($A19,'[2]master plan'!$A:$N,12,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="J19" s="25" t="e">
+        <f>VLOOKUP($A19,'[2]master plan'!$A:$N,13,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="K19" s="25" t="e">
+        <f>VLOOKUP($A19,'[2]master plan'!$A:$N,14,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="L19" s="26"/>
+      <c r="M19" s="40"/>
+      <c r="N19" s="28" t="str">
+        <f>_xlfn.IFNA(VLOOKUP(A19,'[2]master plan'!A:R,18,0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" spans="1:14" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="17"/>
+      <c r="B20" s="18" t="e">
+        <f>VLOOKUP(A20,'[2]master plan'!A:C,3,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C20" s="19" t="e">
+        <f>VLOOKUP($A20,'[2]master plan'!$A:$N,5,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D20" s="20" t="e">
+        <f>VLOOKUP($A20,'[2]master plan'!$A:$N,6,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E20" s="21" t="e">
+        <f>VLOOKUP(A20,'[2]master plan'!A:G,7,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F20" s="22" t="e">
+        <f>VLOOKUP(A20,'[2]master plan'!A:H,8,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="G20" s="23" t="e">
+        <f>VLOOKUP(A20,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H20" s="24" t="e">
+        <f>VLOOKUP(A20,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="I20" s="25" t="e">
+        <f>VLOOKUP($A20,'[2]master plan'!$A:$N,12,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="J20" s="25" t="e">
+        <f>VLOOKUP($A20,'[2]master plan'!$A:$N,13,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="K20" s="25" t="e">
+        <f>VLOOKUP($A20,'[2]master plan'!$A:$N,14,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="L20" s="26"/>
+      <c r="M20" s="40"/>
+      <c r="N20" s="28" t="str">
+        <f>_xlfn.IFNA(VLOOKUP(A20,'[2]master plan'!A:R,18,0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" spans="1:14" s="3" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="41"/>
+      <c r="B21" s="42"/>
+      <c r="C21" s="43"/>
+      <c r="D21" s="43"/>
+      <c r="E21" s="44"/>
+      <c r="F21" s="45"/>
+      <c r="G21" s="45"/>
+      <c r="H21" s="45"/>
+      <c r="I21" s="46"/>
+      <c r="J21" s="47"/>
+      <c r="K21" s="48"/>
+      <c r="L21" s="49"/>
+      <c r="M21" s="50"/>
+      <c r="N21" s="51"/>
+    </row>
+    <row r="22" spans="1:14" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="L22" s="56"/>
+    </row>
+    <row r="23" spans="1:14" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="L23" s="56"/>
+    </row>
+    <row r="24" spans="1:14" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="L24" s="56"/>
+    </row>
+    <row r="25" spans="1:14" s="54" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="2"/>
+      <c r="B25" s="52"/>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
+      <c r="E25" s="59" t="s">
+        <v>21</v>
+      </c>
+      <c r="G25" s="55"/>
+      <c r="I25" s="53"/>
+      <c r="J25" s="53"/>
+      <c r="K25" s="53"/>
+      <c r="L25" s="56"/>
+      <c r="M25" s="57"/>
+      <c r="N25" s="58"/>
+    </row>
+    <row r="26" spans="1:14" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="L26" s="56"/>
+    </row>
+    <row r="27" spans="1:14" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="L27" s="56"/>
+    </row>
+    <row r="28" spans="1:14" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="2"/>
+      <c r="B28" s="52"/>
+      <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
+      <c r="E28" s="53"/>
+      <c r="F28" s="54"/>
+      <c r="G28" s="54"/>
+      <c r="H28" s="55"/>
+      <c r="I28" s="53"/>
+      <c r="J28" s="53"/>
+      <c r="K28" s="53"/>
+      <c r="L28" s="56"/>
+      <c r="M28" s="57"/>
+      <c r="N28" s="58"/>
+    </row>
+    <row r="29" spans="1:14" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="2"/>
+      <c r="B29" s="52"/>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
+      <c r="E29" s="53"/>
+      <c r="F29" s="54"/>
+      <c r="G29" s="54"/>
+      <c r="H29" s="55"/>
+      <c r="I29" s="53"/>
+      <c r="J29" s="53"/>
+      <c r="K29" s="53"/>
+      <c r="L29" s="56"/>
+      <c r="M29" s="57"/>
+      <c r="N29" s="58"/>
+    </row>
+    <row r="30" spans="1:14" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="2"/>
+      <c r="B30" s="52"/>
+      <c r="C30" s="2"/>
+      <c r="D30" s="2"/>
+      <c r="E30" s="53"/>
+      <c r="F30" s="54"/>
+      <c r="G30" s="54"/>
+      <c r="H30" s="55"/>
+      <c r="I30" s="53"/>
+      <c r="J30" s="53"/>
+      <c r="K30" s="53"/>
+      <c r="L30" s="56"/>
+      <c r="M30" s="57"/>
+      <c r="N30" s="58"/>
+    </row>
+    <row r="31" spans="1:14" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="2"/>
+      <c r="B31" s="52"/>
+      <c r="C31" s="2"/>
+      <c r="D31" s="2"/>
+      <c r="E31" s="53"/>
+      <c r="F31" s="54"/>
+      <c r="G31" s="54"/>
+      <c r="H31" s="55"/>
+      <c r="I31" s="53"/>
+      <c r="J31" s="53"/>
+      <c r="K31" s="53"/>
+      <c r="L31" s="56"/>
+      <c r="M31" s="57"/>
+      <c r="N31" s="58"/>
+    </row>
+    <row r="32" spans="1:14" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="2"/>
+      <c r="B32" s="52"/>
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
+      <c r="E32" s="53"/>
+      <c r="F32" s="54"/>
+      <c r="G32" s="54"/>
+      <c r="H32" s="55"/>
+      <c r="I32" s="53"/>
+      <c r="J32" s="53"/>
+      <c r="K32" s="53"/>
+      <c r="L32" s="56"/>
+      <c r="M32" s="57"/>
+      <c r="N32" s="58"/>
+    </row>
+    <row r="33" spans="1:14" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="2"/>
+      <c r="B33" s="52"/>
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
+      <c r="E33" s="53"/>
+      <c r="F33" s="54"/>
+      <c r="G33" s="54"/>
+      <c r="H33" s="55"/>
+      <c r="I33" s="53"/>
+      <c r="J33" s="53"/>
+      <c r="K33" s="53"/>
+      <c r="L33" s="56"/>
+      <c r="M33" s="57"/>
+      <c r="N33" s="58"/>
+    </row>
+    <row r="34" spans="1:14" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="2"/>
+      <c r="B34" s="52"/>
+      <c r="C34" s="2"/>
+      <c r="D34" s="2"/>
+      <c r="E34" s="53"/>
+      <c r="F34" s="54"/>
+      <c r="G34" s="54"/>
+      <c r="H34" s="55"/>
+      <c r="I34" s="53"/>
+      <c r="J34" s="53"/>
+      <c r="K34" s="53"/>
+      <c r="L34" s="56"/>
+      <c r="M34" s="57"/>
+      <c r="N34" s="58"/>
+    </row>
+    <row r="35" spans="1:14" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="2"/>
+      <c r="B35" s="52"/>
+      <c r="C35" s="2"/>
+      <c r="D35" s="2"/>
+      <c r="E35" s="53"/>
+      <c r="F35" s="54"/>
+      <c r="G35" s="54"/>
+      <c r="H35" s="55"/>
+      <c r="I35" s="53"/>
+      <c r="J35" s="53"/>
+      <c r="K35" s="53"/>
+      <c r="L35" s="56"/>
+      <c r="M35" s="57"/>
+      <c r="N35" s="58"/>
+    </row>
+    <row r="36" spans="1:14" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="2"/>
+      <c r="B36" s="52"/>
+      <c r="C36" s="2"/>
+      <c r="D36" s="2"/>
+      <c r="E36" s="53"/>
+      <c r="F36" s="54"/>
+      <c r="G36" s="54"/>
+      <c r="H36" s="55"/>
+      <c r="I36" s="53"/>
+      <c r="J36" s="53"/>
+      <c r="K36" s="53"/>
+      <c r="L36" s="56"/>
+      <c r="M36" s="57"/>
+      <c r="N36" s="58"/>
+    </row>
+    <row r="37" spans="1:14" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="2"/>
+      <c r="B37" s="52"/>
+      <c r="C37" s="2"/>
+      <c r="D37" s="2"/>
+      <c r="E37" s="53"/>
+      <c r="F37" s="54"/>
+      <c r="G37" s="54"/>
+      <c r="H37" s="55"/>
+      <c r="I37" s="53"/>
+      <c r="J37" s="53"/>
+      <c r="K37" s="53"/>
+      <c r="L37" s="56"/>
+      <c r="M37" s="57"/>
+      <c r="N37" s="58"/>
+    </row>
+    <row r="38" spans="1:14" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="2"/>
+      <c r="B38" s="52"/>
+      <c r="C38" s="2"/>
+      <c r="D38" s="2"/>
+      <c r="E38" s="53"/>
+      <c r="F38" s="54"/>
+      <c r="G38" s="54"/>
+      <c r="H38" s="55"/>
+      <c r="I38" s="53"/>
+      <c r="J38" s="53"/>
+      <c r="K38" s="53"/>
+      <c r="L38" s="56"/>
+      <c r="M38" s="57"/>
+      <c r="N38" s="58"/>
+    </row>
+    <row r="39" spans="1:14" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="2"/>
+      <c r="B39" s="52"/>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
+      <c r="E39" s="53"/>
+      <c r="F39" s="54"/>
+      <c r="G39" s="54"/>
+      <c r="H39" s="55"/>
+      <c r="I39" s="53"/>
+      <c r="J39" s="53"/>
+      <c r="K39" s="53"/>
+      <c r="L39" s="56"/>
+      <c r="M39" s="57"/>
+      <c r="N39" s="58"/>
+    </row>
+    <row r="40" spans="1:14" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A40" s="2"/>
+      <c r="B40" s="52"/>
+      <c r="C40" s="2"/>
+      <c r="D40" s="2"/>
+      <c r="E40" s="53"/>
+      <c r="F40" s="54"/>
+      <c r="G40" s="54"/>
+      <c r="H40" s="55"/>
+      <c r="I40" s="53"/>
+      <c r="J40" s="53"/>
+      <c r="K40" s="53"/>
+      <c r="L40" s="56"/>
+      <c r="M40" s="57"/>
+      <c r="N40" s="58"/>
+    </row>
+    <row r="41" spans="1:14" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A41" s="2"/>
+      <c r="B41" s="52"/>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
+      <c r="E41" s="53"/>
+      <c r="F41" s="54"/>
+      <c r="G41" s="54"/>
+      <c r="H41" s="55"/>
+      <c r="I41" s="53"/>
+      <c r="J41" s="53"/>
+      <c r="K41" s="53"/>
+      <c r="L41" s="56"/>
+      <c r="M41" s="57"/>
+      <c r="N41" s="58"/>
+    </row>
+    <row r="42" spans="1:14" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A42" s="2"/>
+      <c r="B42" s="52"/>
+      <c r="C42" s="2"/>
+      <c r="D42" s="2"/>
+      <c r="E42" s="53"/>
+      <c r="F42" s="54"/>
+      <c r="G42" s="54"/>
+      <c r="H42" s="55"/>
+      <c r="I42" s="53"/>
+      <c r="J42" s="53"/>
+      <c r="K42" s="53"/>
+      <c r="L42" s="56"/>
+      <c r="M42" s="57"/>
+      <c r="N42" s="58"/>
+    </row>
+    <row r="43" spans="1:14" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A43" s="2"/>
+      <c r="B43" s="52"/>
+      <c r="C43" s="2"/>
+      <c r="D43" s="2"/>
+      <c r="E43" s="53"/>
+      <c r="F43" s="54"/>
+      <c r="G43" s="54"/>
+      <c r="H43" s="55"/>
+      <c r="I43" s="53"/>
+      <c r="J43" s="53"/>
+      <c r="K43" s="53"/>
+      <c r="L43" s="56"/>
+      <c r="M43" s="57"/>
+      <c r="N43" s="58"/>
+    </row>
+    <row r="44" spans="1:14" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A44" s="2"/>
+      <c r="B44" s="52"/>
+      <c r="C44" s="2"/>
+      <c r="D44" s="2"/>
+      <c r="E44" s="53"/>
+      <c r="F44" s="54"/>
+      <c r="G44" s="54"/>
+      <c r="H44" s="55"/>
+      <c r="I44" s="53"/>
+      <c r="J44" s="53"/>
+      <c r="K44" s="53"/>
+      <c r="L44" s="56"/>
+      <c r="M44" s="57"/>
+      <c r="N44" s="58"/>
+    </row>
+    <row r="45" spans="1:14" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A45" s="2"/>
+      <c r="B45" s="52"/>
+      <c r="C45" s="2"/>
+      <c r="D45" s="2"/>
+      <c r="E45" s="53"/>
+      <c r="F45" s="54"/>
+      <c r="G45" s="54"/>
+      <c r="H45" s="55"/>
+      <c r="I45" s="53"/>
+      <c r="J45" s="53"/>
+      <c r="K45" s="53"/>
+      <c r="L45" s="56"/>
+      <c r="M45" s="57"/>
+      <c r="N45" s="58"/>
+    </row>
+    <row r="46" spans="1:14" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A46" s="2"/>
+      <c r="B46" s="52"/>
+      <c r="C46" s="2"/>
+      <c r="D46" s="2"/>
+      <c r="E46" s="53"/>
+      <c r="F46" s="54"/>
+      <c r="G46" s="54"/>
+      <c r="H46" s="55"/>
+      <c r="I46" s="53"/>
+      <c r="J46" s="53"/>
+      <c r="K46" s="53"/>
+      <c r="L46" s="56"/>
+      <c r="M46" s="57"/>
+      <c r="N46" s="58"/>
+    </row>
+    <row r="47" spans="1:14" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A47" s="2"/>
+      <c r="B47" s="52"/>
+      <c r="C47" s="2"/>
+      <c r="D47" s="2"/>
+      <c r="E47" s="53"/>
+      <c r="F47" s="54"/>
+      <c r="G47" s="54"/>
+      <c r="H47" s="55"/>
+      <c r="I47" s="53"/>
+      <c r="J47" s="53"/>
+      <c r="K47" s="53"/>
+      <c r="L47" s="56"/>
+      <c r="M47" s="57"/>
+      <c r="N47" s="58"/>
+    </row>
+    <row r="48" spans="1:14" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A48" s="2"/>
+      <c r="B48" s="52"/>
+      <c r="C48" s="2"/>
+      <c r="D48" s="2"/>
+      <c r="E48" s="53"/>
+      <c r="F48" s="54"/>
+      <c r="G48" s="54"/>
+      <c r="H48" s="55"/>
+      <c r="I48" s="53"/>
+      <c r="J48" s="53"/>
+      <c r="K48" s="53"/>
+      <c r="L48" s="56"/>
+      <c r="M48" s="57"/>
+      <c r="N48" s="58"/>
+    </row>
+    <row r="49" spans="1:14" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A49" s="2"/>
+      <c r="B49" s="52"/>
+      <c r="C49" s="2"/>
+      <c r="D49" s="2"/>
+      <c r="E49" s="53"/>
+      <c r="F49" s="54"/>
+      <c r="G49" s="54"/>
+      <c r="H49" s="55"/>
+      <c r="I49" s="53"/>
+      <c r="J49" s="53"/>
+      <c r="K49" s="53"/>
+      <c r="L49" s="56"/>
+      <c r="M49" s="57"/>
+      <c r="N49" s="58"/>
+    </row>
+    <row r="50" spans="1:14" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A50" s="2"/>
+      <c r="B50" s="52"/>
+      <c r="C50" s="2"/>
+      <c r="D50" s="2"/>
+      <c r="E50" s="53"/>
+      <c r="F50" s="54"/>
+      <c r="G50" s="54"/>
+      <c r="H50" s="55"/>
+      <c r="I50" s="53"/>
+      <c r="J50" s="53"/>
+      <c r="K50" s="53"/>
+      <c r="L50" s="56"/>
+      <c r="M50" s="57"/>
+      <c r="N50" s="58"/>
+    </row>
+    <row r="51" spans="1:14" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A51" s="2"/>
+      <c r="B51" s="52"/>
+      <c r="C51" s="2"/>
+      <c r="D51" s="2"/>
+      <c r="E51" s="53"/>
+      <c r="F51" s="54"/>
+      <c r="G51" s="54"/>
+      <c r="H51" s="55"/>
+      <c r="I51" s="53"/>
+      <c r="J51" s="53"/>
+      <c r="K51" s="53"/>
+      <c r="L51" s="56"/>
+      <c r="M51" s="57"/>
+      <c r="N51" s="58"/>
+    </row>
+    <row r="52" spans="1:14" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A52" s="2"/>
+      <c r="B52" s="52"/>
+      <c r="C52" s="2"/>
+      <c r="D52" s="2"/>
+      <c r="E52" s="53"/>
+      <c r="F52" s="54"/>
+      <c r="G52" s="54"/>
+      <c r="H52" s="55"/>
+      <c r="I52" s="53"/>
+      <c r="J52" s="53"/>
+      <c r="K52" s="53"/>
+      <c r="L52" s="56"/>
+      <c r="M52" s="57"/>
+      <c r="N52" s="58"/>
+    </row>
+    <row r="53" spans="1:14" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A53" s="2"/>
+      <c r="B53" s="52"/>
+      <c r="C53" s="2"/>
+      <c r="D53" s="2"/>
+      <c r="E53" s="53"/>
+      <c r="F53" s="54"/>
+      <c r="G53" s="54"/>
+      <c r="H53" s="55"/>
+      <c r="I53" s="53"/>
+      <c r="J53" s="53"/>
+      <c r="K53" s="53"/>
+      <c r="L53" s="56"/>
+      <c r="M53" s="57"/>
+      <c r="N53" s="58"/>
+    </row>
+    <row r="54" spans="1:14" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A54" s="2"/>
+      <c r="B54" s="52"/>
+      <c r="C54" s="2"/>
+      <c r="D54" s="2"/>
+      <c r="E54" s="53"/>
+      <c r="F54" s="54"/>
+      <c r="G54" s="54"/>
+      <c r="H54" s="55"/>
+      <c r="I54" s="53"/>
+      <c r="J54" s="53"/>
+      <c r="K54" s="53"/>
+      <c r="L54" s="56"/>
+      <c r="M54" s="57"/>
+      <c r="N54" s="58"/>
+    </row>
+    <row r="55" spans="1:14" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A55" s="2"/>
+      <c r="B55" s="52"/>
+      <c r="C55" s="2"/>
+      <c r="D55" s="2"/>
+      <c r="E55" s="53"/>
+      <c r="F55" s="54"/>
+      <c r="G55" s="54"/>
+      <c r="H55" s="55"/>
+      <c r="I55" s="53"/>
+      <c r="J55" s="53"/>
+      <c r="K55" s="53"/>
+      <c r="L55" s="56"/>
+      <c r="M55" s="57"/>
+      <c r="N55" s="58"/>
+    </row>
+    <row r="664" spans="1:14" s="54" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A664" s="2"/>
+      <c r="B664" s="52"/>
+      <c r="C664" s="2"/>
+      <c r="D664" s="2"/>
+      <c r="E664" s="60"/>
+      <c r="H664" s="55"/>
+      <c r="I664" s="53"/>
+      <c r="J664" s="53"/>
+      <c r="K664" s="53"/>
+      <c r="L664" s="61"/>
+      <c r="M664" s="57"/>
+      <c r="N664" s="58"/>
+    </row>
+  </sheetData>
+  <protectedRanges>
+    <protectedRange algorithmName="SHA-512" hashValue="e1FOu1UlwA7reaiyQlEGzbU6dAFPyHPlKfgo6VzFBBobawyOfUsh2c/+wjC8bICpcXVPmRerMGA9+qKsw5p7Iw==" saltValue="UD2tVZrxqZTGI3vDzMBrHw==" spinCount="100000" sqref="E3:E20" name="Range1_1"/>
+  </protectedRanges>
+  <autoFilter ref="A2:N21" xr:uid="{E2BC4C4A-3703-4A99-A30B-53817C3A378F}">
+    <filterColumn colId="1">
+      <filters blank="1">
+        <filter val="RPRO-260601-0847"/>
+        <filter val="RPRO-260601-0848"/>
+        <filter val="RPRO-260601-0849"/>
+        <filter val="RPRO-260601-0850"/>
+        <filter val="RPRO-260601-0851"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
+  <mergeCells count="1">
+    <mergeCell ref="D1:F1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A2">
+    <cfRule type="duplicateValues" dxfId="6" priority="5"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A3:A20">
+    <cfRule type="duplicateValues" dxfId="5" priority="7"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A23:A1048576">
+    <cfRule type="duplicateValues" dxfId="4" priority="6"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C1:C1048576">
+    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I2:M2">
+    <cfRule type="duplicateValues" dxfId="1" priority="4"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N1">
+    <cfRule type="duplicateValues" dxfId="0" priority="3"/>
+  </conditionalFormatting>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.18" right="0.17" top="0.5" bottom="0" header="0.17" footer="0.17"/>
+  <pageSetup paperSize="9" scale="30" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <headerFooter>
+    <oddFooter>Page &amp;P of &amp;N</oddFooter>
+  </headerFooter>
+  <rowBreaks count="1" manualBreakCount="1">
+    <brk id="21" max="15" man="1"/>
+  </rowBreaks>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update Kế hoach sản xuất Sample.xlsx - June 2nd data
</commit_message>
<xml_diff>
--- a/Kế hoach sản xuất Sample.xlsx
+++ b/Kế hoach sản xuất Sample.xlsx
@@ -39596,7 +39596,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46176.399045833336</v>
+        <v>46176.520486574074</v>
       </c>
       <c r="D1" s="80" t="s">
         <v>1</v>
@@ -41038,7 +41038,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46176.399045833336</v>
+        <v>46176.520486574074</v>
       </c>
       <c r="D1" s="80" t="s">
         <v>1</v>
@@ -42448,7 +42448,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46176.399045833336</v>
+        <v>46176.520486574074</v>
       </c>
       <c r="D1" s="80" t="s">
         <v>1</v>
@@ -43916,7 +43916,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46176.399045833336</v>
+        <v>46176.520486574074</v>
       </c>
       <c r="D1" s="80" t="s">
         <v>1</v>
@@ -45349,7 +45349,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46176.399045833336</v>
+        <v>46176.520486574074</v>
       </c>
       <c r="D1" s="80" t="s">
         <v>1</v>
@@ -46641,7 +46641,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46176.399045833336</v>
+        <v>46176.520486574074</v>
       </c>
       <c r="D1" s="80" t="s">
         <v>1</v>
@@ -48031,7 +48031,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46176.399045833336</v>
+        <v>46176.520486574074</v>
       </c>
       <c r="D1" s="80" t="s">
         <v>1</v>
@@ -49447,7 +49447,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46176.399045833336</v>
+        <v>46176.520486574074</v>
       </c>
       <c r="D1" s="80" t="s">
         <v>1</v>
@@ -50898,7 +50898,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46176.399045833336</v>
+        <v>46176.520486574074</v>
       </c>
       <c r="D1" s="80" t="s">
         <v>1</v>

</xml_diff>

<commit_message>
Update week 24 plan and make sheet lookup robust
</commit_message>
<xml_diff>
--- a/Kế hoach sản xuất Sample.xlsx
+++ b/Kế hoach sản xuất Sample.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ortholitevietnam-my.sharepoint.com/personal/lam_dv2_ortholite_vn/Documents/PROJECT LÂM/DailyFoamingReport/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="104" documentId="8_{C12FF075-160F-4BB4-977C-4D56BABB08BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6D650652-9D11-44C1-8210-99001EF99009}"/>
+  <xr:revisionPtr revIDLastSave="116" documentId="8_{C12FF075-160F-4BB4-977C-4D56BABB08BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{800C6EB4-0DF0-470E-8FE5-3E35347FBA1B}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="2" activeTab="12" xr2:uid="{E780E912-92A1-4ADF-95B1-638FE58CE194}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="3" activeTab="12" xr2:uid="{E780E912-92A1-4ADF-95B1-638FE58CE194}"/>
   </bookViews>
   <sheets>
     <sheet name="13.5" sheetId="1" r:id="rId1"/>
@@ -26,10 +26,11 @@
     <sheet name="3.6" sheetId="11" r:id="rId11"/>
     <sheet name="4.6" sheetId="12" r:id="rId12"/>
     <sheet name="5.6" sheetId="13" r:id="rId13"/>
+    <sheet name="6.6" sheetId="14" r:id="rId14"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId14"/>
     <externalReference r:id="rId15"/>
+    <externalReference r:id="rId16"/>
   </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'1.6'!$A$2:$N$21</definedName>
@@ -45,6 +46,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'3.6'!$A$2:$N$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'4.6'!$A$2:$N$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'5.6'!$A$2:$N$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'6.6'!$A$2:$M$18</definedName>
     <definedName name="AE" localSheetId="8">'[1]Molding-báo cáo BUn'!#REF!</definedName>
     <definedName name="AE" localSheetId="0">'[1]Molding-báo cáo BUn'!#REF!</definedName>
     <definedName name="AE" localSheetId="1">'[1]Molding-báo cáo BUn'!#REF!</definedName>
@@ -58,6 +60,7 @@
     <definedName name="AE" localSheetId="10">'[1]Molding-báo cáo BUn'!#REF!</definedName>
     <definedName name="AE" localSheetId="11">'[1]Molding-báo cáo BUn'!#REF!</definedName>
     <definedName name="AE" localSheetId="12">'[1]Molding-báo cáo BUn'!#REF!</definedName>
+    <definedName name="AE" localSheetId="13">'[1]Molding-báo cáo BUn'!#REF!</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="8">'1.6'!$A$1:$N$21</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'13.5'!$A$1:$N$21</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'15.5'!$A$1:$N$24</definedName>
@@ -71,6 +74,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="10">'3.6'!$A$1:$N$23</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="11">'4.6'!$A$1:$N$22</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="12">'5.6'!$A$1:$N$25</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="13">'6.6'!$A$1:$M$18</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="8">'1.6'!$1:$2</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'13.5'!$1:$2</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'15.5'!$1:$2</definedName>
@@ -84,6 +88,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="10">'3.6'!$1:$2</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="11">'4.6'!$1:$2</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="12">'5.6'!$1:$2</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="13">'6.6'!$1:$2</definedName>
     <definedName name="Z_1811EAD5_BD80_4EFF_9596_8EF0EFF4AD2A_.wvu.FilterData" localSheetId="8" hidden="1">'1.6'!$A$2:$N$2</definedName>
     <definedName name="Z_1811EAD5_BD80_4EFF_9596_8EF0EFF4AD2A_.wvu.FilterData" localSheetId="0" hidden="1">'13.5'!$A$2:$N$2</definedName>
     <definedName name="Z_1811EAD5_BD80_4EFF_9596_8EF0EFF4AD2A_.wvu.FilterData" localSheetId="1" hidden="1">'15.5'!$A$2:$N$2</definedName>
@@ -97,6 +102,7 @@
     <definedName name="Z_1811EAD5_BD80_4EFF_9596_8EF0EFF4AD2A_.wvu.FilterData" localSheetId="10" hidden="1">'3.6'!$A$2:$N$2</definedName>
     <definedName name="Z_1811EAD5_BD80_4EFF_9596_8EF0EFF4AD2A_.wvu.FilterData" localSheetId="11" hidden="1">'4.6'!$A$2:$N$2</definedName>
     <definedName name="Z_1811EAD5_BD80_4EFF_9596_8EF0EFF4AD2A_.wvu.FilterData" localSheetId="12" hidden="1">'5.6'!$A$2:$N$2</definedName>
+    <definedName name="Z_1811EAD5_BD80_4EFF_9596_8EF0EFF4AD2A_.wvu.FilterData" localSheetId="13" hidden="1">'6.6'!$A$2:$M$2</definedName>
     <definedName name="Z_1811EAD5_BD80_4EFF_9596_8EF0EFF4AD2A_.wvu.PrintTitles" localSheetId="8" hidden="1">'1.6'!$1:$2</definedName>
     <definedName name="Z_1811EAD5_BD80_4EFF_9596_8EF0EFF4AD2A_.wvu.PrintTitles" localSheetId="0" hidden="1">'13.5'!$1:$2</definedName>
     <definedName name="Z_1811EAD5_BD80_4EFF_9596_8EF0EFF4AD2A_.wvu.PrintTitles" localSheetId="1" hidden="1">'15.5'!$1:$2</definedName>
@@ -110,6 +116,7 @@
     <definedName name="Z_1811EAD5_BD80_4EFF_9596_8EF0EFF4AD2A_.wvu.PrintTitles" localSheetId="10" hidden="1">'3.6'!$1:$2</definedName>
     <definedName name="Z_1811EAD5_BD80_4EFF_9596_8EF0EFF4AD2A_.wvu.PrintTitles" localSheetId="11" hidden="1">'4.6'!$1:$2</definedName>
     <definedName name="Z_1811EAD5_BD80_4EFF_9596_8EF0EFF4AD2A_.wvu.PrintTitles" localSheetId="12" hidden="1">'5.6'!$1:$2</definedName>
+    <definedName name="Z_1811EAD5_BD80_4EFF_9596_8EF0EFF4AD2A_.wvu.PrintTitles" localSheetId="13" hidden="1">'6.6'!$1:$2</definedName>
     <definedName name="Z_18A7E0A3_1642_489C_8130_3CC9FF80B04E_.wvu.FilterData" localSheetId="8" hidden="1">'1.6'!$B$2:$M$2</definedName>
     <definedName name="Z_18A7E0A3_1642_489C_8130_3CC9FF80B04E_.wvu.FilterData" localSheetId="0" hidden="1">'13.5'!$B$2:$M$2</definedName>
     <definedName name="Z_18A7E0A3_1642_489C_8130_3CC9FF80B04E_.wvu.FilterData" localSheetId="1" hidden="1">'15.5'!$B$2:$M$2</definedName>
@@ -123,6 +130,7 @@
     <definedName name="Z_18A7E0A3_1642_489C_8130_3CC9FF80B04E_.wvu.FilterData" localSheetId="10" hidden="1">'3.6'!$B$2:$M$2</definedName>
     <definedName name="Z_18A7E0A3_1642_489C_8130_3CC9FF80B04E_.wvu.FilterData" localSheetId="11" hidden="1">'4.6'!$B$2:$M$2</definedName>
     <definedName name="Z_18A7E0A3_1642_489C_8130_3CC9FF80B04E_.wvu.FilterData" localSheetId="12" hidden="1">'5.6'!$B$2:$M$2</definedName>
+    <definedName name="Z_18A7E0A3_1642_489C_8130_3CC9FF80B04E_.wvu.FilterData" localSheetId="13" hidden="1">'6.6'!$B$2:$M$2</definedName>
     <definedName name="Z_2653C0F9_59B0_4DB3_BD8D_CACC833527F0_.wvu.FilterData" localSheetId="8" hidden="1">'1.6'!$A$2:$N$2</definedName>
     <definedName name="Z_2653C0F9_59B0_4DB3_BD8D_CACC833527F0_.wvu.FilterData" localSheetId="0" hidden="1">'13.5'!$A$2:$N$2</definedName>
     <definedName name="Z_2653C0F9_59B0_4DB3_BD8D_CACC833527F0_.wvu.FilterData" localSheetId="1" hidden="1">'15.5'!$A$2:$N$2</definedName>
@@ -136,6 +144,7 @@
     <definedName name="Z_2653C0F9_59B0_4DB3_BD8D_CACC833527F0_.wvu.FilterData" localSheetId="10" hidden="1">'3.6'!$A$2:$N$2</definedName>
     <definedName name="Z_2653C0F9_59B0_4DB3_BD8D_CACC833527F0_.wvu.FilterData" localSheetId="11" hidden="1">'4.6'!$A$2:$N$2</definedName>
     <definedName name="Z_2653C0F9_59B0_4DB3_BD8D_CACC833527F0_.wvu.FilterData" localSheetId="12" hidden="1">'5.6'!$A$2:$N$2</definedName>
+    <definedName name="Z_2653C0F9_59B0_4DB3_BD8D_CACC833527F0_.wvu.FilterData" localSheetId="13" hidden="1">'6.6'!$A$2:$M$2</definedName>
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.FilterData" localSheetId="8" hidden="1">'1.6'!$A$2:$N$2</definedName>
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.FilterData" localSheetId="0" hidden="1">'13.5'!$A$2:$N$2</definedName>
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.FilterData" localSheetId="1" hidden="1">'15.5'!$A$2:$N$2</definedName>
@@ -149,6 +158,7 @@
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.FilterData" localSheetId="10" hidden="1">'3.6'!$A$2:$N$2</definedName>
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.FilterData" localSheetId="11" hidden="1">'4.6'!$A$2:$N$2</definedName>
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.FilterData" localSheetId="12" hidden="1">'5.6'!$A$2:$N$2</definedName>
+    <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.FilterData" localSheetId="13" hidden="1">'6.6'!$A$2:$M$2</definedName>
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.PrintTitles" localSheetId="8" hidden="1">'1.6'!$1:$2</definedName>
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.PrintTitles" localSheetId="0" hidden="1">'13.5'!$1:$2</definedName>
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.PrintTitles" localSheetId="1" hidden="1">'15.5'!$1:$2</definedName>
@@ -162,6 +172,7 @@
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.PrintTitles" localSheetId="10" hidden="1">'3.6'!$1:$2</definedName>
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.PrintTitles" localSheetId="11" hidden="1">'4.6'!$1:$2</definedName>
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.PrintTitles" localSheetId="12" hidden="1">'5.6'!$1:$2</definedName>
+    <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.PrintTitles" localSheetId="13" hidden="1">'6.6'!$1:$2</definedName>
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.Rows" localSheetId="8" hidden="1">'1.6'!#REF!</definedName>
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.Rows" localSheetId="0" hidden="1">'13.5'!#REF!</definedName>
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.Rows" localSheetId="1" hidden="1">'15.5'!#REF!</definedName>
@@ -175,6 +186,7 @@
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.Rows" localSheetId="10" hidden="1">'3.6'!#REF!</definedName>
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.Rows" localSheetId="11" hidden="1">'4.6'!#REF!</definedName>
     <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.Rows" localSheetId="12" hidden="1">'5.6'!#REF!</definedName>
+    <definedName name="Z_289C1146_6484_4C42_9E78_5D7EBC42FBCC_.wvu.Rows" localSheetId="13" hidden="1">'6.6'!#REF!</definedName>
     <definedName name="Z_314949E3_0D3B_4560_AE70_4D3C4970782A_.wvu.FilterData" localSheetId="8" hidden="1">'1.6'!$B$2:$M$2</definedName>
     <definedName name="Z_314949E3_0D3B_4560_AE70_4D3C4970782A_.wvu.FilterData" localSheetId="0" hidden="1">'13.5'!$B$2:$M$2</definedName>
     <definedName name="Z_314949E3_0D3B_4560_AE70_4D3C4970782A_.wvu.FilterData" localSheetId="1" hidden="1">'15.5'!$B$2:$M$2</definedName>
@@ -188,6 +200,7 @@
     <definedName name="Z_314949E3_0D3B_4560_AE70_4D3C4970782A_.wvu.FilterData" localSheetId="10" hidden="1">'3.6'!$B$2:$M$2</definedName>
     <definedName name="Z_314949E3_0D3B_4560_AE70_4D3C4970782A_.wvu.FilterData" localSheetId="11" hidden="1">'4.6'!$B$2:$M$2</definedName>
     <definedName name="Z_314949E3_0D3B_4560_AE70_4D3C4970782A_.wvu.FilterData" localSheetId="12" hidden="1">'5.6'!$B$2:$M$2</definedName>
+    <definedName name="Z_314949E3_0D3B_4560_AE70_4D3C4970782A_.wvu.FilterData" localSheetId="13" hidden="1">'6.6'!$B$2:$M$2</definedName>
     <definedName name="Z_318C8B1E_0627_4DC9_8089_60901FDA475B_.wvu.FilterData" localSheetId="8" hidden="1">'1.6'!$B$2:$N$2</definedName>
     <definedName name="Z_318C8B1E_0627_4DC9_8089_60901FDA475B_.wvu.FilterData" localSheetId="0" hidden="1">'13.5'!$B$2:$N$2</definedName>
     <definedName name="Z_318C8B1E_0627_4DC9_8089_60901FDA475B_.wvu.FilterData" localSheetId="1" hidden="1">'15.5'!$B$2:$N$2</definedName>
@@ -201,6 +214,7 @@
     <definedName name="Z_318C8B1E_0627_4DC9_8089_60901FDA475B_.wvu.FilterData" localSheetId="10" hidden="1">'3.6'!$B$2:$N$2</definedName>
     <definedName name="Z_318C8B1E_0627_4DC9_8089_60901FDA475B_.wvu.FilterData" localSheetId="11" hidden="1">'4.6'!$B$2:$N$2</definedName>
     <definedName name="Z_318C8B1E_0627_4DC9_8089_60901FDA475B_.wvu.FilterData" localSheetId="12" hidden="1">'5.6'!$B$2:$N$2</definedName>
+    <definedName name="Z_318C8B1E_0627_4DC9_8089_60901FDA475B_.wvu.FilterData" localSheetId="13" hidden="1">'6.6'!$B$2:$M$2</definedName>
     <definedName name="Z_318C8B1E_0627_4DC9_8089_60901FDA475B_.wvu.PrintTitles" localSheetId="8" hidden="1">'1.6'!$1:$2</definedName>
     <definedName name="Z_318C8B1E_0627_4DC9_8089_60901FDA475B_.wvu.PrintTitles" localSheetId="0" hidden="1">'13.5'!$1:$2</definedName>
     <definedName name="Z_318C8B1E_0627_4DC9_8089_60901FDA475B_.wvu.PrintTitles" localSheetId="1" hidden="1">'15.5'!$1:$2</definedName>
@@ -214,6 +228,7 @@
     <definedName name="Z_318C8B1E_0627_4DC9_8089_60901FDA475B_.wvu.PrintTitles" localSheetId="10" hidden="1">'3.6'!$1:$2</definedName>
     <definedName name="Z_318C8B1E_0627_4DC9_8089_60901FDA475B_.wvu.PrintTitles" localSheetId="11" hidden="1">'4.6'!$1:$2</definedName>
     <definedName name="Z_318C8B1E_0627_4DC9_8089_60901FDA475B_.wvu.PrintTitles" localSheetId="12" hidden="1">'5.6'!$1:$2</definedName>
+    <definedName name="Z_318C8B1E_0627_4DC9_8089_60901FDA475B_.wvu.PrintTitles" localSheetId="13" hidden="1">'6.6'!$1:$2</definedName>
     <definedName name="Z_323B6797_06D8_47A1_B001_797373BE57F2_.wvu.FilterData" localSheetId="8" hidden="1">'1.6'!$B$2:$M$2</definedName>
     <definedName name="Z_323B6797_06D8_47A1_B001_797373BE57F2_.wvu.FilterData" localSheetId="0" hidden="1">'13.5'!$B$2:$M$2</definedName>
     <definedName name="Z_323B6797_06D8_47A1_B001_797373BE57F2_.wvu.FilterData" localSheetId="1" hidden="1">'15.5'!$B$2:$M$2</definedName>
@@ -227,6 +242,7 @@
     <definedName name="Z_323B6797_06D8_47A1_B001_797373BE57F2_.wvu.FilterData" localSheetId="10" hidden="1">'3.6'!$B$2:$M$2</definedName>
     <definedName name="Z_323B6797_06D8_47A1_B001_797373BE57F2_.wvu.FilterData" localSheetId="11" hidden="1">'4.6'!$B$2:$M$2</definedName>
     <definedName name="Z_323B6797_06D8_47A1_B001_797373BE57F2_.wvu.FilterData" localSheetId="12" hidden="1">'5.6'!$B$2:$M$2</definedName>
+    <definedName name="Z_323B6797_06D8_47A1_B001_797373BE57F2_.wvu.FilterData" localSheetId="13" hidden="1">'6.6'!$B$2:$M$2</definedName>
     <definedName name="Z_6A9DC2EA_1959_4EB9_A839_907E58591C36_.wvu.FilterData" localSheetId="8" hidden="1">'1.6'!$B$2:$M$2</definedName>
     <definedName name="Z_6A9DC2EA_1959_4EB9_A839_907E58591C36_.wvu.FilterData" localSheetId="0" hidden="1">'13.5'!$B$2:$M$2</definedName>
     <definedName name="Z_6A9DC2EA_1959_4EB9_A839_907E58591C36_.wvu.FilterData" localSheetId="1" hidden="1">'15.5'!$B$2:$M$2</definedName>
@@ -240,6 +256,7 @@
     <definedName name="Z_6A9DC2EA_1959_4EB9_A839_907E58591C36_.wvu.FilterData" localSheetId="10" hidden="1">'3.6'!$B$2:$M$2</definedName>
     <definedName name="Z_6A9DC2EA_1959_4EB9_A839_907E58591C36_.wvu.FilterData" localSheetId="11" hidden="1">'4.6'!$B$2:$M$2</definedName>
     <definedName name="Z_6A9DC2EA_1959_4EB9_A839_907E58591C36_.wvu.FilterData" localSheetId="12" hidden="1">'5.6'!$B$2:$M$2</definedName>
+    <definedName name="Z_6A9DC2EA_1959_4EB9_A839_907E58591C36_.wvu.FilterData" localSheetId="13" hidden="1">'6.6'!$B$2:$M$2</definedName>
     <definedName name="Z_866BE165_7CE2_41D4_AD4C_D79698D432B1_.wvu.FilterData" localSheetId="8" hidden="1">'1.6'!$B$2:$M$2</definedName>
     <definedName name="Z_866BE165_7CE2_41D4_AD4C_D79698D432B1_.wvu.FilterData" localSheetId="0" hidden="1">'13.5'!$B$2:$M$2</definedName>
     <definedName name="Z_866BE165_7CE2_41D4_AD4C_D79698D432B1_.wvu.FilterData" localSheetId="1" hidden="1">'15.5'!$B$2:$M$2</definedName>
@@ -253,6 +270,7 @@
     <definedName name="Z_866BE165_7CE2_41D4_AD4C_D79698D432B1_.wvu.FilterData" localSheetId="10" hidden="1">'3.6'!$B$2:$M$2</definedName>
     <definedName name="Z_866BE165_7CE2_41D4_AD4C_D79698D432B1_.wvu.FilterData" localSheetId="11" hidden="1">'4.6'!$B$2:$M$2</definedName>
     <definedName name="Z_866BE165_7CE2_41D4_AD4C_D79698D432B1_.wvu.FilterData" localSheetId="12" hidden="1">'5.6'!$B$2:$M$2</definedName>
+    <definedName name="Z_866BE165_7CE2_41D4_AD4C_D79698D432B1_.wvu.FilterData" localSheetId="13" hidden="1">'6.6'!$B$2:$M$2</definedName>
     <definedName name="Z_866CB300_9BE2_4E49_BCB4_72634A7939D7_.wvu.FilterData" localSheetId="8" hidden="1">'1.6'!$B$2:$N$2</definedName>
     <definedName name="Z_866CB300_9BE2_4E49_BCB4_72634A7939D7_.wvu.FilterData" localSheetId="0" hidden="1">'13.5'!$B$2:$N$2</definedName>
     <definedName name="Z_866CB300_9BE2_4E49_BCB4_72634A7939D7_.wvu.FilterData" localSheetId="1" hidden="1">'15.5'!$B$2:$N$2</definedName>
@@ -266,6 +284,7 @@
     <definedName name="Z_866CB300_9BE2_4E49_BCB4_72634A7939D7_.wvu.FilterData" localSheetId="10" hidden="1">'3.6'!$B$2:$N$2</definedName>
     <definedName name="Z_866CB300_9BE2_4E49_BCB4_72634A7939D7_.wvu.FilterData" localSheetId="11" hidden="1">'4.6'!$B$2:$N$2</definedName>
     <definedName name="Z_866CB300_9BE2_4E49_BCB4_72634A7939D7_.wvu.FilterData" localSheetId="12" hidden="1">'5.6'!$B$2:$N$2</definedName>
+    <definedName name="Z_866CB300_9BE2_4E49_BCB4_72634A7939D7_.wvu.FilterData" localSheetId="13" hidden="1">'6.6'!$B$2:$M$2</definedName>
     <definedName name="Z_8CF255E0_B8BB_4016_A366_4FCF106965CF_.wvu.FilterData" localSheetId="8" hidden="1">'1.6'!$A$2:$N$2</definedName>
     <definedName name="Z_8CF255E0_B8BB_4016_A366_4FCF106965CF_.wvu.FilterData" localSheetId="0" hidden="1">'13.5'!$A$2:$N$2</definedName>
     <definedName name="Z_8CF255E0_B8BB_4016_A366_4FCF106965CF_.wvu.FilterData" localSheetId="1" hidden="1">'15.5'!$A$2:$N$2</definedName>
@@ -279,6 +298,7 @@
     <definedName name="Z_8CF255E0_B8BB_4016_A366_4FCF106965CF_.wvu.FilterData" localSheetId="10" hidden="1">'3.6'!$A$2:$N$2</definedName>
     <definedName name="Z_8CF255E0_B8BB_4016_A366_4FCF106965CF_.wvu.FilterData" localSheetId="11" hidden="1">'4.6'!$A$2:$N$2</definedName>
     <definedName name="Z_8CF255E0_B8BB_4016_A366_4FCF106965CF_.wvu.FilterData" localSheetId="12" hidden="1">'5.6'!$A$2:$N$2</definedName>
+    <definedName name="Z_8CF255E0_B8BB_4016_A366_4FCF106965CF_.wvu.FilterData" localSheetId="13" hidden="1">'6.6'!$A$2:$M$2</definedName>
     <definedName name="Z_A4A1FC39_A54C_43AC_9912_8824EB6833F5_.wvu.FilterData" localSheetId="8" hidden="1">'1.6'!$A$2:$N$2</definedName>
     <definedName name="Z_A4A1FC39_A54C_43AC_9912_8824EB6833F5_.wvu.FilterData" localSheetId="0" hidden="1">'13.5'!$A$2:$N$2</definedName>
     <definedName name="Z_A4A1FC39_A54C_43AC_9912_8824EB6833F5_.wvu.FilterData" localSheetId="1" hidden="1">'15.5'!$A$2:$N$2</definedName>
@@ -292,6 +312,7 @@
     <definedName name="Z_A4A1FC39_A54C_43AC_9912_8824EB6833F5_.wvu.FilterData" localSheetId="10" hidden="1">'3.6'!$A$2:$N$2</definedName>
     <definedName name="Z_A4A1FC39_A54C_43AC_9912_8824EB6833F5_.wvu.FilterData" localSheetId="11" hidden="1">'4.6'!$A$2:$N$2</definedName>
     <definedName name="Z_A4A1FC39_A54C_43AC_9912_8824EB6833F5_.wvu.FilterData" localSheetId="12" hidden="1">'5.6'!$A$2:$N$2</definedName>
+    <definedName name="Z_A4A1FC39_A54C_43AC_9912_8824EB6833F5_.wvu.FilterData" localSheetId="13" hidden="1">'6.6'!$A$2:$M$2</definedName>
     <definedName name="Z_AF6B2EAC_2950_4809_A605_2107D254FC8D_.wvu.FilterData" localSheetId="8" hidden="1">'1.6'!$B$2:$N$2</definedName>
     <definedName name="Z_AF6B2EAC_2950_4809_A605_2107D254FC8D_.wvu.FilterData" localSheetId="0" hidden="1">'13.5'!$B$2:$N$2</definedName>
     <definedName name="Z_AF6B2EAC_2950_4809_A605_2107D254FC8D_.wvu.FilterData" localSheetId="1" hidden="1">'15.5'!$B$2:$N$2</definedName>
@@ -305,6 +326,7 @@
     <definedName name="Z_AF6B2EAC_2950_4809_A605_2107D254FC8D_.wvu.FilterData" localSheetId="10" hidden="1">'3.6'!$B$2:$N$2</definedName>
     <definedName name="Z_AF6B2EAC_2950_4809_A605_2107D254FC8D_.wvu.FilterData" localSheetId="11" hidden="1">'4.6'!$B$2:$N$2</definedName>
     <definedName name="Z_AF6B2EAC_2950_4809_A605_2107D254FC8D_.wvu.FilterData" localSheetId="12" hidden="1">'5.6'!$B$2:$N$2</definedName>
+    <definedName name="Z_AF6B2EAC_2950_4809_A605_2107D254FC8D_.wvu.FilterData" localSheetId="13" hidden="1">'6.6'!$B$2:$M$2</definedName>
     <definedName name="Z_AF6B2EAC_2950_4809_A605_2107D254FC8D_.wvu.PrintTitles" localSheetId="8" hidden="1">'1.6'!$1:$2</definedName>
     <definedName name="Z_AF6B2EAC_2950_4809_A605_2107D254FC8D_.wvu.PrintTitles" localSheetId="0" hidden="1">'13.5'!$1:$2</definedName>
     <definedName name="Z_AF6B2EAC_2950_4809_A605_2107D254FC8D_.wvu.PrintTitles" localSheetId="1" hidden="1">'15.5'!$1:$2</definedName>
@@ -318,6 +340,7 @@
     <definedName name="Z_AF6B2EAC_2950_4809_A605_2107D254FC8D_.wvu.PrintTitles" localSheetId="10" hidden="1">'3.6'!$1:$2</definedName>
     <definedName name="Z_AF6B2EAC_2950_4809_A605_2107D254FC8D_.wvu.PrintTitles" localSheetId="11" hidden="1">'4.6'!$1:$2</definedName>
     <definedName name="Z_AF6B2EAC_2950_4809_A605_2107D254FC8D_.wvu.PrintTitles" localSheetId="12" hidden="1">'5.6'!$1:$2</definedName>
+    <definedName name="Z_AF6B2EAC_2950_4809_A605_2107D254FC8D_.wvu.PrintTitles" localSheetId="13" hidden="1">'6.6'!$1:$2</definedName>
     <definedName name="Z_CA92E8A2_92C9_4575_A139_6FE5DA69269F_.wvu.FilterData" localSheetId="8" hidden="1">'1.6'!$B$2:$M$2</definedName>
     <definedName name="Z_CA92E8A2_92C9_4575_A139_6FE5DA69269F_.wvu.FilterData" localSheetId="0" hidden="1">'13.5'!$B$2:$M$2</definedName>
     <definedName name="Z_CA92E8A2_92C9_4575_A139_6FE5DA69269F_.wvu.FilterData" localSheetId="1" hidden="1">'15.5'!$B$2:$M$2</definedName>
@@ -331,6 +354,7 @@
     <definedName name="Z_CA92E8A2_92C9_4575_A139_6FE5DA69269F_.wvu.FilterData" localSheetId="10" hidden="1">'3.6'!$B$2:$M$2</definedName>
     <definedName name="Z_CA92E8A2_92C9_4575_A139_6FE5DA69269F_.wvu.FilterData" localSheetId="11" hidden="1">'4.6'!$B$2:$M$2</definedName>
     <definedName name="Z_CA92E8A2_92C9_4575_A139_6FE5DA69269F_.wvu.FilterData" localSheetId="12" hidden="1">'5.6'!$B$2:$M$2</definedName>
+    <definedName name="Z_CA92E8A2_92C9_4575_A139_6FE5DA69269F_.wvu.FilterData" localSheetId="13" hidden="1">'6.6'!$B$2:$M$2</definedName>
     <definedName name="Z_DF644A2B_B913_48D6_B430_E57F3B482B79_.wvu.FilterData" localSheetId="8" hidden="1">'1.6'!$A$2:$N$2</definedName>
     <definedName name="Z_DF644A2B_B913_48D6_B430_E57F3B482B79_.wvu.FilterData" localSheetId="0" hidden="1">'13.5'!$A$2:$N$2</definedName>
     <definedName name="Z_DF644A2B_B913_48D6_B430_E57F3B482B79_.wvu.FilterData" localSheetId="1" hidden="1">'15.5'!$A$2:$N$2</definedName>
@@ -344,6 +368,7 @@
     <definedName name="Z_DF644A2B_B913_48D6_B430_E57F3B482B79_.wvu.FilterData" localSheetId="10" hidden="1">'3.6'!$A$2:$N$2</definedName>
     <definedName name="Z_DF644A2B_B913_48D6_B430_E57F3B482B79_.wvu.FilterData" localSheetId="11" hidden="1">'4.6'!$A$2:$N$2</definedName>
     <definedName name="Z_DF644A2B_B913_48D6_B430_E57F3B482B79_.wvu.FilterData" localSheetId="12" hidden="1">'5.6'!$A$2:$N$2</definedName>
+    <definedName name="Z_DF644A2B_B913_48D6_B430_E57F3B482B79_.wvu.FilterData" localSheetId="13" hidden="1">'6.6'!$A$2:$M$2</definedName>
     <definedName name="Z_DF644A2B_B913_48D6_B430_E57F3B482B79_.wvu.PrintTitles" localSheetId="8" hidden="1">'1.6'!$1:$2</definedName>
     <definedName name="Z_DF644A2B_B913_48D6_B430_E57F3B482B79_.wvu.PrintTitles" localSheetId="0" hidden="1">'13.5'!$1:$2</definedName>
     <definedName name="Z_DF644A2B_B913_48D6_B430_E57F3B482B79_.wvu.PrintTitles" localSheetId="1" hidden="1">'15.5'!$1:$2</definedName>
@@ -357,6 +382,7 @@
     <definedName name="Z_DF644A2B_B913_48D6_B430_E57F3B482B79_.wvu.PrintTitles" localSheetId="10" hidden="1">'3.6'!$1:$2</definedName>
     <definedName name="Z_DF644A2B_B913_48D6_B430_E57F3B482B79_.wvu.PrintTitles" localSheetId="11" hidden="1">'4.6'!$1:$2</definedName>
     <definedName name="Z_DF644A2B_B913_48D6_B430_E57F3B482B79_.wvu.PrintTitles" localSheetId="12" hidden="1">'5.6'!$1:$2</definedName>
+    <definedName name="Z_DF644A2B_B913_48D6_B430_E57F3B482B79_.wvu.PrintTitles" localSheetId="13" hidden="1">'6.6'!$1:$2</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -379,7 +405,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1073" uniqueCount="512">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1092" uniqueCount="515">
   <si>
     <t>Release Date</t>
   </si>
@@ -1995,6 +2021,15 @@
   <si>
     <t>OrthoLite HybridPlus-Recycled COLORO 063-98-46 (fluorescent) Hybrid 0.12D 25+/-4 Asker C 1.1M 2M 6mm</t>
   </si>
+  <si>
+    <t>S-2026-06-25</t>
+  </si>
+  <si>
+    <t>???</t>
+  </si>
+  <si>
+    <t>????</t>
+  </si>
 </sst>
 </file>
 
@@ -2611,7 +2646,67 @@
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="100">
+  <dxfs count="106">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -3786,12 +3881,14 @@
       <sheetName val="3.6"/>
       <sheetName val="4.6"/>
       <sheetName val="5.6"/>
-      <sheetName val="form 2 (20)"/>
+      <sheetName val="6.6"/>
+      <sheetName val="form 2 (21)"/>
       <sheetName val="In đơn"/>
       <sheetName val="Production BOM"/>
       <sheetName val="Items"/>
       <sheetName val="mm Pu"/>
       <sheetName val="master plan (2)"/>
+      <sheetName val="form 2 (20)"/>
       <sheetName val="form 2 (18)"/>
       <sheetName val="form 2 (19)"/>
       <sheetName val="form 2 (17)"/>
@@ -3837,7 +3934,6 @@
       <sheetName val="22.5"/>
       <sheetName val="30.5"/>
       <sheetName val="3.6 (L)"/>
-      <sheetName val="6.6"/>
       <sheetName val="9.6"/>
       <sheetName val="9.6 (L)"/>
       <sheetName val="10.6"/>
@@ -4017,16 +4113,16 @@
             <v>SAMPLE</v>
           </cell>
           <cell r="H2">
-            <v>24949</v>
+            <v>24969</v>
           </cell>
           <cell r="I2">
-            <v>24949</v>
+            <v>24969</v>
           </cell>
           <cell r="J2">
             <v>23583</v>
           </cell>
           <cell r="K2">
-            <v>1366</v>
+            <v>1386</v>
           </cell>
           <cell r="L2" t="str">
             <v>ASICS</v>
@@ -4048,7 +4144,7 @@
           </cell>
           <cell r="V2"/>
           <cell r="W2">
-            <v>1271</v>
+            <v>1272</v>
           </cell>
         </row>
         <row r="3">
@@ -36614,7 +36710,9 @@
           <cell r="A474" t="str">
             <v>S-2026-05-98</v>
           </cell>
-          <cell r="B474"/>
+          <cell r="B474" t="str">
+            <v xml:space="preserve">Xịn dời ETD </v>
+          </cell>
           <cell r="C474" t="str">
             <v>RPRO-260529-0344</v>
           </cell>
@@ -39210,40 +39308,84 @@
           </cell>
         </row>
         <row r="512">
-          <cell r="A512"/>
-          <cell r="B512"/>
-          <cell r="C512"/>
-          <cell r="D512"/>
-          <cell r="E512"/>
-          <cell r="F512"/>
-          <cell r="G512"/>
-          <cell r="H512"/>
-          <cell r="I512"/>
+          <cell r="A512" t="str">
+            <v>S-2026-06-25</v>
+          </cell>
+          <cell r="B512" t="str">
+            <v>Chưa rl</v>
+          </cell>
+          <cell r="C512" t="str">
+            <v>RPRO-260606-0217</v>
+          </cell>
+          <cell r="D512" t="str">
+            <v xml:space="preserve">PUR2606050003S   </v>
+          </cell>
+          <cell r="E512" t="str">
+            <v>BDB-000067</v>
+          </cell>
+          <cell r="F512" t="str">
+            <v>PVN-003672</v>
+          </cell>
+          <cell r="G512" t="str">
+            <v>OrthoLite Ultra SEEDPEARL/12-0703TPX Flat Sheet 0.085D 25+/-4 Asker C 1.1M 2M 3mm</v>
+          </cell>
+          <cell r="H512">
+            <v>20</v>
+          </cell>
+          <cell r="I512">
+            <v>20</v>
+          </cell>
           <cell r="J512">
             <v>0</v>
           </cell>
           <cell r="K512">
-            <v>0</v>
-          </cell>
-          <cell r="L512"/>
-          <cell r="M512"/>
-          <cell r="N512"/>
-          <cell r="O512"/>
-          <cell r="P512"/>
-          <cell r="Q512"/>
-          <cell r="R512"/>
-          <cell r="S512"/>
-          <cell r="T512"/>
-          <cell r="U512"/>
-          <cell r="V512"/>
-          <cell r="W512"/>
+            <v>20</v>
+          </cell>
+          <cell r="L512" t="str">
+            <v>ADIDAS</v>
+          </cell>
+          <cell r="M512" t="str">
+            <v>SSO-2606-00253  - URGENT (6-13)</v>
+          </cell>
+          <cell r="N512" t="str">
+            <v>Flat sheet</v>
+          </cell>
+          <cell r="O512" t="str">
+            <v>Sample</v>
+          </cell>
+          <cell r="P512">
+            <v>46178</v>
+          </cell>
+          <cell r="Q512">
+            <v>46186</v>
+          </cell>
+          <cell r="R512">
+            <v>46183</v>
+          </cell>
+          <cell r="S512">
+            <v>6</v>
+          </cell>
+          <cell r="T512">
+            <v>8</v>
+          </cell>
+          <cell r="U512">
+            <v>3</v>
+          </cell>
+          <cell r="V512">
+            <v>2.1739999999999999E-2</v>
+          </cell>
+          <cell r="W512">
+            <v>1</v>
+          </cell>
         </row>
         <row r="513">
           <cell r="A513"/>
           <cell r="B513"/>
           <cell r="C513"/>
           <cell r="D513"/>
-          <cell r="E513"/>
+          <cell r="E513" t="str">
+            <v/>
+          </cell>
           <cell r="F513"/>
           <cell r="G513"/>
           <cell r="H513"/>
@@ -39272,7 +39414,9 @@
           <cell r="B514"/>
           <cell r="C514"/>
           <cell r="D514"/>
-          <cell r="E514"/>
+          <cell r="E514" t="str">
+            <v/>
+          </cell>
           <cell r="F514"/>
           <cell r="G514"/>
           <cell r="H514"/>
@@ -39301,7 +39445,9 @@
           <cell r="B515"/>
           <cell r="C515"/>
           <cell r="D515"/>
-          <cell r="E515"/>
+          <cell r="E515" t="str">
+            <v/>
+          </cell>
           <cell r="F515"/>
           <cell r="G515"/>
           <cell r="H515"/>
@@ -39330,7 +39476,9 @@
           <cell r="B516"/>
           <cell r="C516"/>
           <cell r="D516"/>
-          <cell r="E516"/>
+          <cell r="E516" t="str">
+            <v/>
+          </cell>
           <cell r="F516"/>
           <cell r="G516"/>
           <cell r="H516"/>
@@ -39359,7 +39507,9 @@
           <cell r="B517"/>
           <cell r="C517"/>
           <cell r="D517"/>
-          <cell r="E517"/>
+          <cell r="E517" t="str">
+            <v/>
+          </cell>
           <cell r="F517"/>
           <cell r="G517"/>
           <cell r="H517"/>
@@ -39388,7 +39538,9 @@
           <cell r="B518"/>
           <cell r="C518"/>
           <cell r="D518"/>
-          <cell r="E518"/>
+          <cell r="E518" t="str">
+            <v/>
+          </cell>
           <cell r="F518"/>
           <cell r="G518"/>
           <cell r="H518"/>
@@ -39417,7 +39569,9 @@
           <cell r="B519"/>
           <cell r="C519"/>
           <cell r="D519"/>
-          <cell r="E519"/>
+          <cell r="E519" t="str">
+            <v/>
+          </cell>
           <cell r="F519"/>
           <cell r="G519"/>
           <cell r="H519"/>
@@ -39573,18 +39727,18 @@
       <sheetData sheetId="103"/>
       <sheetData sheetId="104"/>
       <sheetData sheetId="105"/>
-      <sheetData sheetId="106">
+      <sheetData sheetId="106"/>
+      <sheetData sheetId="107">
         <row r="1">
           <cell r="F1" t="str">
             <v>No_Item</v>
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="107"/>
       <sheetData sheetId="108"/>
       <sheetData sheetId="109"/>
-      <sheetData sheetId="110" refreshError="1"/>
-      <sheetData sheetId="111" refreshError="1"/>
+      <sheetData sheetId="110"/>
+      <sheetData sheetId="111"/>
       <sheetData sheetId="112" refreshError="1"/>
       <sheetData sheetId="113" refreshError="1"/>
       <sheetData sheetId="114" refreshError="1"/>
@@ -39762,6 +39916,7 @@
       <sheetData sheetId="286" refreshError="1"/>
       <sheetData sheetId="287" refreshError="1"/>
       <sheetData sheetId="288" refreshError="1"/>
+      <sheetData sheetId="289" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -41388,23 +41543,23 @@
     <mergeCell ref="D1:F1"/>
   </mergeCells>
   <conditionalFormatting sqref="A2">
-    <cfRule type="duplicateValues" dxfId="99" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="105" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:A20">
-    <cfRule type="duplicateValues" dxfId="98" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="104" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A23:A1048576">
-    <cfRule type="duplicateValues" dxfId="97" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="103" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="96" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="95" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="102" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="101" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:M2">
-    <cfRule type="duplicateValues" dxfId="94" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="100" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1">
-    <cfRule type="duplicateValues" dxfId="93" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="99" priority="5"/>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.18" right="0.17" top="0.5" bottom="0" header="0.17" footer="0.17"/>
@@ -41450,7 +41605,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46178.924539467589</v>
+        <v>46179.701554050924</v>
       </c>
       <c r="D1" s="83" t="s">
         <v>1</v>
@@ -42831,23 +42986,23 @@
     <mergeCell ref="D1:F1"/>
   </mergeCells>
   <conditionalFormatting sqref="A2">
-    <cfRule type="duplicateValues" dxfId="28" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="34" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:A23">
-    <cfRule type="duplicateValues" dxfId="27" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="33" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A26:A1048576">
-    <cfRule type="duplicateValues" dxfId="26" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="32" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="25" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="24" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="31" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="30" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:M2">
-    <cfRule type="duplicateValues" dxfId="23" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1">
-    <cfRule type="duplicateValues" dxfId="22" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="28" priority="3"/>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.18" right="0.17" top="0.5" bottom="0" header="0.17" footer="0.17"/>
@@ -42893,7 +43048,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46178.924539467589</v>
+        <v>46179.701554050924</v>
       </c>
       <c r="D1" s="83" t="s">
         <v>1</v>
@@ -44274,23 +44429,23 @@
     <mergeCell ref="D1:F1"/>
   </mergeCells>
   <conditionalFormatting sqref="A2">
-    <cfRule type="duplicateValues" dxfId="21" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="27" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:A22">
-    <cfRule type="duplicateValues" dxfId="20" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="26" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A25:A1048576">
-    <cfRule type="duplicateValues" dxfId="19" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="25" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="18" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="17" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="24" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="23" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:M2">
-    <cfRule type="duplicateValues" dxfId="16" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="22" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1">
-    <cfRule type="duplicateValues" dxfId="15" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="3"/>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.18" right="0.17" top="0.5" bottom="0" header="0.17" footer="0.17"/>
@@ -44335,7 +44490,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46178.924539467589</v>
+        <v>46179.701554050924</v>
       </c>
       <c r="D1" s="83" t="s">
         <v>1</v>
@@ -45619,23 +45774,23 @@
     <mergeCell ref="D1:F1"/>
   </mergeCells>
   <conditionalFormatting sqref="A2">
-    <cfRule type="duplicateValues" dxfId="14" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:A21">
-    <cfRule type="duplicateValues" dxfId="13" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="19" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A24:A1048576">
-    <cfRule type="duplicateValues" dxfId="12" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="11" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="10" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:M2">
-    <cfRule type="duplicateValues" dxfId="9" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1">
-    <cfRule type="duplicateValues" dxfId="8" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="3"/>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.18" right="0.17" top="0.5" bottom="0" header="0.17" footer="0.17"/>
@@ -45667,7 +45822,7 @@
     <col min="8" max="8" width="17.1796875" style="55" customWidth="1"/>
     <col min="9" max="10" width="20.1796875" style="53" hidden="1" customWidth="1"/>
     <col min="11" max="11" width="33.54296875" style="53" hidden="1" customWidth="1"/>
-    <col min="12" max="12" width="21.453125" style="61" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="21.453125" style="61" customWidth="1"/>
     <col min="13" max="13" width="22" style="57" hidden="1" customWidth="1"/>
     <col min="14" max="14" width="28.1796875" style="58" customWidth="1"/>
     <col min="15" max="15" width="22.26953125" style="2" bestFit="1" customWidth="1"/>
@@ -45680,7 +45835,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46178.924539467589</v>
+        <v>46179.701554050924</v>
       </c>
       <c r="D1" s="83" t="s">
         <v>1</v>
@@ -45859,8 +46014,8 @@
         <f>_xlfn.IFNA(VLOOKUP(A5,'[2]master plan'!A:R,18,0),"")</f>
         <v>46182</v>
       </c>
-      <c r="O5" s="3" t="s">
-        <v>320</v>
+      <c r="O5" s="58">
+        <v>46240</v>
       </c>
     </row>
     <row r="6" spans="1:15" s="3" customFormat="1" ht="71.25" customHeight="1" x14ac:dyDescent="0.35">
@@ -46093,6 +46248,9 @@
         <f>_xlfn.IFNA(VLOOKUP(A11,'[2]master plan'!A:R,18,0),"")</f>
         <v>46182</v>
       </c>
+      <c r="O11" s="58">
+        <v>46240</v>
+      </c>
     </row>
     <row r="12" spans="1:15" s="3" customFormat="1" ht="71.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="62"/>
@@ -46224,6 +46382,9 @@
         <f>_xlfn.IFNA(VLOOKUP(A15,'[2]master plan'!A:R,18,0),"")</f>
         <v>46182</v>
       </c>
+      <c r="O15" s="3" t="s">
+        <v>513</v>
+      </c>
     </row>
     <row r="16" spans="1:15" s="3" customFormat="1" ht="71.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="62"/>
@@ -46287,6 +46448,9 @@
       <c r="N17" s="28">
         <f>_xlfn.IFNA(VLOOKUP(A17,'[2]master plan'!A:R,18,0),"")</f>
         <v>46182</v>
+      </c>
+      <c r="O17" s="3" t="s">
+        <v>514</v>
       </c>
     </row>
     <row r="18" spans="1:15" s="3" customFormat="1" ht="71.25" customHeight="1" x14ac:dyDescent="0.35">
@@ -47134,26 +47298,26 @@
     <mergeCell ref="D1:F1"/>
   </mergeCells>
   <conditionalFormatting sqref="A2">
-    <cfRule type="duplicateValues" dxfId="7" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:A24">
-    <cfRule type="duplicateValues" dxfId="6" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A27:A1048576">
-    <cfRule type="duplicateValues" dxfId="5" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="4" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D3:D19">
-    <cfRule type="duplicateValues" dxfId="2" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:M2">
-    <cfRule type="duplicateValues" dxfId="1" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1">
-    <cfRule type="duplicateValues" dxfId="0" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="3"/>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.18" right="0.17" top="0.5" bottom="0" header="0.17" footer="0.17"/>
@@ -47163,6 +47327,1296 @@
   </headerFooter>
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="25" max="15" man="1"/>
+  </rowBreaks>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D9B619B-ADEB-444B-B0C4-D546C9681600}">
+  <sheetPr filterMode="1">
+    <tabColor theme="4"/>
+  </sheetPr>
+  <dimension ref="A1:M661"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="74.25" customHeight="1" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="30.26953125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="41.453125" style="52" customWidth="1"/>
+    <col min="3" max="3" width="26.81640625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="28.81640625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="175.54296875" style="53" customWidth="1"/>
+    <col min="6" max="6" width="19.1796875" style="54" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="19" style="54" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="17.1796875" style="55" customWidth="1"/>
+    <col min="9" max="10" width="20.1796875" style="53" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="33.54296875" style="53" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="21.453125" style="61" customWidth="1"/>
+    <col min="13" max="13" width="22" style="57" customWidth="1"/>
+    <col min="14" max="14" width="22.26953125" style="2" bestFit="1" customWidth="1"/>
+    <col min="15" max="16384" width="9.1796875" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" ht="128.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <f ca="1">NOW()</f>
+        <v>46179.701553935185</v>
+      </c>
+      <c r="D1" s="83" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="83"/>
+      <c r="F1" s="83"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="5"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="7"/>
+      <c r="L1" s="8">
+        <f>SUBTOTAL(9,L2:L1048576)</f>
+        <v>1</v>
+      </c>
+      <c r="M1" s="7"/>
+    </row>
+    <row r="2" spans="1:13" s="16" customFormat="1" ht="132.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="I2" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="J2" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="K2" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="L2" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="M2" s="11" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" s="3" customFormat="1" ht="70" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="17" t="s">
+        <v>512</v>
+      </c>
+      <c r="B3" s="18" t="str">
+        <f>VLOOKUP(A3,'[2]master plan'!A:C,3,0)</f>
+        <v>RPRO-260606-0217</v>
+      </c>
+      <c r="C3" s="19" t="str">
+        <f>VLOOKUP($A3,'[2]master plan'!$A:$N,5,0)</f>
+        <v>BDB-000067</v>
+      </c>
+      <c r="D3" s="20" t="str">
+        <f>VLOOKUP($A3,'[2]master plan'!$A:$N,6,0)</f>
+        <v>PVN-003672</v>
+      </c>
+      <c r="E3" s="21" t="str">
+        <f>VLOOKUP(A3,'[2]master plan'!A:G,7,0)</f>
+        <v>OrthoLite Ultra SEEDPEARL/12-0703TPX Flat Sheet 0.085D 25+/-4 Asker C 1.1M 2M 3mm</v>
+      </c>
+      <c r="F3" s="22">
+        <f>VLOOKUP(A3,'[2]master plan'!A:H,8,0)</f>
+        <v>20</v>
+      </c>
+      <c r="G3" s="23">
+        <f>VLOOKUP(A3,'[2]master plan'!A:W,23,0)</f>
+        <v>1</v>
+      </c>
+      <c r="H3" s="24">
+        <f>VLOOKUP(A3,'[2]master plan'!A:W,23,0)</f>
+        <v>1</v>
+      </c>
+      <c r="I3" s="25" t="str">
+        <f>VLOOKUP($A3,'[2]master plan'!$A:$N,12,0)</f>
+        <v>ADIDAS</v>
+      </c>
+      <c r="J3" s="25" t="str">
+        <f>VLOOKUP($A3,'[2]master plan'!$A:$N,13,0)</f>
+        <v>SSO-2606-00253  - URGENT (6-13)</v>
+      </c>
+      <c r="K3" s="25" t="str">
+        <f>VLOOKUP($A3,'[2]master plan'!$A:$N,14,0)</f>
+        <v>Flat sheet</v>
+      </c>
+      <c r="L3" s="26">
+        <v>1</v>
+      </c>
+      <c r="M3" s="27" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="17"/>
+      <c r="B4" s="18" t="e">
+        <f>VLOOKUP(A4,'[2]master plan'!A:C,3,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C4" s="19" t="e">
+        <f>VLOOKUP($A4,'[2]master plan'!$A:$N,5,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D4" s="20" t="e">
+        <f>VLOOKUP($A4,'[2]master plan'!$A:$N,6,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E4" s="21" t="e">
+        <f>VLOOKUP(A4,'[2]master plan'!A:G,7,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F4" s="22" t="e">
+        <f>VLOOKUP(A4,'[2]master plan'!A:H,8,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="G4" s="23" t="e">
+        <f>VLOOKUP(A4,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H4" s="24" t="e">
+        <f>VLOOKUP(A4,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="I4" s="25" t="e">
+        <f>VLOOKUP($A4,'[2]master plan'!$A:$N,12,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="J4" s="25" t="e">
+        <f>VLOOKUP($A4,'[2]master plan'!$A:$N,13,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="K4" s="25" t="e">
+        <f>VLOOKUP($A4,'[2]master plan'!$A:$N,14,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="L4" s="26"/>
+      <c r="M4" s="27"/>
+    </row>
+    <row r="5" spans="1:13" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="17"/>
+      <c r="B5" s="18" t="e">
+        <f>VLOOKUP(A5,'[2]master plan'!A:C,3,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C5" s="19" t="e">
+        <f>VLOOKUP($A5,'[2]master plan'!$A:$N,5,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D5" s="20" t="e">
+        <f>VLOOKUP($A5,'[2]master plan'!$A:$N,6,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E5" s="21" t="e">
+        <f>VLOOKUP(A5,'[2]master plan'!A:G,7,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F5" s="22" t="e">
+        <f>VLOOKUP(A5,'[2]master plan'!A:H,8,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="G5" s="23" t="e">
+        <f>VLOOKUP(A5,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H5" s="24" t="e">
+        <f>VLOOKUP(A5,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="I5" s="25" t="e">
+        <f>VLOOKUP($A5,'[2]master plan'!$A:$N,12,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="J5" s="25" t="e">
+        <f>VLOOKUP($A5,'[2]master plan'!$A:$N,13,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="K5" s="25" t="e">
+        <f>VLOOKUP($A5,'[2]master plan'!$A:$N,14,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="L5" s="26"/>
+      <c r="M5" s="40"/>
+    </row>
+    <row r="6" spans="1:13" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="17"/>
+      <c r="B6" s="18" t="e">
+        <f>VLOOKUP(A6,'[2]master plan'!A:C,3,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C6" s="19" t="e">
+        <f>VLOOKUP($A6,'[2]master plan'!$A:$N,5,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D6" s="20" t="e">
+        <f>VLOOKUP($A6,'[2]master plan'!$A:$N,6,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E6" s="21" t="e">
+        <f>VLOOKUP(A6,'[2]master plan'!A:G,7,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F6" s="22" t="e">
+        <f>VLOOKUP(A6,'[2]master plan'!A:H,8,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="G6" s="23" t="e">
+        <f>VLOOKUP(A6,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H6" s="24" t="e">
+        <f>VLOOKUP(A6,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="I6" s="25" t="e">
+        <f>VLOOKUP($A6,'[2]master plan'!$A:$N,12,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="J6" s="25" t="e">
+        <f>VLOOKUP($A6,'[2]master plan'!$A:$N,13,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="K6" s="25" t="e">
+        <f>VLOOKUP($A6,'[2]master plan'!$A:$N,14,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="L6" s="26"/>
+      <c r="M6" s="27"/>
+    </row>
+    <row r="7" spans="1:13" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="17"/>
+      <c r="B7" s="18" t="e">
+        <f>VLOOKUP(A7,'[2]master plan'!A:C,3,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C7" s="19" t="e">
+        <f>VLOOKUP($A7,'[2]master plan'!$A:$N,5,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D7" s="20" t="e">
+        <f>VLOOKUP($A7,'[2]master plan'!$A:$N,6,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E7" s="21" t="e">
+        <f>VLOOKUP(A7,'[2]master plan'!A:G,7,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F7" s="22" t="e">
+        <f>VLOOKUP(A7,'[2]master plan'!A:H,8,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="G7" s="23" t="e">
+        <f>VLOOKUP(A7,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H7" s="24" t="e">
+        <f>VLOOKUP(A7,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="I7" s="25" t="e">
+        <f>VLOOKUP($A7,'[2]master plan'!$A:$N,12,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="J7" s="25" t="e">
+        <f>VLOOKUP($A7,'[2]master plan'!$A:$N,13,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="K7" s="25" t="e">
+        <f>VLOOKUP($A7,'[2]master plan'!$A:$N,14,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="L7" s="26"/>
+      <c r="M7" s="27"/>
+    </row>
+    <row r="8" spans="1:13" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="17"/>
+      <c r="B8" s="18" t="e">
+        <f>VLOOKUP(A8,'[2]master plan'!A:C,3,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C8" s="19" t="e">
+        <f>VLOOKUP($A8,'[2]master plan'!$A:$N,5,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D8" s="20" t="e">
+        <f>VLOOKUP($A8,'[2]master plan'!$A:$N,6,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E8" s="21" t="e">
+        <f>VLOOKUP(A8,'[2]master plan'!A:G,7,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F8" s="22" t="e">
+        <f>VLOOKUP(A8,'[2]master plan'!A:H,8,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="G8" s="23" t="e">
+        <f>VLOOKUP(A8,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H8" s="24" t="e">
+        <f>VLOOKUP(A8,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="I8" s="25" t="e">
+        <f>VLOOKUP($A8,'[2]master plan'!$A:$N,12,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="J8" s="25" t="e">
+        <f>VLOOKUP($A8,'[2]master plan'!$A:$N,13,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="K8" s="25" t="e">
+        <f>VLOOKUP($A8,'[2]master plan'!$A:$N,14,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="L8" s="26"/>
+      <c r="M8" s="27"/>
+    </row>
+    <row r="9" spans="1:13" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="17"/>
+      <c r="B9" s="18" t="e">
+        <f>VLOOKUP(A9,'[2]master plan'!A:C,3,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C9" s="19" t="e">
+        <f>VLOOKUP($A9,'[2]master plan'!$A:$N,5,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D9" s="20" t="e">
+        <f>VLOOKUP($A9,'[2]master plan'!$A:$N,6,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E9" s="21" t="e">
+        <f>VLOOKUP(A9,'[2]master plan'!A:G,7,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F9" s="22" t="e">
+        <f>VLOOKUP(A9,'[2]master plan'!A:H,8,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="G9" s="23" t="e">
+        <f>VLOOKUP(A9,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H9" s="24" t="e">
+        <f>VLOOKUP(A9,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="I9" s="25" t="e">
+        <f>VLOOKUP($A9,'[2]master plan'!$A:$N,12,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="J9" s="25" t="e">
+        <f>VLOOKUP($A9,'[2]master plan'!$A:$N,13,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="K9" s="25" t="e">
+        <f>VLOOKUP($A9,'[2]master plan'!$A:$N,14,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="L9" s="26"/>
+      <c r="M9" s="40"/>
+    </row>
+    <row r="10" spans="1:13" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="17"/>
+      <c r="B10" s="18" t="e">
+        <f>VLOOKUP(A10,'[2]master plan'!A:C,3,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C10" s="19" t="e">
+        <f>VLOOKUP($A10,'[2]master plan'!$A:$N,5,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D10" s="20" t="e">
+        <f>VLOOKUP($A10,'[2]master plan'!$A:$N,6,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E10" s="21" t="e">
+        <f>VLOOKUP(A10,'[2]master plan'!A:G,7,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F10" s="22" t="e">
+        <f>VLOOKUP(A10,'[2]master plan'!A:H,8,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="G10" s="23" t="e">
+        <f>VLOOKUP(A10,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H10" s="24" t="e">
+        <f>VLOOKUP(A10,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="I10" s="25" t="e">
+        <f>VLOOKUP($A10,'[2]master plan'!$A:$N,12,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="J10" s="25" t="e">
+        <f>VLOOKUP($A10,'[2]master plan'!$A:$N,13,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="K10" s="25" t="e">
+        <f>VLOOKUP($A10,'[2]master plan'!$A:$N,14,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="L10" s="26"/>
+      <c r="M10" s="27"/>
+    </row>
+    <row r="11" spans="1:13" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="17"/>
+      <c r="B11" s="18" t="e">
+        <f>VLOOKUP(A11,'[2]master plan'!A:C,3,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C11" s="19" t="e">
+        <f>VLOOKUP($A11,'[2]master plan'!$A:$N,5,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D11" s="20" t="e">
+        <f>VLOOKUP($A11,'[2]master plan'!$A:$N,6,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E11" s="21" t="e">
+        <f>VLOOKUP(A11,'[2]master plan'!A:G,7,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F11" s="22" t="e">
+        <f>VLOOKUP(A11,'[2]master plan'!A:H,8,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="G11" s="23" t="e">
+        <f>VLOOKUP(A11,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H11" s="24" t="e">
+        <f>VLOOKUP(A11,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="I11" s="25" t="e">
+        <f>VLOOKUP($A11,'[2]master plan'!$A:$N,12,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="J11" s="25" t="e">
+        <f>VLOOKUP($A11,'[2]master plan'!$A:$N,13,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="K11" s="25" t="e">
+        <f>VLOOKUP($A11,'[2]master plan'!$A:$N,14,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="L11" s="26"/>
+      <c r="M11" s="27"/>
+    </row>
+    <row r="12" spans="1:13" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="17"/>
+      <c r="B12" s="18" t="e">
+        <f>VLOOKUP(A12,'[2]master plan'!A:C,3,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C12" s="19" t="e">
+        <f>VLOOKUP($A12,'[2]master plan'!$A:$N,5,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D12" s="20" t="e">
+        <f>VLOOKUP($A12,'[2]master plan'!$A:$N,6,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E12" s="21" t="e">
+        <f>VLOOKUP(A12,'[2]master plan'!A:G,7,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F12" s="22" t="e">
+        <f>VLOOKUP(A12,'[2]master plan'!A:H,8,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="G12" s="23" t="e">
+        <f>VLOOKUP(A12,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H12" s="24" t="e">
+        <f>VLOOKUP(A12,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="I12" s="25" t="e">
+        <f>VLOOKUP($A12,'[2]master plan'!$A:$N,12,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="J12" s="25" t="e">
+        <f>VLOOKUP($A12,'[2]master plan'!$A:$N,13,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="K12" s="25" t="e">
+        <f>VLOOKUP($A12,'[2]master plan'!$A:$N,14,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="L12" s="26"/>
+      <c r="M12" s="40"/>
+    </row>
+    <row r="13" spans="1:13" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="17"/>
+      <c r="B13" s="18" t="e">
+        <f>VLOOKUP(A13,'[2]master plan'!A:C,3,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C13" s="19" t="e">
+        <f>VLOOKUP($A13,'[2]master plan'!$A:$N,5,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D13" s="20" t="e">
+        <f>VLOOKUP($A13,'[2]master plan'!$A:$N,6,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E13" s="21" t="e">
+        <f>VLOOKUP(A13,'[2]master plan'!A:G,7,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F13" s="22" t="e">
+        <f>VLOOKUP(A13,'[2]master plan'!A:H,8,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="G13" s="23" t="e">
+        <f>VLOOKUP(A13,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H13" s="24" t="e">
+        <f>VLOOKUP(A13,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="I13" s="25" t="e">
+        <f>VLOOKUP($A13,'[2]master plan'!$A:$N,12,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="J13" s="25" t="e">
+        <f>VLOOKUP($A13,'[2]master plan'!$A:$N,13,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="K13" s="25" t="e">
+        <f>VLOOKUP($A13,'[2]master plan'!$A:$N,14,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="L13" s="26"/>
+      <c r="M13" s="40"/>
+    </row>
+    <row r="14" spans="1:13" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="17"/>
+      <c r="B14" s="18" t="e">
+        <f>VLOOKUP(A14,'[2]master plan'!A:C,3,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C14" s="19" t="e">
+        <f>VLOOKUP($A14,'[2]master plan'!$A:$N,5,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D14" s="20" t="e">
+        <f>VLOOKUP($A14,'[2]master plan'!$A:$N,6,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E14" s="21" t="e">
+        <f>VLOOKUP(A14,'[2]master plan'!A:G,7,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F14" s="22" t="e">
+        <f>VLOOKUP(A14,'[2]master plan'!A:H,8,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="G14" s="23" t="e">
+        <f>VLOOKUP(A14,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H14" s="24" t="e">
+        <f>VLOOKUP(A14,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="I14" s="25" t="e">
+        <f>VLOOKUP($A14,'[2]master plan'!$A:$N,12,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="J14" s="25" t="e">
+        <f>VLOOKUP($A14,'[2]master plan'!$A:$N,13,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="K14" s="25" t="e">
+        <f>VLOOKUP($A14,'[2]master plan'!$A:$N,14,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="L14" s="26"/>
+      <c r="M14" s="27"/>
+    </row>
+    <row r="15" spans="1:13" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="17"/>
+      <c r="B15" s="18" t="e">
+        <f>VLOOKUP(A15,'[2]master plan'!A:C,3,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C15" s="19" t="e">
+        <f>VLOOKUP($A15,'[2]master plan'!$A:$N,5,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D15" s="20" t="e">
+        <f>VLOOKUP($A15,'[2]master plan'!$A:$N,6,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E15" s="21" t="e">
+        <f>VLOOKUP(A15,'[2]master plan'!A:G,7,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F15" s="22" t="e">
+        <f>VLOOKUP(A15,'[2]master plan'!A:H,8,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="G15" s="23" t="e">
+        <f>VLOOKUP(A15,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H15" s="24" t="e">
+        <f>VLOOKUP(A15,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="I15" s="25" t="e">
+        <f>VLOOKUP($A15,'[2]master plan'!$A:$N,12,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="J15" s="25" t="e">
+        <f>VLOOKUP($A15,'[2]master plan'!$A:$N,13,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="K15" s="25" t="e">
+        <f>VLOOKUP($A15,'[2]master plan'!$A:$N,14,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="L15" s="26"/>
+      <c r="M15" s="40"/>
+    </row>
+    <row r="16" spans="1:13" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="17"/>
+      <c r="B16" s="18" t="e">
+        <f>VLOOKUP(A16,'[2]master plan'!A:C,3,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C16" s="19" t="e">
+        <f>VLOOKUP($A16,'[2]master plan'!$A:$N,5,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D16" s="20" t="e">
+        <f>VLOOKUP($A16,'[2]master plan'!$A:$N,6,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E16" s="21" t="e">
+        <f>VLOOKUP(A16,'[2]master plan'!A:G,7,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F16" s="22" t="e">
+        <f>VLOOKUP(A16,'[2]master plan'!A:H,8,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="G16" s="23" t="e">
+        <f>VLOOKUP(A16,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H16" s="24" t="e">
+        <f>VLOOKUP(A16,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="I16" s="25" t="e">
+        <f>VLOOKUP($A16,'[2]master plan'!$A:$N,12,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="J16" s="25" t="e">
+        <f>VLOOKUP($A16,'[2]master plan'!$A:$N,13,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="K16" s="25" t="e">
+        <f>VLOOKUP($A16,'[2]master plan'!$A:$N,14,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="L16" s="26"/>
+      <c r="M16" s="40"/>
+    </row>
+    <row r="17" spans="1:13" s="3" customFormat="1" ht="70" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="17"/>
+      <c r="B17" s="18" t="e">
+        <f>VLOOKUP(A17,'[2]master plan'!A:C,3,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="C17" s="19" t="e">
+        <f>VLOOKUP($A17,'[2]master plan'!$A:$N,5,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="D17" s="20" t="e">
+        <f>VLOOKUP($A17,'[2]master plan'!$A:$N,6,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="E17" s="21" t="e">
+        <f>VLOOKUP(A17,'[2]master plan'!A:G,7,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="F17" s="22" t="e">
+        <f>VLOOKUP(A17,'[2]master plan'!A:H,8,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="G17" s="23" t="e">
+        <f>VLOOKUP(A17,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="H17" s="24" t="e">
+        <f>VLOOKUP(A17,'[2]master plan'!A:W,23,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="I17" s="25" t="e">
+        <f>VLOOKUP($A17,'[2]master plan'!$A:$N,12,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="J17" s="25" t="e">
+        <f>VLOOKUP($A17,'[2]master plan'!$A:$N,13,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="K17" s="25" t="e">
+        <f>VLOOKUP($A17,'[2]master plan'!$A:$N,14,0)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="L17" s="26"/>
+      <c r="M17" s="40"/>
+    </row>
+    <row r="18" spans="1:13" s="3" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="41"/>
+      <c r="B18" s="42"/>
+      <c r="C18" s="43"/>
+      <c r="D18" s="43"/>
+      <c r="E18" s="44"/>
+      <c r="F18" s="45"/>
+      <c r="G18" s="45"/>
+      <c r="H18" s="45"/>
+      <c r="I18" s="46"/>
+      <c r="J18" s="47"/>
+      <c r="K18" s="48"/>
+      <c r="L18" s="49"/>
+      <c r="M18" s="50"/>
+    </row>
+    <row r="19" spans="1:13" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="L19" s="56"/>
+    </row>
+    <row r="20" spans="1:13" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="L20" s="56"/>
+    </row>
+    <row r="21" spans="1:13" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="L21" s="56"/>
+    </row>
+    <row r="22" spans="1:13" s="54" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="2"/>
+      <c r="B22" s="52"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+      <c r="E22" s="59" t="s">
+        <v>21</v>
+      </c>
+      <c r="G22" s="55"/>
+      <c r="I22" s="53"/>
+      <c r="J22" s="53"/>
+      <c r="K22" s="53"/>
+      <c r="L22" s="56"/>
+      <c r="M22" s="57"/>
+    </row>
+    <row r="23" spans="1:13" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="L23" s="56"/>
+    </row>
+    <row r="24" spans="1:13" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="L24" s="56"/>
+    </row>
+    <row r="25" spans="1:13" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="2"/>
+      <c r="B25" s="52"/>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
+      <c r="E25" s="53"/>
+      <c r="F25" s="54"/>
+      <c r="G25" s="54"/>
+      <c r="H25" s="55"/>
+      <c r="I25" s="53"/>
+      <c r="J25" s="53"/>
+      <c r="K25" s="53"/>
+      <c r="L25" s="56"/>
+      <c r="M25" s="57"/>
+    </row>
+    <row r="26" spans="1:13" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="2"/>
+      <c r="B26" s="52"/>
+      <c r="C26" s="2"/>
+      <c r="D26" s="2"/>
+      <c r="E26" s="53"/>
+      <c r="F26" s="54"/>
+      <c r="G26" s="54"/>
+      <c r="H26" s="55"/>
+      <c r="I26" s="53"/>
+      <c r="J26" s="53"/>
+      <c r="K26" s="53"/>
+      <c r="L26" s="56"/>
+      <c r="M26" s="57"/>
+    </row>
+    <row r="27" spans="1:13" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="2"/>
+      <c r="B27" s="52"/>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
+      <c r="E27" s="53"/>
+      <c r="F27" s="54"/>
+      <c r="G27" s="54"/>
+      <c r="H27" s="55"/>
+      <c r="I27" s="53"/>
+      <c r="J27" s="53"/>
+      <c r="K27" s="53"/>
+      <c r="L27" s="56"/>
+      <c r="M27" s="57"/>
+    </row>
+    <row r="28" spans="1:13" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="2"/>
+      <c r="B28" s="52"/>
+      <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
+      <c r="E28" s="53"/>
+      <c r="F28" s="54"/>
+      <c r="G28" s="54"/>
+      <c r="H28" s="55"/>
+      <c r="I28" s="53"/>
+      <c r="J28" s="53"/>
+      <c r="K28" s="53"/>
+      <c r="L28" s="56"/>
+      <c r="M28" s="57"/>
+    </row>
+    <row r="29" spans="1:13" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="2"/>
+      <c r="B29" s="52"/>
+      <c r="C29" s="2"/>
+      <c r="D29" s="2"/>
+      <c r="E29" s="53"/>
+      <c r="F29" s="54"/>
+      <c r="G29" s="54"/>
+      <c r="H29" s="55"/>
+      <c r="I29" s="53"/>
+      <c r="J29" s="53"/>
+      <c r="K29" s="53"/>
+      <c r="L29" s="56"/>
+      <c r="M29" s="57"/>
+    </row>
+    <row r="30" spans="1:13" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="2"/>
+      <c r="B30" s="52"/>
+      <c r="C30" s="2"/>
+      <c r="D30" s="2"/>
+      <c r="E30" s="53"/>
+      <c r="F30" s="54"/>
+      <c r="G30" s="54"/>
+      <c r="H30" s="55"/>
+      <c r="I30" s="53"/>
+      <c r="J30" s="53"/>
+      <c r="K30" s="53"/>
+      <c r="L30" s="56"/>
+      <c r="M30" s="57"/>
+    </row>
+    <row r="31" spans="1:13" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="2"/>
+      <c r="B31" s="52"/>
+      <c r="C31" s="2"/>
+      <c r="D31" s="2"/>
+      <c r="E31" s="53"/>
+      <c r="F31" s="54"/>
+      <c r="G31" s="54"/>
+      <c r="H31" s="55"/>
+      <c r="I31" s="53"/>
+      <c r="J31" s="53"/>
+      <c r="K31" s="53"/>
+      <c r="L31" s="56"/>
+      <c r="M31" s="57"/>
+    </row>
+    <row r="32" spans="1:13" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="2"/>
+      <c r="B32" s="52"/>
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
+      <c r="E32" s="53"/>
+      <c r="F32" s="54"/>
+      <c r="G32" s="54"/>
+      <c r="H32" s="55"/>
+      <c r="I32" s="53"/>
+      <c r="J32" s="53"/>
+      <c r="K32" s="53"/>
+      <c r="L32" s="56"/>
+      <c r="M32" s="57"/>
+    </row>
+    <row r="33" spans="1:13" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="2"/>
+      <c r="B33" s="52"/>
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
+      <c r="E33" s="53"/>
+      <c r="F33" s="54"/>
+      <c r="G33" s="54"/>
+      <c r="H33" s="55"/>
+      <c r="I33" s="53"/>
+      <c r="J33" s="53"/>
+      <c r="K33" s="53"/>
+      <c r="L33" s="56"/>
+      <c r="M33" s="57"/>
+    </row>
+    <row r="34" spans="1:13" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="2"/>
+      <c r="B34" s="52"/>
+      <c r="C34" s="2"/>
+      <c r="D34" s="2"/>
+      <c r="E34" s="53"/>
+      <c r="F34" s="54"/>
+      <c r="G34" s="54"/>
+      <c r="H34" s="55"/>
+      <c r="I34" s="53"/>
+      <c r="J34" s="53"/>
+      <c r="K34" s="53"/>
+      <c r="L34" s="56"/>
+      <c r="M34" s="57"/>
+    </row>
+    <row r="35" spans="1:13" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="2"/>
+      <c r="B35" s="52"/>
+      <c r="C35" s="2"/>
+      <c r="D35" s="2"/>
+      <c r="E35" s="53"/>
+      <c r="F35" s="54"/>
+      <c r="G35" s="54"/>
+      <c r="H35" s="55"/>
+      <c r="I35" s="53"/>
+      <c r="J35" s="53"/>
+      <c r="K35" s="53"/>
+      <c r="L35" s="56"/>
+      <c r="M35" s="57"/>
+    </row>
+    <row r="36" spans="1:13" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="2"/>
+      <c r="B36" s="52"/>
+      <c r="C36" s="2"/>
+      <c r="D36" s="2"/>
+      <c r="E36" s="53"/>
+      <c r="F36" s="54"/>
+      <c r="G36" s="54"/>
+      <c r="H36" s="55"/>
+      <c r="I36" s="53"/>
+      <c r="J36" s="53"/>
+      <c r="K36" s="53"/>
+      <c r="L36" s="56"/>
+      <c r="M36" s="57"/>
+    </row>
+    <row r="37" spans="1:13" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="2"/>
+      <c r="B37" s="52"/>
+      <c r="C37" s="2"/>
+      <c r="D37" s="2"/>
+      <c r="E37" s="53"/>
+      <c r="F37" s="54"/>
+      <c r="G37" s="54"/>
+      <c r="H37" s="55"/>
+      <c r="I37" s="53"/>
+      <c r="J37" s="53"/>
+      <c r="K37" s="53"/>
+      <c r="L37" s="56"/>
+      <c r="M37" s="57"/>
+    </row>
+    <row r="38" spans="1:13" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="2"/>
+      <c r="B38" s="52"/>
+      <c r="C38" s="2"/>
+      <c r="D38" s="2"/>
+      <c r="E38" s="53"/>
+      <c r="F38" s="54"/>
+      <c r="G38" s="54"/>
+      <c r="H38" s="55"/>
+      <c r="I38" s="53"/>
+      <c r="J38" s="53"/>
+      <c r="K38" s="53"/>
+      <c r="L38" s="56"/>
+      <c r="M38" s="57"/>
+    </row>
+    <row r="39" spans="1:13" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="2"/>
+      <c r="B39" s="52"/>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
+      <c r="E39" s="53"/>
+      <c r="F39" s="54"/>
+      <c r="G39" s="54"/>
+      <c r="H39" s="55"/>
+      <c r="I39" s="53"/>
+      <c r="J39" s="53"/>
+      <c r="K39" s="53"/>
+      <c r="L39" s="56"/>
+      <c r="M39" s="57"/>
+    </row>
+    <row r="40" spans="1:13" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A40" s="2"/>
+      <c r="B40" s="52"/>
+      <c r="C40" s="2"/>
+      <c r="D40" s="2"/>
+      <c r="E40" s="53"/>
+      <c r="F40" s="54"/>
+      <c r="G40" s="54"/>
+      <c r="H40" s="55"/>
+      <c r="I40" s="53"/>
+      <c r="J40" s="53"/>
+      <c r="K40" s="53"/>
+      <c r="L40" s="56"/>
+      <c r="M40" s="57"/>
+    </row>
+    <row r="41" spans="1:13" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A41" s="2"/>
+      <c r="B41" s="52"/>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
+      <c r="E41" s="53"/>
+      <c r="F41" s="54"/>
+      <c r="G41" s="54"/>
+      <c r="H41" s="55"/>
+      <c r="I41" s="53"/>
+      <c r="J41" s="53"/>
+      <c r="K41" s="53"/>
+      <c r="L41" s="56"/>
+      <c r="M41" s="57"/>
+    </row>
+    <row r="42" spans="1:13" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A42" s="2"/>
+      <c r="B42" s="52"/>
+      <c r="C42" s="2"/>
+      <c r="D42" s="2"/>
+      <c r="E42" s="53"/>
+      <c r="F42" s="54"/>
+      <c r="G42" s="54"/>
+      <c r="H42" s="55"/>
+      <c r="I42" s="53"/>
+      <c r="J42" s="53"/>
+      <c r="K42" s="53"/>
+      <c r="L42" s="56"/>
+      <c r="M42" s="57"/>
+    </row>
+    <row r="43" spans="1:13" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A43" s="2"/>
+      <c r="B43" s="52"/>
+      <c r="C43" s="2"/>
+      <c r="D43" s="2"/>
+      <c r="E43" s="53"/>
+      <c r="F43" s="54"/>
+      <c r="G43" s="54"/>
+      <c r="H43" s="55"/>
+      <c r="I43" s="53"/>
+      <c r="J43" s="53"/>
+      <c r="K43" s="53"/>
+      <c r="L43" s="56"/>
+      <c r="M43" s="57"/>
+    </row>
+    <row r="44" spans="1:13" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A44" s="2"/>
+      <c r="B44" s="52"/>
+      <c r="C44" s="2"/>
+      <c r="D44" s="2"/>
+      <c r="E44" s="53"/>
+      <c r="F44" s="54"/>
+      <c r="G44" s="54"/>
+      <c r="H44" s="55"/>
+      <c r="I44" s="53"/>
+      <c r="J44" s="53"/>
+      <c r="K44" s="53"/>
+      <c r="L44" s="56"/>
+      <c r="M44" s="57"/>
+    </row>
+    <row r="45" spans="1:13" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A45" s="2"/>
+      <c r="B45" s="52"/>
+      <c r="C45" s="2"/>
+      <c r="D45" s="2"/>
+      <c r="E45" s="53"/>
+      <c r="F45" s="54"/>
+      <c r="G45" s="54"/>
+      <c r="H45" s="55"/>
+      <c r="I45" s="53"/>
+      <c r="J45" s="53"/>
+      <c r="K45" s="53"/>
+      <c r="L45" s="56"/>
+      <c r="M45" s="57"/>
+    </row>
+    <row r="46" spans="1:13" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A46" s="2"/>
+      <c r="B46" s="52"/>
+      <c r="C46" s="2"/>
+      <c r="D46" s="2"/>
+      <c r="E46" s="53"/>
+      <c r="F46" s="54"/>
+      <c r="G46" s="54"/>
+      <c r="H46" s="55"/>
+      <c r="I46" s="53"/>
+      <c r="J46" s="53"/>
+      <c r="K46" s="53"/>
+      <c r="L46" s="56"/>
+      <c r="M46" s="57"/>
+    </row>
+    <row r="47" spans="1:13" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A47" s="2"/>
+      <c r="B47" s="52"/>
+      <c r="C47" s="2"/>
+      <c r="D47" s="2"/>
+      <c r="E47" s="53"/>
+      <c r="F47" s="54"/>
+      <c r="G47" s="54"/>
+      <c r="H47" s="55"/>
+      <c r="I47" s="53"/>
+      <c r="J47" s="53"/>
+      <c r="K47" s="53"/>
+      <c r="L47" s="56"/>
+      <c r="M47" s="57"/>
+    </row>
+    <row r="48" spans="1:13" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A48" s="2"/>
+      <c r="B48" s="52"/>
+      <c r="C48" s="2"/>
+      <c r="D48" s="2"/>
+      <c r="E48" s="53"/>
+      <c r="F48" s="54"/>
+      <c r="G48" s="54"/>
+      <c r="H48" s="55"/>
+      <c r="I48" s="53"/>
+      <c r="J48" s="53"/>
+      <c r="K48" s="53"/>
+      <c r="L48" s="56"/>
+      <c r="M48" s="57"/>
+    </row>
+    <row r="49" spans="1:13" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A49" s="2"/>
+      <c r="B49" s="52"/>
+      <c r="C49" s="2"/>
+      <c r="D49" s="2"/>
+      <c r="E49" s="53"/>
+      <c r="F49" s="54"/>
+      <c r="G49" s="54"/>
+      <c r="H49" s="55"/>
+      <c r="I49" s="53"/>
+      <c r="J49" s="53"/>
+      <c r="K49" s="53"/>
+      <c r="L49" s="56"/>
+      <c r="M49" s="57"/>
+    </row>
+    <row r="50" spans="1:13" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A50" s="2"/>
+      <c r="B50" s="52"/>
+      <c r="C50" s="2"/>
+      <c r="D50" s="2"/>
+      <c r="E50" s="53"/>
+      <c r="F50" s="54"/>
+      <c r="G50" s="54"/>
+      <c r="H50" s="55"/>
+      <c r="I50" s="53"/>
+      <c r="J50" s="53"/>
+      <c r="K50" s="53"/>
+      <c r="L50" s="56"/>
+      <c r="M50" s="57"/>
+    </row>
+    <row r="51" spans="1:13" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A51" s="2"/>
+      <c r="B51" s="52"/>
+      <c r="C51" s="2"/>
+      <c r="D51" s="2"/>
+      <c r="E51" s="53"/>
+      <c r="F51" s="54"/>
+      <c r="G51" s="54"/>
+      <c r="H51" s="55"/>
+      <c r="I51" s="53"/>
+      <c r="J51" s="53"/>
+      <c r="K51" s="53"/>
+      <c r="L51" s="56"/>
+      <c r="M51" s="57"/>
+    </row>
+    <row r="52" spans="1:13" s="10" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A52" s="2"/>
+      <c r="B52" s="52"/>
+      <c r="C52" s="2"/>
+      <c r="D52" s="2"/>
+      <c r="E52" s="53"/>
+      <c r="F52" s="54"/>
+      <c r="G52" s="54"/>
+      <c r="H52" s="55"/>
+      <c r="I52" s="53"/>
+      <c r="J52" s="53"/>
+      <c r="K52" s="53"/>
+      <c r="L52" s="56"/>
+      <c r="M52" s="57"/>
+    </row>
+    <row r="661" spans="1:13" s="54" customFormat="1" ht="74.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A661" s="2"/>
+      <c r="B661" s="52"/>
+      <c r="C661" s="2"/>
+      <c r="D661" s="2"/>
+      <c r="E661" s="60"/>
+      <c r="H661" s="55"/>
+      <c r="I661" s="53"/>
+      <c r="J661" s="53"/>
+      <c r="K661" s="53"/>
+      <c r="L661" s="61"/>
+      <c r="M661" s="57"/>
+    </row>
+  </sheetData>
+  <protectedRanges>
+    <protectedRange algorithmName="SHA-512" hashValue="e1FOu1UlwA7reaiyQlEGzbU6dAFPyHPlKfgo6VzFBBobawyOfUsh2c/+wjC8bICpcXVPmRerMGA9+qKsw5p7Iw==" saltValue="UD2tVZrxqZTGI3vDzMBrHw==" spinCount="100000" sqref="E3:E17" name="Range1_1"/>
+  </protectedRanges>
+  <autoFilter ref="A2:M18" xr:uid="{E2BC4C4A-3703-4A99-A30B-53817C3A378F}">
+    <filterColumn colId="3">
+      <filters blank="1">
+        <filter val="PVN-003672"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
+  <mergeCells count="1">
+    <mergeCell ref="D1:F1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A2">
+    <cfRule type="duplicateValues" dxfId="5" priority="4"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A3:A17">
+    <cfRule type="duplicateValues" dxfId="4" priority="6"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A20:A1048576">
+    <cfRule type="duplicateValues" dxfId="3" priority="5"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C1:C1048576">
+    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I2:M2">
+    <cfRule type="duplicateValues" dxfId="0" priority="3"/>
+  </conditionalFormatting>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.18" right="0.17" top="0.5" bottom="0" header="0.17" footer="0.17"/>
+  <pageSetup paperSize="9" scale="30" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <headerFooter>
+    <oddFooter>Page &amp;P of &amp;N</oddFooter>
+  </headerFooter>
+  <rowBreaks count="1" manualBreakCount="1">
+    <brk id="18" max="15" man="1"/>
   </rowBreaks>
 </worksheet>
 </file>
@@ -47198,7 +48652,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46178.924539467589</v>
+        <v>46179.701554050924</v>
       </c>
       <c r="D1" s="83" t="s">
         <v>1</v>
@@ -48547,23 +50001,23 @@
     <mergeCell ref="D1:F1"/>
   </mergeCells>
   <conditionalFormatting sqref="A2">
-    <cfRule type="duplicateValues" dxfId="92" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="98" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:A23">
-    <cfRule type="duplicateValues" dxfId="91" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="97" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A26:A1048576">
-    <cfRule type="duplicateValues" dxfId="90" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="96" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="89" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="88" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="95" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="94" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:M2">
-    <cfRule type="duplicateValues" dxfId="87" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="93" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1">
-    <cfRule type="duplicateValues" dxfId="86" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="92" priority="3"/>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.18" right="0.17" top="0.5" bottom="0" header="0.17" footer="0.17"/>
@@ -48608,7 +50062,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46178.924539467589</v>
+        <v>46179.701554050924</v>
       </c>
       <c r="D1" s="83" t="s">
         <v>1</v>
@@ -50015,23 +51469,23 @@
     <mergeCell ref="D1:F1"/>
   </mergeCells>
   <conditionalFormatting sqref="A2">
-    <cfRule type="duplicateValues" dxfId="85" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="91" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:A28">
-    <cfRule type="duplicateValues" dxfId="84" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="90" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A31:A1048576">
-    <cfRule type="duplicateValues" dxfId="83" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="89" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="82" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="81" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="88" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="87" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:M2">
-    <cfRule type="duplicateValues" dxfId="80" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="86" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1">
-    <cfRule type="duplicateValues" dxfId="79" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="85" priority="3"/>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.18" right="0.17" top="0.5" bottom="0" header="0.17" footer="0.17"/>
@@ -50076,7 +51530,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46178.924539467589</v>
+        <v>46179.701554050924</v>
       </c>
       <c r="D1" s="83" t="s">
         <v>1</v>
@@ -51449,23 +52903,23 @@
     <mergeCell ref="D1:F1"/>
   </mergeCells>
   <conditionalFormatting sqref="A2">
-    <cfRule type="duplicateValues" dxfId="78" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="84" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:A25">
-    <cfRule type="duplicateValues" dxfId="77" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="83" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A28:A1048576">
-    <cfRule type="duplicateValues" dxfId="76" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="82" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="75" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="74" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="81" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="80" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:M2">
-    <cfRule type="duplicateValues" dxfId="73" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="79" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1">
-    <cfRule type="duplicateValues" dxfId="72" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="78" priority="3"/>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.18" right="0.17" top="0.5" bottom="0" header="0.17" footer="0.17"/>
@@ -51509,7 +52963,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46178.924539467589</v>
+        <v>46179.701554050924</v>
       </c>
       <c r="D1" s="83" t="s">
         <v>1</v>
@@ -52724,39 +54178,39 @@
     <mergeCell ref="D7:F7"/>
   </mergeCells>
   <conditionalFormatting sqref="A2">
-    <cfRule type="duplicateValues" dxfId="71" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="77" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:A6 A14:A18">
-    <cfRule type="duplicateValues" dxfId="70" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="76" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A8">
-    <cfRule type="duplicateValues" dxfId="69" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="75" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A9:A13">
-    <cfRule type="duplicateValues" dxfId="68" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="74" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A21:A1048576">
-    <cfRule type="duplicateValues" dxfId="67" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="73" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C6 C14:C1048576">
-    <cfRule type="duplicateValues" dxfId="66" priority="7"/>
-    <cfRule type="duplicateValues" dxfId="65" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="72" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="71" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C7:C13">
-    <cfRule type="duplicateValues" dxfId="64" priority="2"/>
-    <cfRule type="duplicateValues" dxfId="63" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="70" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="69" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I8:L8">
-    <cfRule type="duplicateValues" dxfId="62" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="68" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:M2">
-    <cfRule type="duplicateValues" dxfId="61" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="67" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="M7">
-    <cfRule type="duplicateValues" dxfId="60" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="66" priority="1"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1">
-    <cfRule type="duplicateValues" dxfId="59" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="65" priority="9"/>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.18" right="0.17" top="0.5" bottom="0" header="0.17" footer="0.17"/>
@@ -52801,7 +54255,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46178.924539467589</v>
+        <v>46179.701554050924</v>
       </c>
       <c r="D1" s="83" t="s">
         <v>1</v>
@@ -54126,26 +55580,26 @@
     <mergeCell ref="D1:F1"/>
   </mergeCells>
   <conditionalFormatting sqref="A2">
-    <cfRule type="duplicateValues" dxfId="58" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="64" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:A15">
-    <cfRule type="duplicateValues" dxfId="57" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="63" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A16:A21">
-    <cfRule type="duplicateValues" dxfId="56" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="62" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A24:A1048576">
-    <cfRule type="duplicateValues" dxfId="55" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="61" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="54" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="53" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="60" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="59" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:M2">
-    <cfRule type="duplicateValues" dxfId="52" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="58" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1">
-    <cfRule type="duplicateValues" dxfId="51" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="57" priority="3"/>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.18" right="0.17" top="0.5" bottom="0" header="0.17" footer="0.17"/>
@@ -54191,7 +55645,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46178.924539467589</v>
+        <v>46179.701554050924</v>
       </c>
       <c r="D1" s="83" t="s">
         <v>1</v>
@@ -55546,23 +57000,23 @@
     <mergeCell ref="D1:F1"/>
   </mergeCells>
   <conditionalFormatting sqref="A2">
-    <cfRule type="duplicateValues" dxfId="50" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="56" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:A21">
-    <cfRule type="duplicateValues" dxfId="49" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="55" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A24:A1048576">
-    <cfRule type="duplicateValues" dxfId="48" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="54" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="47" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="46" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="53" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="52" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:M2">
-    <cfRule type="duplicateValues" dxfId="45" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="51" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1">
-    <cfRule type="duplicateValues" dxfId="44" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="50" priority="3"/>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.18" right="0.17" top="0.5" bottom="0" header="0.17" footer="0.17"/>
@@ -55607,7 +57061,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46178.924539467589</v>
+        <v>46179.701554050924</v>
       </c>
       <c r="D1" s="83" t="s">
         <v>1</v>
@@ -56995,24 +58449,24 @@
     <mergeCell ref="D1:F1"/>
   </mergeCells>
   <conditionalFormatting sqref="A2">
-    <cfRule type="duplicateValues" dxfId="43" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="49" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:A24">
-    <cfRule type="duplicateValues" dxfId="42" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="48" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A27:A1048576">
-    <cfRule type="duplicateValues" dxfId="41" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="47" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="40" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="39" priority="2"/>
-    <cfRule type="duplicateValues" dxfId="38" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="46" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="45" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="44" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:M2">
-    <cfRule type="duplicateValues" dxfId="37" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="43" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1">
-    <cfRule type="duplicateValues" dxfId="36" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="42" priority="4"/>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.18" right="0.17" top="0.5" bottom="0" header="0.17" footer="0.17"/>
@@ -57058,7 +58512,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46178.924539467589</v>
+        <v>46179.701554050924</v>
       </c>
       <c r="D1" s="83" t="s">
         <v>1</v>
@@ -58403,23 +59857,23 @@
     <mergeCell ref="D1:F1"/>
   </mergeCells>
   <conditionalFormatting sqref="A2">
-    <cfRule type="duplicateValues" dxfId="35" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="41" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:A20">
-    <cfRule type="duplicateValues" dxfId="34" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="40" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A23:A1048576">
-    <cfRule type="duplicateValues" dxfId="33" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="39" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="32" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="31" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="38" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="37" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:M2">
-    <cfRule type="duplicateValues" dxfId="30" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="36" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="N1">
-    <cfRule type="duplicateValues" dxfId="29" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="35" priority="3"/>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.18" right="0.17" top="0.5" bottom="0" header="0.17" footer="0.17"/>

</xml_diff>

<commit_message>
fix: sync encoding issues and upload all sample plans
</commit_message>
<xml_diff>
--- a/Kế hoach sản xuất Sample.xlsx
+++ b/Kế hoach sản xuất Sample.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="117" documentId="8_{C12FF075-160F-4BB4-977C-4D56BABB08BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{75102B01-28E5-4879-8A68-12ED4C094023}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="4" activeTab="14" xr2:uid="{E780E912-92A1-4ADF-95B1-638FE58CE194}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="4" activeTab="10" xr2:uid="{E780E912-92A1-4ADF-95B1-638FE58CE194}"/>
   </bookViews>
   <sheets>
     <sheet name="13.5" sheetId="1" r:id="rId1"/>
@@ -4229,84 +4229,49 @@
       <sheetData sheetId="2"/>
       <sheetData sheetId="3">
         <row r="1">
-          <cell r="A1"/>
-          <cell r="B1"/>
           <cell r="C1" t="str">
             <v>TẠM THỜI NGƯNG NHẬN LAZY</v>
           </cell>
-          <cell r="D1"/>
-          <cell r="E1"/>
-          <cell r="F1"/>
           <cell r="G1" t="str">
             <v>ASICS 12MM DÙNG BOM 132 (roundup(12/132),5)</v>
           </cell>
-          <cell r="H1"/>
-          <cell r="I1"/>
-          <cell r="J1"/>
-          <cell r="K1"/>
-          <cell r="L1"/>
-          <cell r="M1"/>
-          <cell r="N1"/>
-          <cell r="O1"/>
-          <cell r="P1"/>
-          <cell r="Q1"/>
-          <cell r="R1"/>
-          <cell r="S1"/>
-          <cell r="T1"/>
-          <cell r="U1"/>
-          <cell r="V1"/>
-          <cell r="W1"/>
         </row>
         <row r="2">
-          <cell r="A2"/>
-          <cell r="B2"/>
-          <cell r="C2"/>
-          <cell r="D2"/>
-          <cell r="E2"/>
-          <cell r="F2"/>
           <cell r="G2" t="str">
             <v>SAMPLE</v>
           </cell>
           <cell r="H2">
-            <v>25179</v>
+            <v>267</v>
           </cell>
           <cell r="I2">
-            <v>25179</v>
+            <v>267</v>
           </cell>
           <cell r="J2">
-            <v>24163</v>
+            <v>0</v>
           </cell>
           <cell r="K2">
-            <v>1016</v>
+            <v>267</v>
           </cell>
           <cell r="L2" t="str">
             <v>ASICS</v>
           </cell>
-          <cell r="M2"/>
-          <cell r="N2"/>
-          <cell r="O2"/>
-          <cell r="P2"/>
           <cell r="Q2" t="str">
             <v>ETD hệ thống+1ngay</v>
           </cell>
           <cell r="R2" t="e">
             <v>#VALUE!</v>
           </cell>
-          <cell r="S2"/>
-          <cell r="T2"/>
           <cell r="U2">
             <v>12</v>
           </cell>
-          <cell r="V2"/>
           <cell r="W2">
-            <v>1283</v>
+            <v>10</v>
           </cell>
         </row>
         <row r="3">
           <cell r="A3" t="str">
             <v>NO.Order</v>
           </cell>
-          <cell r="B3"/>
           <cell r="C3" t="str">
             <v>Firm plan
 (PU PVN)</v>
@@ -4391,7 +4356,6 @@
           <cell r="A4" t="str">
             <v>S-2026-01-01</v>
           </cell>
-          <cell r="B4"/>
           <cell r="C4" t="str">
             <v>RPRO-260105-0668</v>
           </cell>
@@ -4744,7 +4708,6 @@
           <cell r="A9" t="str">
             <v>S-2026-01-06</v>
           </cell>
-          <cell r="B9"/>
           <cell r="C9" t="str">
             <v>RPRO-260105-0673</v>
           </cell>
@@ -4813,7 +4776,6 @@
           <cell r="A10" t="str">
             <v>S-2026-01-07</v>
           </cell>
-          <cell r="B10"/>
           <cell r="C10" t="str">
             <v>RPRO-260105-0674</v>
           </cell>
@@ -4882,7 +4844,6 @@
           <cell r="A11" t="str">
             <v>S-2026-01-08</v>
           </cell>
-          <cell r="B11"/>
           <cell r="C11" t="str">
             <v>RPRO-260105-0675</v>
           </cell>
@@ -5093,7 +5054,6 @@
           <cell r="A14" t="str">
             <v>L-2026-01-11</v>
           </cell>
-          <cell r="B14"/>
           <cell r="C14" t="str">
             <v>RPRO-260105-0678</v>
           </cell>
@@ -5127,7 +5087,6 @@
           <cell r="M14" t="str">
             <v>Lab test</v>
           </cell>
-          <cell r="N14"/>
           <cell r="O14" t="str">
             <v>Lab test</v>
           </cell>
@@ -5160,7 +5119,6 @@
           <cell r="A15" t="str">
             <v>L-2026-01-12</v>
           </cell>
-          <cell r="B15"/>
           <cell r="C15" t="str">
             <v>RPRO-260105-0679</v>
           </cell>
@@ -5194,7 +5152,6 @@
           <cell r="M15" t="str">
             <v>Lab test</v>
           </cell>
-          <cell r="N15"/>
           <cell r="O15" t="str">
             <v>Lab test</v>
           </cell>
@@ -5227,7 +5184,6 @@
           <cell r="A16" t="str">
             <v>L-2026-01-13</v>
           </cell>
-          <cell r="B16"/>
           <cell r="C16" t="str">
             <v>RPRO-260105-0680</v>
           </cell>
@@ -5261,7 +5217,6 @@
           <cell r="M16" t="str">
             <v>Lab test</v>
           </cell>
-          <cell r="N16"/>
           <cell r="O16" t="str">
             <v>Lab test</v>
           </cell>
@@ -5294,7 +5249,6 @@
           <cell r="A17" t="str">
             <v>L-2026-01-14</v>
           </cell>
-          <cell r="B17"/>
           <cell r="C17" t="str">
             <v>RPRO-260105-0681</v>
           </cell>
@@ -5328,7 +5282,6 @@
           <cell r="M17" t="str">
             <v>Lab test</v>
           </cell>
-          <cell r="N17"/>
           <cell r="O17" t="str">
             <v>Lab test</v>
           </cell>
@@ -5397,7 +5350,6 @@
           <cell r="M18" t="str">
             <v>Lab test</v>
           </cell>
-          <cell r="N18"/>
           <cell r="O18" t="str">
             <v>Lab test</v>
           </cell>
@@ -5466,7 +5418,6 @@
           <cell r="M19" t="str">
             <v>Lab test</v>
           </cell>
-          <cell r="N19"/>
           <cell r="O19" t="str">
             <v>Lab test</v>
           </cell>
@@ -5854,7 +5805,6 @@
           <cell r="A25" t="str">
             <v>L-2026-01-22</v>
           </cell>
-          <cell r="B25"/>
           <cell r="C25" t="str">
             <v>RPRO-260109-0095</v>
           </cell>
@@ -5888,7 +5838,6 @@
           <cell r="M25" t="str">
             <v>Lab test</v>
           </cell>
-          <cell r="N25"/>
           <cell r="O25" t="str">
             <v>Lab test</v>
           </cell>
@@ -5921,7 +5870,6 @@
           <cell r="A26" t="str">
             <v>S-2026-01-23</v>
           </cell>
-          <cell r="B26"/>
           <cell r="C26" t="str">
             <v>RPRO-260113-0624</v>
           </cell>
@@ -5990,7 +5938,6 @@
           <cell r="A27" t="str">
             <v>S-2026-01-24</v>
           </cell>
-          <cell r="B27"/>
           <cell r="C27" t="str">
             <v>RPRO-260113-0625</v>
           </cell>
@@ -6059,7 +6006,6 @@
           <cell r="A28" t="str">
             <v>S-2026-01-25</v>
           </cell>
-          <cell r="B28"/>
           <cell r="C28" t="str">
             <v>RPRO-260113-0626</v>
           </cell>
@@ -6128,7 +6074,6 @@
           <cell r="A29" t="str">
             <v>S-2026-01-26</v>
           </cell>
-          <cell r="B29"/>
           <cell r="C29" t="str">
             <v>RPRO-260113-0627</v>
           </cell>
@@ -6197,7 +6142,6 @@
           <cell r="A30" t="str">
             <v>S-2026-01-27</v>
           </cell>
-          <cell r="B30"/>
           <cell r="C30" t="str">
             <v>RPRO-260113-0628</v>
           </cell>
@@ -6266,7 +6210,6 @@
           <cell r="A31" t="str">
             <v>S-2026-01-28</v>
           </cell>
-          <cell r="B31"/>
           <cell r="C31" t="str">
             <v>RPRO-260113-0629</v>
           </cell>
@@ -6335,7 +6278,6 @@
           <cell r="A32" t="str">
             <v>S-2026-01-29</v>
           </cell>
-          <cell r="B32"/>
           <cell r="C32" t="str">
             <v>RPRO-260113-0630</v>
           </cell>
@@ -6404,7 +6346,6 @@
           <cell r="A33" t="str">
             <v>S-2026-01-30</v>
           </cell>
-          <cell r="B33"/>
           <cell r="C33" t="str">
             <v>RPRO-260115-0298</v>
           </cell>
@@ -6473,7 +6414,6 @@
           <cell r="A34" t="str">
             <v>S-2026-01-31</v>
           </cell>
-          <cell r="B34"/>
           <cell r="C34" t="str">
             <v>RPRO-260115-0299</v>
           </cell>
@@ -6542,7 +6482,6 @@
           <cell r="A35" t="str">
             <v>S-2026-01-32</v>
           </cell>
-          <cell r="B35"/>
           <cell r="C35" t="str">
             <v>RPRO-260115-0300</v>
           </cell>
@@ -6611,7 +6550,6 @@
           <cell r="A36" t="str">
             <v>S-2026-01-33</v>
           </cell>
-          <cell r="B36"/>
           <cell r="C36" t="str">
             <v>RPRO-260115-0301</v>
           </cell>
@@ -6680,7 +6618,6 @@
           <cell r="A37" t="str">
             <v>S-2026-01-34</v>
           </cell>
-          <cell r="B37"/>
           <cell r="C37" t="str">
             <v>RPRO-260115-0302</v>
           </cell>
@@ -6749,7 +6686,6 @@
           <cell r="A38" t="str">
             <v>S-2026-01-35</v>
           </cell>
-          <cell r="B38"/>
           <cell r="C38" t="str">
             <v>RPRO-260115-0303</v>
           </cell>
@@ -6818,7 +6754,6 @@
           <cell r="A39" t="str">
             <v>S-2026-01-36</v>
           </cell>
-          <cell r="B39"/>
           <cell r="C39" t="str">
             <v>RPRO-260115-0304</v>
           </cell>
@@ -6887,7 +6822,6 @@
           <cell r="A40" t="str">
             <v>S-2026-01-37</v>
           </cell>
-          <cell r="B40"/>
           <cell r="C40" t="str">
             <v>RPRO-260115-0305</v>
           </cell>
@@ -6956,7 +6890,6 @@
           <cell r="A41" t="str">
             <v>S-2026-01-38</v>
           </cell>
-          <cell r="B41"/>
           <cell r="C41" t="str">
             <v>RPRO-260115-0306</v>
           </cell>
@@ -7025,7 +6958,6 @@
           <cell r="A42" t="str">
             <v>S-2026-01-39</v>
           </cell>
-          <cell r="B42"/>
           <cell r="C42" t="str">
             <v>RPRO-260115-0307</v>
           </cell>
@@ -7094,7 +7026,6 @@
           <cell r="A43" t="str">
             <v>S-2026-01-40</v>
           </cell>
-          <cell r="B43"/>
           <cell r="C43" t="str">
             <v>RPRO-260115-0308</v>
           </cell>
@@ -7163,7 +7094,6 @@
           <cell r="A44" t="str">
             <v>S-2026-01-41</v>
           </cell>
-          <cell r="B44"/>
           <cell r="C44" t="str">
             <v>RPRO-260115-0309</v>
           </cell>
@@ -7232,7 +7162,6 @@
           <cell r="A45" t="str">
             <v>S-2026-01-42</v>
           </cell>
-          <cell r="B45"/>
           <cell r="C45" t="str">
             <v>RPRO-260109-0096</v>
           </cell>
@@ -7301,7 +7230,6 @@
           <cell r="A46" t="str">
             <v>S-2026-01-43</v>
           </cell>
-          <cell r="B46"/>
           <cell r="C46" t="str">
             <v>RPRO-260109-0097</v>
           </cell>
@@ -7370,7 +7298,6 @@
           <cell r="A47" t="str">
             <v>S-2026-01-44</v>
           </cell>
-          <cell r="B47"/>
           <cell r="C47" t="str">
             <v>RPRO-260109-0098</v>
           </cell>
@@ -7439,7 +7366,6 @@
           <cell r="A48" t="str">
             <v>S-2026-01-45</v>
           </cell>
-          <cell r="B48"/>
           <cell r="C48" t="str">
             <v>RPRO-260109-0099</v>
           </cell>
@@ -7508,7 +7434,6 @@
           <cell r="A49" t="str">
             <v>S-2026-01-46</v>
           </cell>
-          <cell r="B49"/>
           <cell r="C49" t="str">
             <v>RPRO-260120-0349</v>
           </cell>
@@ -7577,7 +7502,6 @@
           <cell r="A50" t="str">
             <v>S-2026-01-47</v>
           </cell>
-          <cell r="B50"/>
           <cell r="C50" t="str">
             <v>RPRO-260120-0350</v>
           </cell>
@@ -7646,7 +7570,6 @@
           <cell r="A51" t="str">
             <v>S-2026-01-48</v>
           </cell>
-          <cell r="B51"/>
           <cell r="C51" t="str">
             <v>RPRO-260120-0351</v>
           </cell>
@@ -7715,7 +7638,6 @@
           <cell r="A52" t="str">
             <v>S-2026-01-49</v>
           </cell>
-          <cell r="B52"/>
           <cell r="C52" t="str">
             <v>RPRO-260120-0352</v>
           </cell>
@@ -7784,7 +7706,6 @@
           <cell r="A53" t="str">
             <v>S-2026-01-50</v>
           </cell>
-          <cell r="B53"/>
           <cell r="C53" t="str">
             <v>RPRO-260120-0353</v>
           </cell>
@@ -7853,7 +7774,6 @@
           <cell r="A54" t="str">
             <v>S-2026-01-51</v>
           </cell>
-          <cell r="B54"/>
           <cell r="C54" t="str">
             <v>RPRO-260120-0354</v>
           </cell>
@@ -7922,7 +7842,6 @@
           <cell r="A55" t="str">
             <v>S-2026-01-52</v>
           </cell>
-          <cell r="B55"/>
           <cell r="C55" t="str">
             <v>RPRO-260113-0631</v>
           </cell>
@@ -7991,7 +7910,6 @@
           <cell r="A56" t="str">
             <v>S-2026-01-53</v>
           </cell>
-          <cell r="B56"/>
           <cell r="C56" t="str">
             <v>RPRO-260120-0355</v>
           </cell>
@@ -8060,7 +7978,6 @@
           <cell r="A57" t="str">
             <v>S-2026-01-54</v>
           </cell>
-          <cell r="B57"/>
           <cell r="C57" t="str">
             <v>RPRO-260120-0356</v>
           </cell>
@@ -8129,7 +8046,6 @@
           <cell r="A58" t="str">
             <v>S-2026-01-55</v>
           </cell>
-          <cell r="B58"/>
           <cell r="C58" t="str">
             <v>RPRO-260120-0357</v>
           </cell>
@@ -8198,7 +8114,6 @@
           <cell r="A59" t="str">
             <v>S-2026-01-56</v>
           </cell>
-          <cell r="B59"/>
           <cell r="C59" t="str">
             <v>RPRO-260120-0358</v>
           </cell>
@@ -8267,7 +8182,6 @@
           <cell r="A60" t="str">
             <v>S-2026-01-57</v>
           </cell>
-          <cell r="B60"/>
           <cell r="C60" t="str">
             <v>RPRO-260120-0359</v>
           </cell>
@@ -8336,7 +8250,6 @@
           <cell r="A61" t="str">
             <v>S-2026-01-58</v>
           </cell>
-          <cell r="B61"/>
           <cell r="C61" t="str">
             <v>RPRO-260120-0360</v>
           </cell>
@@ -8405,7 +8318,6 @@
           <cell r="A62" t="str">
             <v>S-2026-01-59</v>
           </cell>
-          <cell r="B62"/>
           <cell r="C62" t="str">
             <v>RPRO-260116-0276</v>
           </cell>
@@ -8474,7 +8386,6 @@
           <cell r="A63" t="str">
             <v>S-2026-01-60</v>
           </cell>
-          <cell r="B63"/>
           <cell r="C63" t="str">
             <v>RPRO-260115-0310</v>
           </cell>
@@ -8543,7 +8454,6 @@
           <cell r="A64" t="str">
             <v>S-2026-01-61</v>
           </cell>
-          <cell r="B64"/>
           <cell r="C64" t="str">
             <v>RPRO-260120-0361</v>
           </cell>
@@ -8683,7 +8593,6 @@
           <cell r="A66" t="str">
             <v>S-2026-01-63</v>
           </cell>
-          <cell r="B66"/>
           <cell r="C66" t="str">
             <v>RPRO-260122-1562</v>
           </cell>
@@ -8752,7 +8661,6 @@
           <cell r="A67" t="str">
             <v>S-2026-01-64</v>
           </cell>
-          <cell r="B67"/>
           <cell r="C67" t="str">
             <v>RPRO-260122-1563</v>
           </cell>
@@ -8821,7 +8729,6 @@
           <cell r="A68" t="str">
             <v>S-2026-01-65</v>
           </cell>
-          <cell r="B68"/>
           <cell r="C68" t="str">
             <v>RPRO-260122-1564</v>
           </cell>
@@ -8890,7 +8797,6 @@
           <cell r="A69" t="str">
             <v>S-2026-01-66</v>
           </cell>
-          <cell r="B69"/>
           <cell r="C69" t="str">
             <v>RPRO-260122-1565</v>
           </cell>
@@ -8959,7 +8865,6 @@
           <cell r="A70" t="str">
             <v>S-2026-01-67</v>
           </cell>
-          <cell r="B70"/>
           <cell r="C70" t="str">
             <v>RPRO-260122-1566</v>
           </cell>
@@ -9028,7 +8933,6 @@
           <cell r="A71" t="str">
             <v>S-2026-01-68</v>
           </cell>
-          <cell r="B71"/>
           <cell r="C71" t="str">
             <v>RPRO-260122-1567</v>
           </cell>
@@ -9097,7 +9001,6 @@
           <cell r="A72" t="str">
             <v>S-2026-01-69</v>
           </cell>
-          <cell r="B72"/>
           <cell r="C72" t="str">
             <v>RPRO-260122-1568</v>
           </cell>
@@ -9166,7 +9069,6 @@
           <cell r="A73" t="str">
             <v>S-2026-01-70</v>
           </cell>
-          <cell r="B73"/>
           <cell r="C73" t="str">
             <v>RPRO-260122-1569</v>
           </cell>
@@ -9235,7 +9137,6 @@
           <cell r="A74" t="str">
             <v>S-2026-01-71</v>
           </cell>
-          <cell r="B74"/>
           <cell r="C74" t="str">
             <v>RPRO-260122-1570</v>
           </cell>
@@ -9304,7 +9205,6 @@
           <cell r="A75" t="str">
             <v>S-2026-01-72</v>
           </cell>
-          <cell r="B75"/>
           <cell r="C75" t="str">
             <v>RPRO-260122-1571</v>
           </cell>
@@ -9586,7 +9486,6 @@
           <cell r="A79" t="str">
             <v>S-2026-01-76</v>
           </cell>
-          <cell r="B79"/>
           <cell r="C79" t="str">
             <v>RPRO-260122-1573</v>
           </cell>
@@ -9655,7 +9554,6 @@
           <cell r="A80" t="str">
             <v>S-2026-01-77</v>
           </cell>
-          <cell r="B80"/>
           <cell r="C80" t="str">
             <v>RPRO-260122-1574</v>
           </cell>
@@ -9724,7 +9622,6 @@
           <cell r="A81" t="str">
             <v>S-2026-01-78</v>
           </cell>
-          <cell r="B81"/>
           <cell r="C81" t="str">
             <v>RPRO-260122-1575</v>
           </cell>
@@ -9793,7 +9690,6 @@
           <cell r="A82" t="str">
             <v>S-2026-01-79</v>
           </cell>
-          <cell r="B82"/>
           <cell r="C82" t="str">
             <v>RPRO-260122-1576</v>
           </cell>
@@ -9862,7 +9758,6 @@
           <cell r="A83" t="str">
             <v>S-2026-01-80</v>
           </cell>
-          <cell r="B83"/>
           <cell r="C83" t="str">
             <v>RPRO-260122-1577</v>
           </cell>
@@ -9931,7 +9826,6 @@
           <cell r="A84" t="str">
             <v>S-2026-01-81</v>
           </cell>
-          <cell r="B84"/>
           <cell r="C84" t="str">
             <v>RPRO-260122-1578</v>
           </cell>
@@ -10000,7 +9894,6 @@
           <cell r="A85" t="str">
             <v>S-2026-01-82</v>
           </cell>
-          <cell r="B85"/>
           <cell r="C85" t="str">
             <v>RPRO-260122-1579</v>
           </cell>
@@ -10069,7 +9962,6 @@
           <cell r="A86" t="str">
             <v>S-2026-01-83</v>
           </cell>
-          <cell r="B86"/>
           <cell r="C86" t="str">
             <v>RPRO-260122-1580</v>
           </cell>
@@ -10141,7 +10033,6 @@
           <cell r="B87" t="str">
             <v>hủy</v>
           </cell>
-          <cell r="C87"/>
           <cell r="D87" t="str">
             <v>OV-0385</v>
           </cell>
@@ -10210,7 +10101,6 @@
           <cell r="B88" t="str">
             <v>hủy</v>
           </cell>
-          <cell r="C88"/>
           <cell r="D88" t="str">
             <v>OV-0385</v>
           </cell>
@@ -10279,7 +10169,6 @@
           <cell r="B89" t="str">
             <v>hủy</v>
           </cell>
-          <cell r="C89"/>
           <cell r="D89" t="str">
             <v>OV-0385</v>
           </cell>
@@ -10345,7 +10234,6 @@
           <cell r="A90" t="str">
             <v>S-2026-01-87</v>
           </cell>
-          <cell r="B90"/>
           <cell r="C90" t="str">
             <v>RPRO-260127-0875</v>
           </cell>
@@ -10414,7 +10302,6 @@
           <cell r="A91" t="str">
             <v>S-2026-01-88</v>
           </cell>
-          <cell r="B91"/>
           <cell r="C91" t="str">
             <v>RPRO-260127-0877</v>
           </cell>
@@ -10483,7 +10370,6 @@
           <cell r="A92" t="str">
             <v>S-2026-01-89</v>
           </cell>
-          <cell r="B92"/>
           <cell r="C92" t="str">
             <v>RPRO-260127-0879</v>
           </cell>
@@ -10552,7 +10438,6 @@
           <cell r="A93" t="str">
             <v>S-2026-01-90</v>
           </cell>
-          <cell r="B93"/>
           <cell r="C93" t="str">
             <v>RPRO-260128-1270</v>
           </cell>
@@ -10621,7 +10506,6 @@
           <cell r="A94" t="str">
             <v>S-2026-01-91</v>
           </cell>
-          <cell r="B94"/>
           <cell r="C94" t="str">
             <v>RPRO-260128-1271</v>
           </cell>
@@ -10690,7 +10574,6 @@
           <cell r="A95" t="str">
             <v>S-2026-01-92</v>
           </cell>
-          <cell r="B95"/>
           <cell r="C95" t="str">
             <v>RPRO-260128-1272</v>
           </cell>
@@ -10759,7 +10642,6 @@
           <cell r="A96" t="str">
             <v>S-2026-01-93</v>
           </cell>
-          <cell r="B96"/>
           <cell r="C96" t="str">
             <v>RPRO-260128-1273</v>
           </cell>
@@ -10828,7 +10710,6 @@
           <cell r="A97" t="str">
             <v>S-2026-01-94</v>
           </cell>
-          <cell r="B97"/>
           <cell r="C97" t="str">
             <v>RPRO-260128-1274</v>
           </cell>
@@ -10897,7 +10778,6 @@
           <cell r="A98" t="str">
             <v>S-2026-01-95</v>
           </cell>
-          <cell r="B98"/>
           <cell r="C98" t="str">
             <v>RPRO-260128-1275</v>
           </cell>
@@ -10966,7 +10846,6 @@
           <cell r="A99" t="str">
             <v>S-2026-01-96</v>
           </cell>
-          <cell r="B99"/>
           <cell r="C99" t="str">
             <v>RPRO-260128-1276</v>
           </cell>
@@ -11035,7 +10914,6 @@
           <cell r="A100" t="str">
             <v>S-2026-01-97</v>
           </cell>
-          <cell r="B100"/>
           <cell r="C100" t="str">
             <v>RPRO-260128-1277</v>
           </cell>
@@ -11104,7 +10982,6 @@
           <cell r="A101" t="str">
             <v>S-2026-01-98</v>
           </cell>
-          <cell r="B101"/>
           <cell r="C101" t="str">
             <v>RPRO-260129-0656</v>
           </cell>
@@ -11173,7 +11050,6 @@
           <cell r="A102" t="str">
             <v>S-2026-02-01</v>
           </cell>
-          <cell r="B102"/>
           <cell r="C102" t="str">
             <v>RPRO-260203-0021</v>
           </cell>
@@ -11242,7 +11118,6 @@
           <cell r="A103" t="str">
             <v>S-2026-02-02</v>
           </cell>
-          <cell r="B103"/>
           <cell r="C103" t="str">
             <v>RPRO-260203-0022</v>
           </cell>
@@ -11311,7 +11186,6 @@
           <cell r="A104" t="str">
             <v>S-2026-02-03</v>
           </cell>
-          <cell r="B104"/>
           <cell r="C104" t="str">
             <v>RPRO-260203-0770</v>
           </cell>
@@ -11380,7 +11254,6 @@
           <cell r="A105" t="str">
             <v>S-2026-02-04</v>
           </cell>
-          <cell r="B105"/>
           <cell r="C105" t="str">
             <v>RPRO-260203-0771</v>
           </cell>
@@ -11449,7 +11322,6 @@
           <cell r="A106" t="str">
             <v>S-2026-02-05</v>
           </cell>
-          <cell r="B106"/>
           <cell r="C106" t="str">
             <v>RPRO-260203-0772</v>
           </cell>
@@ -11518,7 +11390,6 @@
           <cell r="A107" t="str">
             <v>S-2026-02-06</v>
           </cell>
-          <cell r="B107"/>
           <cell r="C107" t="str">
             <v>RPRO-260203-0773</v>
           </cell>
@@ -11587,7 +11458,6 @@
           <cell r="A108" t="str">
             <v>S-2026-02-07</v>
           </cell>
-          <cell r="B108"/>
           <cell r="C108" t="str">
             <v>RPRO-260203-0774</v>
           </cell>
@@ -11656,7 +11526,6 @@
           <cell r="A109" t="str">
             <v>S-2026-02-08</v>
           </cell>
-          <cell r="B109"/>
           <cell r="C109" t="str">
             <v>RPRO-260203-0775</v>
           </cell>
@@ -11725,7 +11594,6 @@
           <cell r="A110" t="str">
             <v>S-2026-02-09</v>
           </cell>
-          <cell r="B110"/>
           <cell r="C110" t="str">
             <v>RPRO-260203-0776</v>
           </cell>
@@ -11794,7 +11662,6 @@
           <cell r="A111" t="str">
             <v>S-2026-02-10</v>
           </cell>
-          <cell r="B111"/>
           <cell r="C111" t="str">
             <v>RPRO-260203-0777</v>
           </cell>
@@ -11863,7 +11730,6 @@
           <cell r="A112" t="str">
             <v>S-2026-02-11</v>
           </cell>
-          <cell r="B112"/>
           <cell r="C112" t="str">
             <v>RPRO-260203-0778</v>
           </cell>
@@ -11932,7 +11798,6 @@
           <cell r="A113" t="str">
             <v>S-2026-02-12</v>
           </cell>
-          <cell r="B113"/>
           <cell r="C113" t="str">
             <v>RPRO-260203-0779</v>
           </cell>
@@ -12001,7 +11866,6 @@
           <cell r="A114" t="str">
             <v>S-2026-02-13</v>
           </cell>
-          <cell r="B114"/>
           <cell r="C114" t="str">
             <v>RPRO-260203-0780</v>
           </cell>
@@ -12070,7 +11934,6 @@
           <cell r="A115" t="str">
             <v>S-2026-02-14</v>
           </cell>
-          <cell r="B115"/>
           <cell r="C115" t="str">
             <v>RPRO-260203-0781</v>
           </cell>
@@ -12139,7 +12002,6 @@
           <cell r="A116" t="str">
             <v>S-2026-02-15</v>
           </cell>
-          <cell r="B116"/>
           <cell r="C116" t="str">
             <v>RPRO-260203-0782</v>
           </cell>
@@ -12208,7 +12070,6 @@
           <cell r="A117" t="str">
             <v>S-2026-02-16</v>
           </cell>
-          <cell r="B117"/>
           <cell r="C117" t="str">
             <v>RPRO-260203-0783</v>
           </cell>
@@ -12277,7 +12138,6 @@
           <cell r="A118" t="str">
             <v>S-2026-02-17</v>
           </cell>
-          <cell r="B118"/>
           <cell r="C118" t="str">
             <v>RPRO-260203-0784</v>
           </cell>
@@ -12346,7 +12206,6 @@
           <cell r="A119" t="str">
             <v>S-2026-02-18</v>
           </cell>
-          <cell r="B119"/>
           <cell r="C119" t="str">
             <v>RPRO-260204-0399</v>
           </cell>
@@ -12415,7 +12274,6 @@
           <cell r="A120" t="str">
             <v>S-2026-02-19</v>
           </cell>
-          <cell r="B120"/>
           <cell r="C120" t="str">
             <v>RPRO-260204-0400</v>
           </cell>
@@ -12484,7 +12342,6 @@
           <cell r="A121" t="str">
             <v>L-2026-02-20</v>
           </cell>
-          <cell r="B121"/>
           <cell r="C121" t="str">
             <v>RPRO-260204-0401</v>
           </cell>
@@ -12518,7 +12375,6 @@
           <cell r="M121" t="str">
             <v>Lab test</v>
           </cell>
-          <cell r="N121"/>
           <cell r="O121" t="str">
             <v>Lab test</v>
           </cell>
@@ -12551,7 +12407,6 @@
           <cell r="A122" t="str">
             <v>L-2026-02-21</v>
           </cell>
-          <cell r="B122"/>
           <cell r="C122" t="str">
             <v>RPRO-260204-0402</v>
           </cell>
@@ -12585,7 +12440,6 @@
           <cell r="M122" t="str">
             <v>Lab test</v>
           </cell>
-          <cell r="N122"/>
           <cell r="O122" t="str">
             <v>Lab test</v>
           </cell>
@@ -12689,7 +12543,6 @@
           <cell r="A124" t="str">
             <v>S-2026-02-23</v>
           </cell>
-          <cell r="B124"/>
           <cell r="C124" t="str">
             <v>RPRO-260210-0003</v>
           </cell>
@@ -12829,7 +12682,6 @@
           <cell r="A126" t="str">
             <v>S-2026-02-25</v>
           </cell>
-          <cell r="B126"/>
           <cell r="C126" t="str">
             <v>RPRO-260210-0005</v>
           </cell>
@@ -12898,7 +12750,6 @@
           <cell r="A127" t="str">
             <v>S-2026-02-26</v>
           </cell>
-          <cell r="B127"/>
           <cell r="C127" t="str">
             <v>RPRO-260210-0006</v>
           </cell>
@@ -12967,7 +12818,6 @@
           <cell r="A128" t="str">
             <v>S-2026-02-27</v>
           </cell>
-          <cell r="B128"/>
           <cell r="C128" t="str">
             <v>RPRO-260210-0007</v>
           </cell>
@@ -13036,7 +12886,6 @@
           <cell r="A129" t="str">
             <v>S-2026-02-28</v>
           </cell>
-          <cell r="B129"/>
           <cell r="C129" t="str">
             <v>RPRO-260210-0008</v>
           </cell>
@@ -13105,7 +12954,6 @@
           <cell r="A130" t="str">
             <v>S-2026-02-29</v>
           </cell>
-          <cell r="B130"/>
           <cell r="C130" t="str">
             <v>RPRO-260210-0009</v>
           </cell>
@@ -13174,7 +13022,6 @@
           <cell r="A131" t="str">
             <v>S-2026-02-30</v>
           </cell>
-          <cell r="B131"/>
           <cell r="C131" t="str">
             <v>RPRO-260210-0010</v>
           </cell>
@@ -13243,7 +13090,6 @@
           <cell r="A132" t="str">
             <v>S-2026-02-31</v>
           </cell>
-          <cell r="B132"/>
           <cell r="C132" t="str">
             <v>RPRO-260210-0011</v>
           </cell>
@@ -13313,7 +13159,6 @@
           <cell r="A133" t="str">
             <v>S-2026-02-32</v>
           </cell>
-          <cell r="B133"/>
           <cell r="C133" t="str">
             <v>RPRO-260210-0012</v>
           </cell>
@@ -13383,7 +13228,6 @@
           <cell r="A134" t="str">
             <v>S-2026-02-33</v>
           </cell>
-          <cell r="B134"/>
           <cell r="C134" t="str">
             <v>RPRO-260210-0013</v>
           </cell>
@@ -13452,7 +13296,6 @@
           <cell r="A135" t="str">
             <v>S-2026-02-34</v>
           </cell>
-          <cell r="B135"/>
           <cell r="C135" t="str">
             <v>RPRO-260211-0001</v>
           </cell>
@@ -13523,7 +13366,6 @@
           <cell r="A136" t="str">
             <v>S-2026-02-35</v>
           </cell>
-          <cell r="B136"/>
           <cell r="C136" t="str">
             <v>RPRO-260227-0335</v>
           </cell>
@@ -13592,7 +13434,6 @@
           <cell r="A137" t="str">
             <v>S-2026-02-36</v>
           </cell>
-          <cell r="B137"/>
           <cell r="C137" t="str">
             <v>RPRO-260227-0336</v>
           </cell>
@@ -13661,7 +13502,6 @@
           <cell r="A138" t="str">
             <v>S-2026-02-37</v>
           </cell>
-          <cell r="B138"/>
           <cell r="C138" t="str">
             <v>RPRO-260227-0337</v>
           </cell>
@@ -13730,7 +13570,6 @@
           <cell r="A139" t="str">
             <v>S-2026-02-38</v>
           </cell>
-          <cell r="B139"/>
           <cell r="C139" t="str">
             <v>RPRO-260227-0338</v>
           </cell>
@@ -13799,7 +13638,6 @@
           <cell r="A140" t="str">
             <v>S-2026-02-39</v>
           </cell>
-          <cell r="B140"/>
           <cell r="C140" t="str">
             <v>RPRO-260227-0339</v>
           </cell>
@@ -13868,7 +13706,6 @@
           <cell r="A141" t="str">
             <v>L-2026-02-40</v>
           </cell>
-          <cell r="B141"/>
           <cell r="C141" t="str">
             <v>RPRO-260227-0340</v>
           </cell>
@@ -13902,7 +13739,6 @@
           <cell r="M141" t="str">
             <v>Lab test</v>
           </cell>
-          <cell r="N141"/>
           <cell r="O141" t="str">
             <v>Lab test</v>
           </cell>
@@ -13935,7 +13771,6 @@
           <cell r="A142" t="str">
             <v>S-2026-02-41</v>
           </cell>
-          <cell r="B142"/>
           <cell r="C142" t="str">
             <v>RPRO-260227-0341</v>
           </cell>
@@ -14004,7 +13839,6 @@
           <cell r="A143" t="str">
             <v>S-2026-02-42</v>
           </cell>
-          <cell r="B143"/>
           <cell r="C143" t="str">
             <v>RPRO-260227-0342</v>
           </cell>
@@ -14073,7 +13907,6 @@
           <cell r="A144" t="str">
             <v>S-2026-02-43</v>
           </cell>
-          <cell r="B144"/>
           <cell r="C144" t="str">
             <v>RPRO-260227-0343</v>
           </cell>
@@ -14142,7 +13975,6 @@
           <cell r="A145" t="str">
             <v>S-2026-02-44</v>
           </cell>
-          <cell r="B145"/>
           <cell r="C145" t="str">
             <v>RPRO-260227-0344</v>
           </cell>
@@ -14211,7 +14043,6 @@
           <cell r="A146" t="str">
             <v>S-2026-02-45</v>
           </cell>
-          <cell r="B146"/>
           <cell r="C146" t="str">
             <v>RPRO-260227-0345</v>
           </cell>
@@ -14351,7 +14182,6 @@
           <cell r="A148" t="str">
             <v>S-2026-02-47</v>
           </cell>
-          <cell r="B148"/>
           <cell r="C148" t="str">
             <v>RPRO-260227-0347</v>
           </cell>
@@ -14420,7 +14250,6 @@
           <cell r="A149" t="str">
             <v>S-2026-02-48</v>
           </cell>
-          <cell r="B149"/>
           <cell r="C149" t="str">
             <v>RPRO-260227-0348</v>
           </cell>
@@ -14489,7 +14318,6 @@
           <cell r="A150" t="str">
             <v>S-2026-02-49</v>
           </cell>
-          <cell r="B150"/>
           <cell r="C150" t="str">
             <v>RPRO-260302-0004</v>
           </cell>
@@ -14558,7 +14386,6 @@
           <cell r="A151" t="str">
             <v>S-2026-02-50</v>
           </cell>
-          <cell r="B151"/>
           <cell r="C151" t="str">
             <v>RPRO-260227-0349</v>
           </cell>
@@ -14627,7 +14454,6 @@
           <cell r="A152" t="str">
             <v>S-2026-02-51</v>
           </cell>
-          <cell r="B152"/>
           <cell r="C152" t="str">
             <v>RPRO-260227-0350</v>
           </cell>
@@ -14696,7 +14522,6 @@
           <cell r="A153" t="str">
             <v>S-2026-02-52</v>
           </cell>
-          <cell r="B153"/>
           <cell r="C153" t="str">
             <v>RPRO-260227-0351</v>
           </cell>
@@ -14765,7 +14590,6 @@
           <cell r="A154" t="str">
             <v>S-2026-02-53</v>
           </cell>
-          <cell r="B154"/>
           <cell r="C154" t="str">
             <v>RPRO-260227-0352</v>
           </cell>
@@ -14834,7 +14658,6 @@
           <cell r="A155" t="str">
             <v>L-2026-03-01</v>
           </cell>
-          <cell r="B155"/>
           <cell r="C155" t="str">
             <v>RPRO-260303-0005</v>
           </cell>
@@ -14868,7 +14691,6 @@
           <cell r="M155" t="str">
             <v xml:space="preserve">Lab test </v>
           </cell>
-          <cell r="N155"/>
           <cell r="O155" t="str">
             <v>Lab test</v>
           </cell>
@@ -14901,7 +14723,6 @@
           <cell r="A156" t="str">
             <v>L-2026-03-02</v>
           </cell>
-          <cell r="B156"/>
           <cell r="C156" t="str">
             <v>RPRO-260303-0006</v>
           </cell>
@@ -14935,7 +14756,6 @@
           <cell r="M156" t="str">
             <v xml:space="preserve">Lab test </v>
           </cell>
-          <cell r="N156"/>
           <cell r="O156" t="str">
             <v>Lab test</v>
           </cell>
@@ -15252,7 +15072,6 @@
           <cell r="A161" t="str">
             <v>S-2026-03-07</v>
           </cell>
-          <cell r="B161"/>
           <cell r="C161" t="str">
             <v>RPRO-260303-0011</v>
           </cell>
@@ -15321,7 +15140,6 @@
           <cell r="A162" t="str">
             <v>S-2026-03-08</v>
           </cell>
-          <cell r="B162"/>
           <cell r="C162" t="str">
             <v>RPRO-260303-0012</v>
           </cell>
@@ -15390,7 +15208,6 @@
           <cell r="A163" t="str">
             <v>S-2026-03-09</v>
           </cell>
-          <cell r="B163"/>
           <cell r="C163" t="str">
             <v>RPRO-260303-0013</v>
           </cell>
@@ -15459,7 +15276,6 @@
           <cell r="A164" t="str">
             <v>S-2026-03-10</v>
           </cell>
-          <cell r="B164"/>
           <cell r="C164" t="str">
             <v>RPRO-260303-0014</v>
           </cell>
@@ -15528,7 +15344,6 @@
           <cell r="A165" t="str">
             <v>S-2026-03-11</v>
           </cell>
-          <cell r="B165"/>
           <cell r="C165" t="str">
             <v>RPRO-260313-0139</v>
           </cell>
@@ -15562,7 +15377,6 @@
           <cell r="M165" t="str">
             <v>INSOLE/ MOLDED/ FLAT SHEET or DIE CUT</v>
           </cell>
-          <cell r="N165"/>
           <cell r="O165" t="str">
             <v>Sample</v>
           </cell>
@@ -15595,7 +15409,6 @@
           <cell r="A166" t="str">
             <v>S-2026-03-12</v>
           </cell>
-          <cell r="B166"/>
           <cell r="C166" t="str">
             <v>RPRO-260313-0140</v>
           </cell>
@@ -15629,7 +15442,6 @@
           <cell r="M166" t="str">
             <v>INSOLE/ MOLDED/ FLAT SHEET or DIE CUT</v>
           </cell>
-          <cell r="N166"/>
           <cell r="O166" t="str">
             <v>Sample</v>
           </cell>
@@ -15662,7 +15474,6 @@
           <cell r="A167" t="str">
             <v>S-2026-03-13</v>
           </cell>
-          <cell r="B167"/>
           <cell r="C167" t="str">
             <v>RPRO-260313-0141</v>
           </cell>
@@ -15696,7 +15507,6 @@
           <cell r="M167" t="str">
             <v>INSOLE/ MOLDED/ FLAT SHEET or DIE CUT</v>
           </cell>
-          <cell r="N167"/>
           <cell r="O167" t="str">
             <v>Sample</v>
           </cell>
@@ -15800,7 +15610,6 @@
           <cell r="A169" t="str">
             <v>S-2026-03-15</v>
           </cell>
-          <cell r="B169"/>
           <cell r="C169" t="str">
             <v>RPRO-260306-1547</v>
           </cell>
@@ -15869,7 +15678,6 @@
           <cell r="A170" t="str">
             <v>S-2026-03-16</v>
           </cell>
-          <cell r="B170"/>
           <cell r="C170" t="str">
             <v>RPRO-260306-1548</v>
           </cell>
@@ -15938,7 +15746,6 @@
           <cell r="A171" t="str">
             <v>S-2026-03-17</v>
           </cell>
-          <cell r="B171"/>
           <cell r="C171" t="str">
             <v>RPRO-260306-1549</v>
           </cell>
@@ -16007,7 +15814,6 @@
           <cell r="A172" t="str">
             <v>S-2026-03-18</v>
           </cell>
-          <cell r="B172"/>
           <cell r="C172" t="str">
             <v>RPRO-260306-1550</v>
           </cell>
@@ -16076,7 +15882,6 @@
           <cell r="A173" t="str">
             <v>S-2026-03-19</v>
           </cell>
-          <cell r="B173"/>
           <cell r="C173" t="str">
             <v>RPRO-260306-1551</v>
           </cell>
@@ -16145,7 +15950,6 @@
           <cell r="A174" t="str">
             <v>S-2026-03-20</v>
           </cell>
-          <cell r="B174"/>
           <cell r="C174" t="str">
             <v>RPRO-260306-1552</v>
           </cell>
@@ -16214,7 +16018,6 @@
           <cell r="A175" t="str">
             <v>S-2026-03-21</v>
           </cell>
-          <cell r="B175"/>
           <cell r="C175" t="str">
             <v>RPRO-260306-1553</v>
           </cell>
@@ -16283,7 +16086,6 @@
           <cell r="A176" t="str">
             <v>S-2026-03-22</v>
           </cell>
-          <cell r="B176"/>
           <cell r="C176" t="str">
             <v>RPRO-260306-1554</v>
           </cell>
@@ -16352,7 +16154,6 @@
           <cell r="A177" t="str">
             <v>S-2026-03-23</v>
           </cell>
-          <cell r="B177"/>
           <cell r="C177" t="str">
             <v>RPRO-260306-1555</v>
           </cell>
@@ -16421,7 +16222,6 @@
           <cell r="A178" t="str">
             <v>S-2026-03-24</v>
           </cell>
-          <cell r="B178"/>
           <cell r="C178" t="str">
             <v>RPRO-260306-1556</v>
           </cell>
@@ -16561,7 +16361,6 @@
           <cell r="A180" t="str">
             <v>L-2026-03-26</v>
           </cell>
-          <cell r="B180"/>
           <cell r="C180" t="str">
             <v>RPRO-260305-1288</v>
           </cell>
@@ -16595,7 +16394,6 @@
           <cell r="M180" t="str">
             <v xml:space="preserve">Lab test </v>
           </cell>
-          <cell r="N180"/>
           <cell r="O180" t="str">
             <v>Lab test</v>
           </cell>
@@ -16699,7 +16497,6 @@
           <cell r="A182" t="str">
             <v>S-2026-03-28</v>
           </cell>
-          <cell r="B182"/>
           <cell r="C182" t="str">
             <v>RPRO-260306-1559</v>
           </cell>
@@ -16768,7 +16565,6 @@
           <cell r="A183" t="str">
             <v>S-2026-03-29</v>
           </cell>
-          <cell r="B183"/>
           <cell r="C183" t="str">
             <v>RPRO-260306-1560</v>
           </cell>
@@ -16837,7 +16633,6 @@
           <cell r="A184" t="str">
             <v>S-2026-03-30</v>
           </cell>
-          <cell r="B184"/>
           <cell r="C184" t="str">
             <v>RPRO-260306-1561</v>
           </cell>
@@ -16906,7 +16701,6 @@
           <cell r="A185" t="str">
             <v>S-2026-03-31</v>
           </cell>
-          <cell r="B185"/>
           <cell r="C185" t="str">
             <v>RPRO-260306-1562</v>
           </cell>
@@ -16975,7 +16769,6 @@
           <cell r="A186" t="str">
             <v>S-2026-03-32</v>
           </cell>
-          <cell r="B186"/>
           <cell r="C186" t="str">
             <v>RPRO-260306-1563</v>
           </cell>
@@ -17044,7 +16837,6 @@
           <cell r="A187" t="str">
             <v>S-2026-03-33</v>
           </cell>
-          <cell r="B187"/>
           <cell r="C187" t="str">
             <v>RPRO-260306-1564</v>
           </cell>
@@ -17113,7 +16905,6 @@
           <cell r="A188" t="str">
             <v>S-2026-03-34</v>
           </cell>
-          <cell r="B188"/>
           <cell r="C188" t="str">
             <v>RPRO-260306-1565</v>
           </cell>
@@ -17182,7 +16973,6 @@
           <cell r="A189" t="str">
             <v>S-2026-03-35</v>
           </cell>
-          <cell r="B189"/>
           <cell r="C189" t="str">
             <v>RPRO-260306-1566</v>
           </cell>
@@ -17251,7 +17041,6 @@
           <cell r="A190" t="str">
             <v>S-2026-03-36</v>
           </cell>
-          <cell r="B190"/>
           <cell r="C190" t="str">
             <v>RPRO-260307-0080</v>
           </cell>
@@ -17320,7 +17109,6 @@
           <cell r="A191" t="str">
             <v>S-2026-03-37</v>
           </cell>
-          <cell r="B191"/>
           <cell r="C191" t="str">
             <v>RPRO-260306-1736</v>
           </cell>
@@ -17389,7 +17177,6 @@
           <cell r="A192" t="str">
             <v>S-2026-03-38</v>
           </cell>
-          <cell r="B192"/>
           <cell r="C192" t="str">
             <v>RPRO-260306-1737</v>
           </cell>
@@ -17458,7 +17245,6 @@
           <cell r="A193" t="str">
             <v>S-2026-03-39</v>
           </cell>
-          <cell r="B193"/>
           <cell r="C193" t="str">
             <v>RPRO-260306-1738</v>
           </cell>
@@ -17527,7 +17313,6 @@
           <cell r="A194" t="str">
             <v>S-2026-03-40</v>
           </cell>
-          <cell r="B194"/>
           <cell r="C194" t="str">
             <v>RPRO-260306-1739</v>
           </cell>
@@ -17596,7 +17381,6 @@
           <cell r="A195" t="str">
             <v>S-2026-03-41</v>
           </cell>
-          <cell r="B195"/>
           <cell r="C195" t="str">
             <v>RPRO-260306-1740</v>
           </cell>
@@ -17665,7 +17449,6 @@
           <cell r="A196" t="str">
             <v>S-2026-03-42</v>
           </cell>
-          <cell r="B196"/>
           <cell r="C196" t="str">
             <v>RPRO-260307-0081</v>
           </cell>
@@ -17734,7 +17517,6 @@
           <cell r="A197" t="str">
             <v>S-2026-03-43</v>
           </cell>
-          <cell r="B197"/>
           <cell r="C197" t="str">
             <v>RPRO-260307-0082</v>
           </cell>
@@ -17803,7 +17585,6 @@
           <cell r="A198" t="str">
             <v>S-2026-03-44</v>
           </cell>
-          <cell r="B198"/>
           <cell r="C198" t="str">
             <v>RPRO-260307-0083</v>
           </cell>
@@ -17872,7 +17653,6 @@
           <cell r="A199" t="str">
             <v>S-2026-03-45</v>
           </cell>
-          <cell r="B199"/>
           <cell r="C199" t="str">
             <v>RPRO-260307-0084</v>
           </cell>
@@ -17941,7 +17721,6 @@
           <cell r="A200" t="str">
             <v>S-2026-03-46</v>
           </cell>
-          <cell r="B200"/>
           <cell r="C200" t="str">
             <v>RPRO-260307-0085</v>
           </cell>
@@ -18010,7 +17789,6 @@
           <cell r="A201" t="str">
             <v>S-2026-03-47</v>
           </cell>
-          <cell r="B201"/>
           <cell r="C201" t="str">
             <v>RPRO-260310-0362</v>
           </cell>
@@ -18150,7 +17928,6 @@
           <cell r="A203" t="str">
             <v>S-2026-03-49</v>
           </cell>
-          <cell r="B203"/>
           <cell r="C203" t="str">
             <v>RPRO-260310-0364</v>
           </cell>
@@ -18219,7 +17996,6 @@
           <cell r="A204" t="str">
             <v>S-2026-03-50</v>
           </cell>
-          <cell r="B204"/>
           <cell r="C204" t="str">
             <v>RPRO-260310-0365</v>
           </cell>
@@ -18359,7 +18135,6 @@
           <cell r="A206" t="str">
             <v>S-2026-03-52</v>
           </cell>
-          <cell r="B206"/>
           <cell r="C206" t="str">
             <v>RPRO-260310-0367</v>
           </cell>
@@ -18428,7 +18203,6 @@
           <cell r="A207" t="str">
             <v>S-2026-03-53</v>
           </cell>
-          <cell r="B207"/>
           <cell r="C207" t="str">
             <v>RPRO-260310-0368</v>
           </cell>
@@ -18497,7 +18271,6 @@
           <cell r="A208" t="str">
             <v>S-2026-03-54</v>
           </cell>
-          <cell r="B208"/>
           <cell r="C208" t="str">
             <v>RPRO-260310-0369</v>
           </cell>
@@ -18566,7 +18339,6 @@
           <cell r="A209" t="str">
             <v>S-2026-03-55</v>
           </cell>
-          <cell r="B209"/>
           <cell r="C209" t="str">
             <v>RPRO-260310-0370</v>
           </cell>
@@ -18635,7 +18407,6 @@
           <cell r="A210" t="str">
             <v>S-2026-03-56</v>
           </cell>
-          <cell r="B210"/>
           <cell r="C210" t="str">
             <v>RPRO-260310-0371</v>
           </cell>
@@ -18704,7 +18475,6 @@
           <cell r="A211" t="str">
             <v>S-2026-03-57</v>
           </cell>
-          <cell r="B211"/>
           <cell r="C211" t="str">
             <v>RPRO-260310-0372</v>
           </cell>
@@ -18773,7 +18543,6 @@
           <cell r="A212" t="str">
             <v>S-2026-03-58</v>
           </cell>
-          <cell r="B212"/>
           <cell r="C212" t="str">
             <v>RPRO-260310-0373</v>
           </cell>
@@ -18842,7 +18611,6 @@
           <cell r="A213" t="str">
             <v>S-2026-03-59</v>
           </cell>
-          <cell r="B213"/>
           <cell r="C213" t="str">
             <v>RPRO-260310-0374</v>
           </cell>
@@ -18911,7 +18679,6 @@
           <cell r="A214" t="str">
             <v>S-2026-03-60</v>
           </cell>
-          <cell r="B214"/>
           <cell r="C214" t="str">
             <v>RPRO-260310-0375</v>
           </cell>
@@ -18980,7 +18747,6 @@
           <cell r="A215" t="str">
             <v>S-2026-03-61</v>
           </cell>
-          <cell r="B215"/>
           <cell r="C215" t="str">
             <v>RPRO-260310-0376</v>
           </cell>
@@ -19052,7 +18818,6 @@
           <cell r="B216" t="str">
             <v>huy</v>
           </cell>
-          <cell r="C216"/>
           <cell r="D216" t="str">
             <v>ly.vtc@ortholite.vn</v>
           </cell>
@@ -19083,7 +18848,6 @@
           <cell r="M216" t="str">
             <v xml:space="preserve">Lab test </v>
           </cell>
-          <cell r="N216"/>
           <cell r="O216" t="str">
             <v>Lab test</v>
           </cell>
@@ -19119,7 +18883,6 @@
           <cell r="B217" t="str">
             <v>huy</v>
           </cell>
-          <cell r="C217"/>
           <cell r="D217" t="str">
             <v>ly.vtc@ortholite.vn</v>
           </cell>
@@ -19150,7 +18913,6 @@
           <cell r="M217" t="str">
             <v xml:space="preserve">Lab test </v>
           </cell>
-          <cell r="N217"/>
           <cell r="O217" t="str">
             <v>Lab test</v>
           </cell>
@@ -19183,7 +18945,6 @@
           <cell r="A218" t="str">
             <v>S-2026-03-64</v>
           </cell>
-          <cell r="B218"/>
           <cell r="C218" t="str">
             <v>RPRO-260313-0142</v>
           </cell>
@@ -19252,7 +19013,6 @@
           <cell r="A219" t="str">
             <v>S-2026-03-65</v>
           </cell>
-          <cell r="B219"/>
           <cell r="C219" t="str">
             <v>RPRO-260313-0143</v>
           </cell>
@@ -19321,7 +19081,6 @@
           <cell r="A220" t="str">
             <v>S-2026-03-66</v>
           </cell>
-          <cell r="B220"/>
           <cell r="C220" t="str">
             <v>RPRO-260313-0144</v>
           </cell>
@@ -19390,7 +19149,6 @@
           <cell r="A221" t="str">
             <v>S-2026-03-67</v>
           </cell>
-          <cell r="B221"/>
           <cell r="C221" t="str">
             <v>RPRO-260313-0145</v>
           </cell>
@@ -19459,7 +19217,6 @@
           <cell r="A222" t="str">
             <v>S-2026-03-68</v>
           </cell>
-          <cell r="B222"/>
           <cell r="C222" t="str">
             <v>RPRO-260313-0146</v>
           </cell>
@@ -19528,7 +19285,6 @@
           <cell r="A223" t="str">
             <v>S-2026-03-69</v>
           </cell>
-          <cell r="B223"/>
           <cell r="C223" t="str">
             <v>RPRO-260313-0147</v>
           </cell>
@@ -19597,7 +19353,6 @@
           <cell r="A224" t="str">
             <v>S-2026-03-70</v>
           </cell>
-          <cell r="B224"/>
           <cell r="C224" t="str">
             <v>RPRO-260313-0148</v>
           </cell>
@@ -19666,7 +19421,6 @@
           <cell r="A225" t="str">
             <v>S-2026-03-71</v>
           </cell>
-          <cell r="B225"/>
           <cell r="C225" t="str">
             <v>RPRO-260313-0149</v>
           </cell>
@@ -19735,7 +19489,6 @@
           <cell r="A226" t="str">
             <v>S-2026-03-72</v>
           </cell>
-          <cell r="B226"/>
           <cell r="C226" t="str">
             <v>RPRO-260313-0150</v>
           </cell>
@@ -19804,7 +19557,6 @@
           <cell r="A227" t="str">
             <v>S-2026-03-73</v>
           </cell>
-          <cell r="B227"/>
           <cell r="C227" t="str">
             <v>RPRO-260313-0151</v>
           </cell>
@@ -19873,7 +19625,6 @@
           <cell r="A228" t="str">
             <v>S-2026-03-74</v>
           </cell>
-          <cell r="B228"/>
           <cell r="C228" t="str">
             <v>RPRO-260313-0152</v>
           </cell>
@@ -19942,7 +19693,6 @@
           <cell r="A229" t="str">
             <v>S-2026-03-75</v>
           </cell>
-          <cell r="B229"/>
           <cell r="C229" t="str">
             <v>RPRO-260313-0318</v>
           </cell>
@@ -20011,7 +19761,6 @@
           <cell r="A230" t="str">
             <v>S-2026-03-76</v>
           </cell>
-          <cell r="B230"/>
           <cell r="C230" t="str">
             <v>RPRO-260313-0319</v>
           </cell>
@@ -20080,7 +19829,6 @@
           <cell r="A231" t="str">
             <v>S-2026-03-77</v>
           </cell>
-          <cell r="B231"/>
           <cell r="C231" t="str">
             <v>RPRO-260314-0198</v>
           </cell>
@@ -20149,7 +19897,6 @@
           <cell r="A232" t="str">
             <v>S-2026-03-78</v>
           </cell>
-          <cell r="B232"/>
           <cell r="C232" t="str">
             <v>RPRO-260314-0199</v>
           </cell>
@@ -20218,7 +19965,6 @@
           <cell r="A233" t="str">
             <v>S-2026-03-79</v>
           </cell>
-          <cell r="B233"/>
           <cell r="C233" t="str">
             <v>RPRO-260317-0628</v>
           </cell>
@@ -20287,7 +20033,6 @@
           <cell r="A234" t="str">
             <v>S-2026-03-80</v>
           </cell>
-          <cell r="B234"/>
           <cell r="C234" t="str">
             <v>RPRO-260317-0629</v>
           </cell>
@@ -20356,7 +20101,6 @@
           <cell r="A235" t="str">
             <v>S-2026-03-81</v>
           </cell>
-          <cell r="B235"/>
           <cell r="C235" t="str">
             <v>RPRO-260317-0630</v>
           </cell>
@@ -20425,7 +20169,6 @@
           <cell r="A236" t="str">
             <v>S-2026-03-82</v>
           </cell>
-          <cell r="B236"/>
           <cell r="C236" t="str">
             <v>RPRO-260317-0631</v>
           </cell>
@@ -20494,7 +20237,6 @@
           <cell r="A237" t="str">
             <v>S-2026-03-83</v>
           </cell>
-          <cell r="B237"/>
           <cell r="C237" t="str">
             <v>RPRO-260317-0632</v>
           </cell>
@@ -20563,7 +20305,6 @@
           <cell r="A238" t="str">
             <v>S-2026-03-84</v>
           </cell>
-          <cell r="B238"/>
           <cell r="C238" t="str">
             <v>RPRO-260317-0633</v>
           </cell>
@@ -20632,7 +20373,6 @@
           <cell r="A239" t="str">
             <v>S-2026-03-85</v>
           </cell>
-          <cell r="B239"/>
           <cell r="C239" t="str">
             <v>RPRO-260317-0634</v>
           </cell>
@@ -20701,7 +20441,6 @@
           <cell r="A240" t="str">
             <v>S-2026-03-86</v>
           </cell>
-          <cell r="B240"/>
           <cell r="C240" t="str">
             <v>RPRO-260317-0635</v>
           </cell>
@@ -20770,7 +20509,6 @@
           <cell r="A241" t="str">
             <v>S-2026-03-87</v>
           </cell>
-          <cell r="B241"/>
           <cell r="C241" t="str">
             <v>RPRO-260317-0636</v>
           </cell>
@@ -20839,7 +20577,6 @@
           <cell r="A242" t="str">
             <v>L-2026-03-88</v>
           </cell>
-          <cell r="B242"/>
           <cell r="C242" t="str">
             <v>RPRO-260317-0637</v>
           </cell>
@@ -20873,7 +20610,6 @@
           <cell r="M242" t="str">
             <v xml:space="preserve">Lab test </v>
           </cell>
-          <cell r="N242"/>
           <cell r="O242" t="str">
             <v>Lab test</v>
           </cell>
@@ -20942,7 +20678,6 @@
           <cell r="M243" t="str">
             <v xml:space="preserve">Lab test </v>
           </cell>
-          <cell r="N243"/>
           <cell r="O243" t="str">
             <v>Lab test</v>
           </cell>
@@ -20975,7 +20710,6 @@
           <cell r="A244" t="str">
             <v>S-2026-03-90</v>
           </cell>
-          <cell r="B244"/>
           <cell r="C244" t="str">
             <v>RPRO-260317-0639</v>
           </cell>
@@ -21044,7 +20778,6 @@
           <cell r="A245" t="str">
             <v>S-2026-03-91</v>
           </cell>
-          <cell r="B245"/>
           <cell r="C245" t="str">
             <v>RPRO-260317-0640</v>
           </cell>
@@ -21113,7 +20846,6 @@
           <cell r="A246" t="str">
             <v>S-2026-03-92</v>
           </cell>
-          <cell r="B246"/>
           <cell r="C246" t="str">
             <v>RPRO-260317-0641</v>
           </cell>
@@ -21182,7 +20914,6 @@
           <cell r="A247" t="str">
             <v>L-2026-03-93</v>
           </cell>
-          <cell r="B247"/>
           <cell r="C247" t="str">
             <v>RPRO-260318-0477</v>
           </cell>
@@ -21216,7 +20947,6 @@
           <cell r="M247" t="str">
             <v xml:space="preserve">Lab test </v>
           </cell>
-          <cell r="N247"/>
           <cell r="O247" t="str">
             <v>Lab test</v>
           </cell>
@@ -21249,7 +20979,6 @@
           <cell r="A248" t="str">
             <v>L-2026-03-94</v>
           </cell>
-          <cell r="B248"/>
           <cell r="C248" t="str">
             <v>RPRO-260318-0478</v>
           </cell>
@@ -21283,7 +21012,6 @@
           <cell r="M248" t="str">
             <v xml:space="preserve">Lab test </v>
           </cell>
-          <cell r="N248"/>
           <cell r="O248" t="str">
             <v>Lab test</v>
           </cell>
@@ -21387,7 +21115,6 @@
           <cell r="A250" t="str">
             <v>S-2026-03-96</v>
           </cell>
-          <cell r="B250"/>
           <cell r="C250" t="str">
             <v>RPRO-260318-0482</v>
           </cell>
@@ -21456,7 +21183,6 @@
           <cell r="A251" t="str">
             <v>S-2026-03-97</v>
           </cell>
-          <cell r="B251"/>
           <cell r="C251" t="str">
             <v>RPRO-260324-0278</v>
           </cell>
@@ -21525,7 +21251,6 @@
           <cell r="A252" t="str">
             <v>S-2026-03-98</v>
           </cell>
-          <cell r="B252"/>
           <cell r="C252" t="str">
             <v>RPRO-260324-0279</v>
           </cell>
@@ -21665,7 +21390,6 @@
           <cell r="A254" t="str">
             <v>S-2026-03-100</v>
           </cell>
-          <cell r="B254"/>
           <cell r="C254" t="str">
             <v>RPRO-260324-0281</v>
           </cell>
@@ -21734,7 +21458,6 @@
           <cell r="A255" t="str">
             <v>S-2026-03-101</v>
           </cell>
-          <cell r="B255"/>
           <cell r="C255" t="str">
             <v>RPRO-260324-0282</v>
           </cell>
@@ -21803,7 +21526,6 @@
           <cell r="A256" t="str">
             <v>S-2026-03-102</v>
           </cell>
-          <cell r="B256"/>
           <cell r="C256" t="str">
             <v>RPRO-260324-0531</v>
           </cell>
@@ -21872,7 +21594,6 @@
           <cell r="A257" t="str">
             <v>S-2026-03-103</v>
           </cell>
-          <cell r="B257"/>
           <cell r="C257" t="str">
             <v>RPRO-260324-0283</v>
           </cell>
@@ -21941,7 +21662,6 @@
           <cell r="A258" t="str">
             <v>S-2026-03-104</v>
           </cell>
-          <cell r="B258"/>
           <cell r="C258" t="str">
             <v>RPRO-260324-0284</v>
           </cell>
@@ -22010,7 +21730,6 @@
           <cell r="A259" t="str">
             <v>L-2026-03-105</v>
           </cell>
-          <cell r="B259"/>
           <cell r="C259" t="str">
             <v>RPRO-260321-0027</v>
           </cell>
@@ -22044,7 +21763,6 @@
           <cell r="M259" t="str">
             <v xml:space="preserve">Lab test </v>
           </cell>
-          <cell r="N259"/>
           <cell r="O259" t="str">
             <v>Lab test</v>
           </cell>
@@ -22077,7 +21795,6 @@
           <cell r="A260" t="str">
             <v>L-2026-03-106</v>
           </cell>
-          <cell r="B260"/>
           <cell r="C260" t="str">
             <v>RPRO-260321-0028</v>
           </cell>
@@ -22111,7 +21828,6 @@
           <cell r="M260" t="str">
             <v xml:space="preserve">Lab test </v>
           </cell>
-          <cell r="N260"/>
           <cell r="O260" t="str">
             <v>Lab test</v>
           </cell>
@@ -22144,7 +21860,6 @@
           <cell r="A261" t="str">
             <v>S-2026-03-107</v>
           </cell>
-          <cell r="B261"/>
           <cell r="C261" t="str">
             <v>RPRO-260321-0029</v>
           </cell>
@@ -22213,7 +21928,6 @@
           <cell r="A262" t="str">
             <v>S-2026-03-108</v>
           </cell>
-          <cell r="B262"/>
           <cell r="C262" t="str">
             <v>RPRO-260324-0285</v>
           </cell>
@@ -22282,7 +21996,6 @@
           <cell r="A263" t="str">
             <v>L-2026-03-109</v>
           </cell>
-          <cell r="B263"/>
           <cell r="C263" t="str">
             <v>RPRO-260324-0286</v>
           </cell>
@@ -22310,11 +22023,9 @@
           <cell r="K263">
             <v>0</v>
           </cell>
-          <cell r="L263"/>
           <cell r="M263" t="str">
             <v xml:space="preserve">Lab test </v>
           </cell>
-          <cell r="N263"/>
           <cell r="O263" t="str">
             <v>Lab test</v>
           </cell>
@@ -22347,7 +22058,6 @@
           <cell r="A264" t="str">
             <v>S-2026-03-110</v>
           </cell>
-          <cell r="B264"/>
           <cell r="C264" t="str">
             <v>RPRO-260324-0287</v>
           </cell>
@@ -22416,7 +22126,6 @@
           <cell r="A265" t="str">
             <v>S-2026-03-111</v>
           </cell>
-          <cell r="B265"/>
           <cell r="C265" t="str">
             <v>RPRO-260324-0288</v>
           </cell>
@@ -22485,7 +22194,6 @@
           <cell r="A266" t="str">
             <v>S-2026-03-112</v>
           </cell>
-          <cell r="B266"/>
           <cell r="C266" t="str">
             <v>RPRO-260324-0289</v>
           </cell>
@@ -22554,7 +22262,6 @@
           <cell r="A267" t="str">
             <v>S-2026-03-113</v>
           </cell>
-          <cell r="B267"/>
           <cell r="C267" t="str">
             <v>RPRO-260324-0532</v>
           </cell>
@@ -22623,7 +22330,6 @@
           <cell r="A268" t="str">
             <v>S-2026-03-114</v>
           </cell>
-          <cell r="B268"/>
           <cell r="C268" t="str">
             <v>RPRO-260324-0533</v>
           </cell>
@@ -22692,7 +22398,6 @@
           <cell r="A269" t="str">
             <v>S-2026-03-115</v>
           </cell>
-          <cell r="B269"/>
           <cell r="C269" t="str">
             <v>RPRO-260324-0534</v>
           </cell>
@@ -22761,7 +22466,6 @@
           <cell r="A270" t="str">
             <v>S-2026-03-116</v>
           </cell>
-          <cell r="B270"/>
           <cell r="C270" t="str">
             <v>RPRO-260325-0407</v>
           </cell>
@@ -22830,7 +22534,6 @@
           <cell r="A271" t="str">
             <v>S-2026-03-117</v>
           </cell>
-          <cell r="B271"/>
           <cell r="C271" t="str">
             <v>RPRO-260325-0408</v>
           </cell>
@@ -22899,7 +22602,6 @@
           <cell r="A272" t="str">
             <v>S-2026-03-118</v>
           </cell>
-          <cell r="B272"/>
           <cell r="C272" t="str">
             <v>RPRO-260325-0409</v>
           </cell>
@@ -22968,7 +22670,6 @@
           <cell r="A273" t="str">
             <v>S-2026-03-119</v>
           </cell>
-          <cell r="B273"/>
           <cell r="C273" t="str">
             <v>RPRO-260325-0410</v>
           </cell>
@@ -23037,7 +22738,6 @@
           <cell r="A274" t="str">
             <v>S-2026-03-120</v>
           </cell>
-          <cell r="B274"/>
           <cell r="C274" t="str">
             <v>RPRO-260325-0411</v>
           </cell>
@@ -23106,7 +22806,6 @@
           <cell r="A275" t="str">
             <v>S-2026-03-121</v>
           </cell>
-          <cell r="B275"/>
           <cell r="C275" t="str">
             <v>RPRO-260325-0412</v>
           </cell>
@@ -23175,7 +22874,6 @@
           <cell r="A276" t="str">
             <v>S-2026-03-122</v>
           </cell>
-          <cell r="B276"/>
           <cell r="C276" t="str">
             <v>RPRO-260325-0413</v>
           </cell>
@@ -23244,7 +22942,6 @@
           <cell r="A277" t="str">
             <v>S-2026-03-123</v>
           </cell>
-          <cell r="B277"/>
           <cell r="C277" t="str">
             <v>RPRO-260325-0414</v>
           </cell>
@@ -23313,7 +23010,6 @@
           <cell r="A278" t="str">
             <v>S-2026-03-124</v>
           </cell>
-          <cell r="B278"/>
           <cell r="C278" t="str">
             <v>RPRO-260325-0415</v>
           </cell>
@@ -23453,7 +23149,6 @@
           <cell r="A280" t="str">
             <v>S-2026-03-126</v>
           </cell>
-          <cell r="B280"/>
           <cell r="C280" t="str">
             <v>RPRO-260325-0417</v>
           </cell>
@@ -23522,7 +23217,6 @@
           <cell r="A281" t="str">
             <v>S-2026-03-127</v>
           </cell>
-          <cell r="B281"/>
           <cell r="C281" t="str">
             <v>RPRO-260325-0418</v>
           </cell>
@@ -23591,7 +23285,6 @@
           <cell r="A282" t="str">
             <v>S-2026-03-128</v>
           </cell>
-          <cell r="B282"/>
           <cell r="C282" t="str">
             <v>RPRO-260325-0419</v>
           </cell>
@@ -23660,7 +23353,6 @@
           <cell r="A283" t="str">
             <v>S-2026-03-129</v>
           </cell>
-          <cell r="B283"/>
           <cell r="C283" t="str">
             <v>RPRO-260325-0421</v>
           </cell>
@@ -23729,7 +23421,6 @@
           <cell r="A284" t="str">
             <v>S-2026-03-130</v>
           </cell>
-          <cell r="B284"/>
           <cell r="C284" t="str">
             <v>RPRO-260327-0930</v>
           </cell>
@@ -23940,7 +23631,6 @@
           <cell r="A287" t="str">
             <v>S-2026-03-133</v>
           </cell>
-          <cell r="B287"/>
           <cell r="C287" t="str">
             <v>RPRO-260327-0933</v>
           </cell>
@@ -24009,7 +23699,6 @@
           <cell r="A288" t="str">
             <v>S-2026-03-134</v>
           </cell>
-          <cell r="B288"/>
           <cell r="C288" t="str">
             <v>RPRO-260327-0934</v>
           </cell>
@@ -24220,7 +23909,6 @@
           <cell r="A291" t="str">
             <v>S-2026-03-137</v>
           </cell>
-          <cell r="B291"/>
           <cell r="C291" t="str">
             <v>RPRO-260327-0937</v>
           </cell>
@@ -24360,7 +24048,6 @@
           <cell r="A293" t="str">
             <v>S-2026-03-139</v>
           </cell>
-          <cell r="B293"/>
           <cell r="C293" t="str">
             <v>RPRO-260327-0939</v>
           </cell>
@@ -24500,7 +24187,6 @@
           <cell r="A295" t="str">
             <v>S-2026-03-141</v>
           </cell>
-          <cell r="B295"/>
           <cell r="C295" t="str">
             <v>RPRO-260327-0941</v>
           </cell>
@@ -24569,7 +24255,6 @@
           <cell r="A296" t="str">
             <v>S-2026-03-142</v>
           </cell>
-          <cell r="B296"/>
           <cell r="C296" t="str">
             <v>RPRO-260401-0245</v>
           </cell>
@@ -24709,7 +24394,6 @@
           <cell r="A298" t="str">
             <v>S-2026-03-144</v>
           </cell>
-          <cell r="B298"/>
           <cell r="C298" t="str">
             <v>RPRO-260401-0247</v>
           </cell>
@@ -24778,7 +24462,6 @@
           <cell r="A299" t="str">
             <v>S-2026-03-145</v>
           </cell>
-          <cell r="B299"/>
           <cell r="C299" t="str">
             <v>RPRO-260401-0248</v>
           </cell>
@@ -24847,7 +24530,6 @@
           <cell r="A300" t="str">
             <v>S-2026-03-146</v>
           </cell>
-          <cell r="B300"/>
           <cell r="C300" t="str">
             <v>RPRO-260401-0249</v>
           </cell>
@@ -24916,7 +24598,6 @@
           <cell r="A301" t="str">
             <v>S-2026-04-01</v>
           </cell>
-          <cell r="B301"/>
           <cell r="C301" t="str">
             <v>RPRO-260401-0250</v>
           </cell>
@@ -24985,7 +24666,6 @@
           <cell r="A302" t="str">
             <v>S-2026-04-02</v>
           </cell>
-          <cell r="B302"/>
           <cell r="C302" t="str">
             <v>RPRO-260401-0251</v>
           </cell>
@@ -25054,7 +24734,6 @@
           <cell r="A303" t="str">
             <v>S-2026-04-03</v>
           </cell>
-          <cell r="B303"/>
           <cell r="C303" t="str">
             <v>RPRO-260402-0737</v>
           </cell>
@@ -25123,7 +24802,6 @@
           <cell r="A304" t="str">
             <v>S-2026-04-04</v>
           </cell>
-          <cell r="B304"/>
           <cell r="C304" t="str">
             <v>RPRO-260402-0738</v>
           </cell>
@@ -25192,7 +24870,6 @@
           <cell r="A305" t="str">
             <v>S-2026-04-05</v>
           </cell>
-          <cell r="B305"/>
           <cell r="C305" t="str">
             <v>RPRO-260403-0489</v>
           </cell>
@@ -25261,7 +24938,6 @@
           <cell r="A306" t="str">
             <v>S-2026-04-06</v>
           </cell>
-          <cell r="B306"/>
           <cell r="C306" t="str">
             <v>RPRO-260403-0490</v>
           </cell>
@@ -25330,7 +25006,6 @@
           <cell r="A307" t="str">
             <v>S-2026-04-07</v>
           </cell>
-          <cell r="B307"/>
           <cell r="C307" t="str">
             <v>RPRO-260403-0491</v>
           </cell>
@@ -25399,7 +25074,6 @@
           <cell r="A308" t="str">
             <v>S-2026-04-08</v>
           </cell>
-          <cell r="B308"/>
           <cell r="C308" t="str">
             <v>RPRO-260403-0492</v>
           </cell>
@@ -25468,7 +25142,6 @@
           <cell r="A309" t="str">
             <v>S-2026-04-09</v>
           </cell>
-          <cell r="B309"/>
           <cell r="C309" t="str">
             <v>RPRO-260406-1201</v>
           </cell>
@@ -25537,7 +25210,6 @@
           <cell r="A310" t="str">
             <v>S-2026-04-10</v>
           </cell>
-          <cell r="B310"/>
           <cell r="C310" t="str">
             <v>RPRO-260406-1202</v>
           </cell>
@@ -25606,7 +25278,6 @@
           <cell r="A311" t="str">
             <v>S-2026-04-11</v>
           </cell>
-          <cell r="B311"/>
           <cell r="C311" t="str">
             <v>RPRO-260406-1203</v>
           </cell>
@@ -25675,7 +25346,6 @@
           <cell r="A312" t="str">
             <v>S-2026-04-12</v>
           </cell>
-          <cell r="B312"/>
           <cell r="C312" t="str">
             <v>RPRO-260407-0417</v>
           </cell>
@@ -25744,7 +25414,6 @@
           <cell r="A313" t="str">
             <v>S-2026-04-13</v>
           </cell>
-          <cell r="B313"/>
           <cell r="C313" t="str">
             <v>RPRO-260407-0418</v>
           </cell>
@@ -25813,7 +25482,6 @@
           <cell r="A314" t="str">
             <v>S-2026-04-14</v>
           </cell>
-          <cell r="B314"/>
           <cell r="C314" t="str">
             <v>RPRO-260407-0419</v>
           </cell>
@@ -25882,7 +25550,6 @@
           <cell r="A315" t="str">
             <v>S-2026-04-15</v>
           </cell>
-          <cell r="B315"/>
           <cell r="C315" t="str">
             <v>RPRO-260407-0420</v>
           </cell>
@@ -25951,7 +25618,6 @@
           <cell r="A316" t="str">
             <v>S-2026-04-16</v>
           </cell>
-          <cell r="B316"/>
           <cell r="C316" t="str">
             <v>RPRO-260409-0346</v>
           </cell>
@@ -26020,7 +25686,6 @@
           <cell r="A317" t="str">
             <v>S-2026-04-17</v>
           </cell>
-          <cell r="B317"/>
           <cell r="C317" t="str">
             <v>RPRO-260409-0347</v>
           </cell>
@@ -26089,7 +25754,6 @@
           <cell r="A318" t="str">
             <v>S-2026-04-18</v>
           </cell>
-          <cell r="B318"/>
           <cell r="C318" t="str">
             <v>RPRO-260409-0348</v>
           </cell>
@@ -26158,7 +25822,6 @@
           <cell r="A319" t="str">
             <v>S-2026-04-19</v>
           </cell>
-          <cell r="B319"/>
           <cell r="C319" t="str">
             <v>RPRO-260409-0349</v>
           </cell>
@@ -26227,7 +25890,6 @@
           <cell r="A320" t="str">
             <v>S-2026-04-20</v>
           </cell>
-          <cell r="B320"/>
           <cell r="C320" t="str">
             <v>RPRO-260409-0350</v>
           </cell>
@@ -26296,7 +25958,6 @@
           <cell r="A321" t="str">
             <v>L-2026-04-21</v>
           </cell>
-          <cell r="B321"/>
           <cell r="C321" t="str">
             <v>RPRO-260410-0280</v>
           </cell>
@@ -26330,7 +25991,6 @@
           <cell r="M321" t="str">
             <v xml:space="preserve">Lab test </v>
           </cell>
-          <cell r="N321"/>
           <cell r="O321" t="str">
             <v>Lab test</v>
           </cell>
@@ -26363,7 +26023,6 @@
           <cell r="A322" t="str">
             <v>L-2026-04-22</v>
           </cell>
-          <cell r="B322"/>
           <cell r="C322" t="str">
             <v>RPRO-260410-0281</v>
           </cell>
@@ -26397,7 +26056,6 @@
           <cell r="M322" t="str">
             <v xml:space="preserve">Lab test </v>
           </cell>
-          <cell r="N322"/>
           <cell r="O322" t="str">
             <v>Lab test</v>
           </cell>
@@ -26430,7 +26088,6 @@
           <cell r="A323" t="str">
             <v>S-2026-04-23</v>
           </cell>
-          <cell r="B323"/>
           <cell r="C323" t="str">
             <v>RPRO-260410-0282</v>
           </cell>
@@ -26499,7 +26156,6 @@
           <cell r="A324" t="str">
             <v>S-2026-04-24</v>
           </cell>
-          <cell r="B324"/>
           <cell r="C324" t="str">
             <v>RPRO-260410-0283</v>
           </cell>
@@ -26568,7 +26224,6 @@
           <cell r="A325" t="str">
             <v>S-2026-04-25</v>
           </cell>
-          <cell r="B325"/>
           <cell r="C325" t="str">
             <v>RPRO-260410-0284</v>
           </cell>
@@ -26637,7 +26292,6 @@
           <cell r="A326" t="str">
             <v>S-2026-04-26</v>
           </cell>
-          <cell r="B326"/>
           <cell r="C326" t="str">
             <v>RPRO-260410-0285</v>
           </cell>
@@ -26706,7 +26360,6 @@
           <cell r="A327" t="str">
             <v>S-2026-04-27</v>
           </cell>
-          <cell r="B327"/>
           <cell r="C327" t="str">
             <v>RPRO-260410-0286</v>
           </cell>
@@ -26775,7 +26428,6 @@
           <cell r="A328" t="str">
             <v>S-2026-04-28</v>
           </cell>
-          <cell r="B328"/>
           <cell r="C328" t="str">
             <v>RPRO-260410-0287</v>
           </cell>
@@ -26915,7 +26567,6 @@
           <cell r="A330" t="str">
             <v>S-2026-04-30</v>
           </cell>
-          <cell r="B330"/>
           <cell r="C330" t="str">
             <v>RPRO-260414-0202</v>
           </cell>
@@ -26984,7 +26635,6 @@
           <cell r="A331" t="str">
             <v>S-2026-04-31</v>
           </cell>
-          <cell r="B331"/>
           <cell r="C331" t="str">
             <v>RPRO-260414-0203</v>
           </cell>
@@ -27053,7 +26703,6 @@
           <cell r="A332" t="str">
             <v>S-2026-04-32</v>
           </cell>
-          <cell r="B332"/>
           <cell r="C332" t="str">
             <v>RPRO-260414-0204</v>
           </cell>
@@ -27122,7 +26771,6 @@
           <cell r="A333" t="str">
             <v>S-2026-04-33</v>
           </cell>
-          <cell r="B333"/>
           <cell r="C333" t="str">
             <v>RPRO-260414-0205</v>
           </cell>
@@ -27191,7 +26839,6 @@
           <cell r="A334" t="str">
             <v>S-2026-04-34</v>
           </cell>
-          <cell r="B334"/>
           <cell r="C334" t="str">
             <v>RPRO-260414-0206</v>
           </cell>
@@ -27260,7 +26907,6 @@
           <cell r="A335" t="str">
             <v>S-2026-04-35</v>
           </cell>
-          <cell r="B335"/>
           <cell r="C335" t="str">
             <v>RPRO-260414-0207</v>
           </cell>
@@ -27329,7 +26975,6 @@
           <cell r="A336" t="str">
             <v>S-2026-04-36</v>
           </cell>
-          <cell r="B336"/>
           <cell r="C336" t="str">
             <v>RPRO-260414-0208</v>
           </cell>
@@ -27398,7 +27043,6 @@
           <cell r="A337" t="str">
             <v>S-2026-04-37</v>
           </cell>
-          <cell r="B337"/>
           <cell r="C337" t="str">
             <v>RPRO-260414-0209</v>
           </cell>
@@ -27467,7 +27111,6 @@
           <cell r="A338" t="str">
             <v>S-2026-04-38</v>
           </cell>
-          <cell r="B338"/>
           <cell r="C338" t="str">
             <v>RPRO-260414-0210</v>
           </cell>
@@ -27536,7 +27179,6 @@
           <cell r="A339" t="str">
             <v>S-2026-04-39</v>
           </cell>
-          <cell r="B339"/>
           <cell r="C339" t="str">
             <v>RPRO-260414-0211</v>
           </cell>
@@ -27605,7 +27247,6 @@
           <cell r="A340" t="str">
             <v>S-2026-04-40</v>
           </cell>
-          <cell r="B340"/>
           <cell r="C340" t="str">
             <v>RPRO-260414-0212</v>
           </cell>
@@ -27710,7 +27351,6 @@
           <cell r="M341" t="str">
             <v xml:space="preserve">Lab test </v>
           </cell>
-          <cell r="N341"/>
           <cell r="O341" t="str">
             <v>Lab test</v>
           </cell>
@@ -27779,7 +27419,6 @@
           <cell r="M342" t="str">
             <v xml:space="preserve">Lab test </v>
           </cell>
-          <cell r="N342"/>
           <cell r="O342" t="str">
             <v>Lab test</v>
           </cell>
@@ -27812,7 +27451,6 @@
           <cell r="A343" t="str">
             <v>S-2026-04-43</v>
           </cell>
-          <cell r="B343"/>
           <cell r="C343" t="str">
             <v>RPRO-260417-0243</v>
           </cell>
@@ -27881,7 +27519,6 @@
           <cell r="A344" t="str">
             <v>S-2026-04-44</v>
           </cell>
-          <cell r="B344"/>
           <cell r="C344" t="str">
             <v>RPRO-260417-0244</v>
           </cell>
@@ -27950,7 +27587,6 @@
           <cell r="A345" t="str">
             <v>S-2026-04-45</v>
           </cell>
-          <cell r="B345"/>
           <cell r="C345" t="str">
             <v>RPRO-260417-0245</v>
           </cell>
@@ -28019,7 +27655,6 @@
           <cell r="A346" t="str">
             <v>S-2026-04-46</v>
           </cell>
-          <cell r="B346"/>
           <cell r="C346" t="str">
             <v>RPRO-260417-0246</v>
           </cell>
@@ -28088,7 +27723,6 @@
           <cell r="A347" t="str">
             <v>S-2026-04-47</v>
           </cell>
-          <cell r="B347"/>
           <cell r="C347" t="str">
             <v>RPRO-260417-0247</v>
           </cell>
@@ -28157,7 +27791,6 @@
           <cell r="A348" t="str">
             <v>S-2026-04-48</v>
           </cell>
-          <cell r="B348"/>
           <cell r="C348" t="str">
             <v>RPRO-260421-0623</v>
           </cell>
@@ -28226,7 +27859,6 @@
           <cell r="A349" t="str">
             <v>S-2026-04-49</v>
           </cell>
-          <cell r="B349"/>
           <cell r="C349" t="str">
             <v>RPRO-260421-0624</v>
           </cell>
@@ -28295,7 +27927,6 @@
           <cell r="A350" t="str">
             <v>S-2026-04-50</v>
           </cell>
-          <cell r="B350"/>
           <cell r="C350" t="str">
             <v>RPRO-260421-0625</v>
           </cell>
@@ -28364,7 +27995,6 @@
           <cell r="A351" t="str">
             <v>S-2026-04-51</v>
           </cell>
-          <cell r="B351"/>
           <cell r="C351" t="str">
             <v>RPRO-260421-0626</v>
           </cell>
@@ -28433,7 +28063,6 @@
           <cell r="A352" t="str">
             <v>S-2026-04-52</v>
           </cell>
-          <cell r="B352"/>
           <cell r="C352" t="str">
             <v>RPRO-260421-0627</v>
           </cell>
@@ -28502,7 +28131,6 @@
           <cell r="A353" t="str">
             <v>S-2026-04-53</v>
           </cell>
-          <cell r="B353"/>
           <cell r="C353" t="str">
             <v>RPRO-260421-0628</v>
           </cell>
@@ -28571,7 +28199,6 @@
           <cell r="A354" t="str">
             <v>S-2026-04-54</v>
           </cell>
-          <cell r="B354"/>
           <cell r="C354" t="str">
             <v>RPRO-260421-0629</v>
           </cell>
@@ -28640,7 +28267,6 @@
           <cell r="A355" t="str">
             <v>S-2026-04-55</v>
           </cell>
-          <cell r="B355"/>
           <cell r="C355" t="str">
             <v>RPRO-260421-0630</v>
           </cell>
@@ -28709,7 +28335,6 @@
           <cell r="A356" t="str">
             <v>S-2026-04-56</v>
           </cell>
-          <cell r="B356"/>
           <cell r="C356" t="str">
             <v>RPRO-260421-0631</v>
           </cell>
@@ -28778,7 +28403,6 @@
           <cell r="A357" t="str">
             <v>S-2026-04-57</v>
           </cell>
-          <cell r="B357"/>
           <cell r="C357" t="str">
             <v>RPRO-260421-0632</v>
           </cell>
@@ -28847,7 +28471,6 @@
           <cell r="A358" t="str">
             <v>S-2026-04-58</v>
           </cell>
-          <cell r="B358"/>
           <cell r="C358" t="str">
             <v>RPRO-260421-0633</v>
           </cell>
@@ -28916,7 +28539,6 @@
           <cell r="A359" t="str">
             <v>S-2026-04-59</v>
           </cell>
-          <cell r="B359"/>
           <cell r="C359" t="str">
             <v>RPRO-260422-0268</v>
           </cell>
@@ -28985,7 +28607,6 @@
           <cell r="A360" t="str">
             <v>S-2026-04-60</v>
           </cell>
-          <cell r="B360"/>
           <cell r="C360" t="str">
             <v>RPRO-260423-0486</v>
           </cell>
@@ -29054,7 +28675,6 @@
           <cell r="A361" t="str">
             <v>S-2026-04-61</v>
           </cell>
-          <cell r="B361"/>
           <cell r="C361" t="str">
             <v>RPRO-260423-0487</v>
           </cell>
@@ -29123,7 +28743,6 @@
           <cell r="A362" t="str">
             <v>S-2026-04-62</v>
           </cell>
-          <cell r="B362"/>
           <cell r="C362" t="str">
             <v>RPRO-260424-1197</v>
           </cell>
@@ -29192,7 +28811,6 @@
           <cell r="A363" t="str">
             <v>S-2026-04-63</v>
           </cell>
-          <cell r="B363"/>
           <cell r="C363" t="str">
             <v>RPRO-260424-1198</v>
           </cell>
@@ -29261,7 +28879,6 @@
           <cell r="A364" t="str">
             <v>S-2026-04-64</v>
           </cell>
-          <cell r="B364"/>
           <cell r="C364" t="str">
             <v>RPRO-260424-1199</v>
           </cell>
@@ -29330,7 +28947,6 @@
           <cell r="A365" t="str">
             <v>S-2026-04-65</v>
           </cell>
-          <cell r="B365"/>
           <cell r="C365" t="str">
             <v>RPRO-260424-1200</v>
           </cell>
@@ -29399,7 +29015,6 @@
           <cell r="A366" t="str">
             <v>S-2026-04-66</v>
           </cell>
-          <cell r="B366"/>
           <cell r="C366" t="str">
             <v>RPRO-260424-1201</v>
           </cell>
@@ -29539,7 +29154,6 @@
           <cell r="A368" t="str">
             <v>S-2026-04-68</v>
           </cell>
-          <cell r="B368"/>
           <cell r="C368" t="str">
             <v>RPRO-260424-1203</v>
           </cell>
@@ -29608,7 +29222,6 @@
           <cell r="A369" t="str">
             <v>S-2026-04-69</v>
           </cell>
-          <cell r="B369"/>
           <cell r="C369" t="str">
             <v>RPRO-260424-1204</v>
           </cell>
@@ -29677,7 +29290,6 @@
           <cell r="A370" t="str">
             <v>S-2026-04-70</v>
           </cell>
-          <cell r="B370"/>
           <cell r="C370" t="str">
             <v>RPRO-260424-1205</v>
           </cell>
@@ -29746,7 +29358,6 @@
           <cell r="A371" t="str">
             <v>S-2026-04-71</v>
           </cell>
-          <cell r="B371"/>
           <cell r="C371" t="str">
             <v>RPRO-260424-1206</v>
           </cell>
@@ -29815,7 +29426,6 @@
           <cell r="A372" t="str">
             <v>S-2026-04-72</v>
           </cell>
-          <cell r="B372"/>
           <cell r="C372" t="str">
             <v>RPRO-260428-0920</v>
           </cell>
@@ -29884,7 +29494,6 @@
           <cell r="A373" t="str">
             <v>S-2026-04-73</v>
           </cell>
-          <cell r="B373"/>
           <cell r="C373" t="str">
             <v>RPRO-260429-0109</v>
           </cell>
@@ -29953,7 +29562,6 @@
           <cell r="A374" t="str">
             <v>S-2026-04-74</v>
           </cell>
-          <cell r="B374"/>
           <cell r="C374" t="str">
             <v>RPRO-260429-0110</v>
           </cell>
@@ -30022,7 +29630,6 @@
           <cell r="A375" t="str">
             <v>S-2026-04-75</v>
           </cell>
-          <cell r="B375"/>
           <cell r="C375" t="str">
             <v>RPRO-260429-0126</v>
           </cell>
@@ -30091,7 +29698,6 @@
           <cell r="A376" t="str">
             <v>S-2026-04-76</v>
           </cell>
-          <cell r="B376"/>
           <cell r="C376" t="str">
             <v>RPRO-260429-0127</v>
           </cell>
@@ -30160,7 +29766,6 @@
           <cell r="A377" t="str">
             <v>S-2026-05-01</v>
           </cell>
-          <cell r="B377"/>
           <cell r="C377" t="str">
             <v>RPRO-260505-0654</v>
           </cell>
@@ -30300,7 +29905,6 @@
           <cell r="A379" t="str">
             <v>S-2026-05-03</v>
           </cell>
-          <cell r="B379"/>
           <cell r="C379" t="str">
             <v>RPRO-260505-0656</v>
           </cell>
@@ -30369,7 +29973,6 @@
           <cell r="A380" t="str">
             <v>S-2026-05-04</v>
           </cell>
-          <cell r="B380"/>
           <cell r="C380" t="str">
             <v>RPRO-260505-0657</v>
           </cell>
@@ -30438,7 +30041,6 @@
           <cell r="A381" t="str">
             <v>S-2026-05-05</v>
           </cell>
-          <cell r="B381"/>
           <cell r="C381" t="str">
             <v>RPRO-260505-0658</v>
           </cell>
@@ -30507,7 +30109,6 @@
           <cell r="A382" t="str">
             <v>S-2026-05-06</v>
           </cell>
-          <cell r="B382"/>
           <cell r="C382" t="str">
             <v>RPRO-260505-0659</v>
           </cell>
@@ -30576,7 +30177,6 @@
           <cell r="A383" t="str">
             <v>S-2026-05-07</v>
           </cell>
-          <cell r="B383"/>
           <cell r="C383" t="str">
             <v>RPRO-260505-0660</v>
           </cell>
@@ -30716,7 +30316,6 @@
           <cell r="A385" t="str">
             <v>S-2026-05-09</v>
           </cell>
-          <cell r="B385"/>
           <cell r="C385" t="str">
             <v>RPRO-260505-0662</v>
           </cell>
@@ -30785,7 +30384,6 @@
           <cell r="A386" t="str">
             <v>S-2026-05-10</v>
           </cell>
-          <cell r="B386"/>
           <cell r="C386" t="str">
             <v>RPRO-260505-0663</v>
           </cell>
@@ -30925,7 +30523,6 @@
           <cell r="A388" t="str">
             <v>S-2026-05-12</v>
           </cell>
-          <cell r="B388"/>
           <cell r="C388" t="str">
             <v>RPRO-260505-0802</v>
           </cell>
@@ -30994,7 +30591,6 @@
           <cell r="A389" t="str">
             <v>S-2026-05-13</v>
           </cell>
-          <cell r="B389"/>
           <cell r="C389" t="str">
             <v>RPRO-260505-0803</v>
           </cell>
@@ -31063,7 +30659,6 @@
           <cell r="A390" t="str">
             <v>S-2026-05-14</v>
           </cell>
-          <cell r="B390"/>
           <cell r="C390" t="str">
             <v>RPRO-260506-0394</v>
           </cell>
@@ -31132,7 +30727,6 @@
           <cell r="A391" t="str">
             <v>S-2026-05-15</v>
           </cell>
-          <cell r="B391"/>
           <cell r="C391" t="str">
             <v>RPRO-260506-0395</v>
           </cell>
@@ -31201,7 +30795,6 @@
           <cell r="A392" t="str">
             <v>S-2026-05-16</v>
           </cell>
-          <cell r="B392"/>
           <cell r="C392" t="str">
             <v>RPRO-260506-0396</v>
           </cell>
@@ -31270,7 +30863,6 @@
           <cell r="A393" t="str">
             <v>S-2026-05-17</v>
           </cell>
-          <cell r="B393"/>
           <cell r="C393" t="str">
             <v>RPRO-260506-0397</v>
           </cell>
@@ -31339,7 +30931,6 @@
           <cell r="A394" t="str">
             <v>S-2026-05-18</v>
           </cell>
-          <cell r="B394"/>
           <cell r="C394" t="str">
             <v>RPRO-260506-0415</v>
           </cell>
@@ -31408,7 +30999,6 @@
           <cell r="A395" t="str">
             <v>S-2026-05-19</v>
           </cell>
-          <cell r="B395"/>
           <cell r="C395" t="str">
             <v>RPRO-260508-0581</v>
           </cell>
@@ -31477,7 +31067,6 @@
           <cell r="A396" t="str">
             <v>S-2026-05-20</v>
           </cell>
-          <cell r="B396"/>
           <cell r="C396" t="str">
             <v>RPRO-260508-0582</v>
           </cell>
@@ -31546,7 +31135,6 @@
           <cell r="A397" t="str">
             <v>S-2026-05-21</v>
           </cell>
-          <cell r="B397"/>
           <cell r="C397" t="str">
             <v>RPRO-260508-0583</v>
           </cell>
@@ -31615,7 +31203,6 @@
           <cell r="A398" t="str">
             <v>S-2026-05-22</v>
           </cell>
-          <cell r="B398"/>
           <cell r="C398" t="str">
             <v>RPRO-260508-0584</v>
           </cell>
@@ -31684,7 +31271,6 @@
           <cell r="A399" t="str">
             <v>S-2026-05-23</v>
           </cell>
-          <cell r="B399"/>
           <cell r="C399" t="str">
             <v>RPRO-260508-0585</v>
           </cell>
@@ -31753,7 +31339,6 @@
           <cell r="A400" t="str">
             <v>S-2026-05-24</v>
           </cell>
-          <cell r="B400"/>
           <cell r="C400" t="str">
             <v>RPRO-260508-0586</v>
           </cell>
@@ -31822,7 +31407,6 @@
           <cell r="A401" t="str">
             <v>S-2026-05-25</v>
           </cell>
-          <cell r="B401"/>
           <cell r="C401" t="str">
             <v>RPRO-260508-0587</v>
           </cell>
@@ -31891,7 +31475,6 @@
           <cell r="A402" t="str">
             <v>S-2026-05-26</v>
           </cell>
-          <cell r="B402"/>
           <cell r="C402" t="str">
             <v>RPRO-260508-0588</v>
           </cell>
@@ -31960,7 +31543,6 @@
           <cell r="A403" t="str">
             <v>S-2026-05-27</v>
           </cell>
-          <cell r="B403"/>
           <cell r="C403" t="str">
             <v>RPRO-260512-0580</v>
           </cell>
@@ -31991,7 +31573,6 @@
           <cell r="L403" t="str">
             <v>TBS</v>
           </cell>
-          <cell r="M403"/>
           <cell r="N403" t="str">
             <v>INSOLE/ MOLDED</v>
           </cell>
@@ -32027,7 +31608,6 @@
           <cell r="A404" t="str">
             <v>S-2026-05-28</v>
           </cell>
-          <cell r="B404"/>
           <cell r="C404" t="str">
             <v>RPRO-260512-0581</v>
           </cell>
@@ -32058,7 +31638,6 @@
           <cell r="L404" t="str">
             <v>TBS</v>
           </cell>
-          <cell r="M404"/>
           <cell r="N404" t="str">
             <v>INSOLE/ MOLDED</v>
           </cell>
@@ -32094,7 +31673,6 @@
           <cell r="A405" t="str">
             <v>S-2026-05-29</v>
           </cell>
-          <cell r="B405"/>
           <cell r="C405" t="str">
             <v>RPRO-260512-0582</v>
           </cell>
@@ -32163,7 +31741,6 @@
           <cell r="A406" t="str">
             <v>S-2026-05-30</v>
           </cell>
-          <cell r="B406"/>
           <cell r="C406" t="str">
             <v>RPRO-260512-0583</v>
           </cell>
@@ -32232,7 +31809,6 @@
           <cell r="A407" t="str">
             <v>S-2026-05-31</v>
           </cell>
-          <cell r="B407"/>
           <cell r="C407" t="str">
             <v>RPRO-260513-0945</v>
           </cell>
@@ -32301,7 +31877,6 @@
           <cell r="A408" t="str">
             <v>S-2026-05-32</v>
           </cell>
-          <cell r="B408"/>
           <cell r="C408" t="str">
             <v>RPRO-260513-0946</v>
           </cell>
@@ -32370,7 +31945,6 @@
           <cell r="A409" t="str">
             <v>S-2026-05-33</v>
           </cell>
-          <cell r="B409"/>
           <cell r="C409" t="str">
             <v>RPRO-260513-0947</v>
           </cell>
@@ -32439,7 +32013,6 @@
           <cell r="A410" t="str">
             <v>S-2026-05-34</v>
           </cell>
-          <cell r="B410"/>
           <cell r="C410" t="str">
             <v>RPRO-260513-0948</v>
           </cell>
@@ -32579,7 +32152,6 @@
           <cell r="A412" t="str">
             <v>S-2026-05-36</v>
           </cell>
-          <cell r="B412"/>
           <cell r="C412" t="str">
             <v>RPRO-260513-0950</v>
           </cell>
@@ -32648,7 +32220,6 @@
           <cell r="A413" t="str">
             <v>S-2026-05-37</v>
           </cell>
-          <cell r="B413"/>
           <cell r="C413" t="str">
             <v>RPRO-260515-0272</v>
           </cell>
@@ -32717,7 +32288,6 @@
           <cell r="A414" t="str">
             <v>S-2026-05-38</v>
           </cell>
-          <cell r="B414"/>
           <cell r="C414" t="str">
             <v>RPRO-260515-0273</v>
           </cell>
@@ -32786,7 +32356,6 @@
           <cell r="A415" t="str">
             <v>S-2026-05-39</v>
           </cell>
-          <cell r="B415"/>
           <cell r="C415" t="str">
             <v>RPRO-260515-0274</v>
           </cell>
@@ -32855,7 +32424,6 @@
           <cell r="A416" t="str">
             <v>S-2026-05-40</v>
           </cell>
-          <cell r="B416"/>
           <cell r="C416" t="str">
             <v>RPRO-260515-0275</v>
           </cell>
@@ -32924,7 +32492,6 @@
           <cell r="A417" t="str">
             <v>S-2026-05-41</v>
           </cell>
-          <cell r="B417"/>
           <cell r="C417" t="str">
             <v>RPRO-260515-0276</v>
           </cell>
@@ -32993,7 +32560,6 @@
           <cell r="A418" t="str">
             <v>S-2026-05-42</v>
           </cell>
-          <cell r="B418"/>
           <cell r="C418" t="str">
             <v>RPRO-260515-0277</v>
           </cell>
@@ -33062,7 +32628,6 @@
           <cell r="A419" t="str">
             <v>S-2026-05-43</v>
           </cell>
-          <cell r="B419"/>
           <cell r="C419" t="str">
             <v>RPRO-260515-0278</v>
           </cell>
@@ -33131,7 +32696,6 @@
           <cell r="A420" t="str">
             <v>S-2026-05-44</v>
           </cell>
-          <cell r="B420"/>
           <cell r="C420" t="str">
             <v>RPRO-260515-0279</v>
           </cell>
@@ -33200,7 +32764,6 @@
           <cell r="A421" t="str">
             <v>S-2026-05-45</v>
           </cell>
-          <cell r="B421"/>
           <cell r="C421" t="str">
             <v>RPRO-260515-0280</v>
           </cell>
@@ -33269,7 +32832,6 @@
           <cell r="A422" t="str">
             <v>S-2026-05-46</v>
           </cell>
-          <cell r="B422"/>
           <cell r="C422" t="str">
             <v>RPRO-260518-0853</v>
           </cell>
@@ -33338,7 +32900,6 @@
           <cell r="A423" t="str">
             <v>S-2026-05-47</v>
           </cell>
-          <cell r="B423"/>
           <cell r="C423" t="str">
             <v>RPRO-260518-0854</v>
           </cell>
@@ -33407,7 +32968,6 @@
           <cell r="A424" t="str">
             <v>S-2026-05-48</v>
           </cell>
-          <cell r="B424"/>
           <cell r="C424" t="str">
             <v>RPRO-260518-0855</v>
           </cell>
@@ -33476,7 +33036,6 @@
           <cell r="A425" t="str">
             <v>S-2026-05-49</v>
           </cell>
-          <cell r="B425"/>
           <cell r="C425" t="str">
             <v>RPRO-260518-0856</v>
           </cell>
@@ -33758,7 +33317,6 @@
           <cell r="A429" t="str">
             <v>S-2026-05-53</v>
           </cell>
-          <cell r="B429"/>
           <cell r="C429" t="str">
             <v>RPRO-260518-0860</v>
           </cell>
@@ -33827,7 +33385,6 @@
           <cell r="A430" t="str">
             <v>S-2026-05-54</v>
           </cell>
-          <cell r="B430"/>
           <cell r="C430" t="str">
             <v>RPRO-260518-0861</v>
           </cell>
@@ -33896,7 +33453,6 @@
           <cell r="A431" t="str">
             <v>S-2026-05-55</v>
           </cell>
-          <cell r="B431"/>
           <cell r="C431" t="str">
             <v>RPRO-260518-0862</v>
           </cell>
@@ -33965,7 +33521,6 @@
           <cell r="A432" t="str">
             <v>S-2026-05-56</v>
           </cell>
-          <cell r="B432"/>
           <cell r="C432" t="str">
             <v>RPRO-260518-0863</v>
           </cell>
@@ -34034,7 +33589,6 @@
           <cell r="A433" t="str">
             <v>S-2026-05-57</v>
           </cell>
-          <cell r="B433"/>
           <cell r="C433" t="str">
             <v>RPRO-260518-0864</v>
           </cell>
@@ -34103,7 +33657,6 @@
           <cell r="A434" t="str">
             <v>S-2026-05-58</v>
           </cell>
-          <cell r="B434"/>
           <cell r="C434" t="str">
             <v>RPRO-260518-0865</v>
           </cell>
@@ -34172,7 +33725,6 @@
           <cell r="A435" t="str">
             <v>S-2026-05-59</v>
           </cell>
-          <cell r="B435"/>
           <cell r="C435" t="str">
             <v>RPRO-260518-0866</v>
           </cell>
@@ -34241,7 +33793,6 @@
           <cell r="A436" t="str">
             <v>S-2026-05-60</v>
           </cell>
-          <cell r="B436"/>
           <cell r="C436" t="str">
             <v>RPRO-260520-0192</v>
           </cell>
@@ -34310,7 +33861,6 @@
           <cell r="A437" t="str">
             <v>S-2026-05-61</v>
           </cell>
-          <cell r="B437"/>
           <cell r="C437" t="str">
             <v>RPRO-260520-0193</v>
           </cell>
@@ -34379,7 +33929,6 @@
           <cell r="A438" t="str">
             <v>S-2026-05-62</v>
           </cell>
-          <cell r="B438"/>
           <cell r="C438" t="str">
             <v>RPRO-260520-0194</v>
           </cell>
@@ -34448,7 +33997,6 @@
           <cell r="A439" t="str">
             <v>S-2026-05-63</v>
           </cell>
-          <cell r="B439"/>
           <cell r="C439" t="str">
             <v>RPRO-260520-0195</v>
           </cell>
@@ -34517,7 +34065,6 @@
           <cell r="A440" t="str">
             <v>S-2026-05-64</v>
           </cell>
-          <cell r="B440"/>
           <cell r="C440" t="str">
             <v>RPRO-260520-0196</v>
           </cell>
@@ -34586,7 +34133,6 @@
           <cell r="A441" t="str">
             <v>S-2026-05-65</v>
           </cell>
-          <cell r="B441"/>
           <cell r="C441" t="str">
             <v>RPRO-260520-0197</v>
           </cell>
@@ -34655,7 +34201,6 @@
           <cell r="A442" t="str">
             <v>S-2026-05-66</v>
           </cell>
-          <cell r="B442"/>
           <cell r="C442" t="str">
             <v>RPRO-260520-0225</v>
           </cell>
@@ -34724,7 +34269,6 @@
           <cell r="A443" t="str">
             <v>S-2026-05-67</v>
           </cell>
-          <cell r="B443"/>
           <cell r="C443" t="str">
             <v>RPRO-260520-0226</v>
           </cell>
@@ -34793,7 +34337,6 @@
           <cell r="A444" t="str">
             <v>S-2026-05-68</v>
           </cell>
-          <cell r="B444"/>
           <cell r="C444" t="str">
             <v>RPRO-260520-0227</v>
           </cell>
@@ -34862,7 +34405,6 @@
           <cell r="A445" t="str">
             <v>S-2026-05-69</v>
           </cell>
-          <cell r="B445"/>
           <cell r="C445" t="str">
             <v>RPRO-260520-0228</v>
           </cell>
@@ -34931,7 +34473,6 @@
           <cell r="A446" t="str">
             <v>S-2026-05-70</v>
           </cell>
-          <cell r="B446"/>
           <cell r="C446" t="str">
             <v>RPRO-260520-0229</v>
           </cell>
@@ -35000,7 +34541,6 @@
           <cell r="A447" t="str">
             <v>S-2026-05-71</v>
           </cell>
-          <cell r="B447"/>
           <cell r="C447" t="str">
             <v>RPRO-260521-0669</v>
           </cell>
@@ -35069,7 +34609,6 @@
           <cell r="A448" t="str">
             <v>S-2026-05-72</v>
           </cell>
-          <cell r="B448"/>
           <cell r="C448" t="str">
             <v>RPRO-260521-0670</v>
           </cell>
@@ -35138,7 +34677,6 @@
           <cell r="A449" t="str">
             <v>S-2026-05-73</v>
           </cell>
-          <cell r="B449"/>
           <cell r="C449" t="str">
             <v>RPRO-260523-0221</v>
           </cell>
@@ -35207,7 +34745,6 @@
           <cell r="A450" t="str">
             <v>S-2026-05-74</v>
           </cell>
-          <cell r="B450"/>
           <cell r="C450" t="str">
             <v>RPRO-260523-0222</v>
           </cell>
@@ -35276,7 +34813,6 @@
           <cell r="A451" t="str">
             <v>S-2026-05-75</v>
           </cell>
-          <cell r="B451"/>
           <cell r="C451" t="str">
             <v>RPRO-260523-0223</v>
           </cell>
@@ -35345,7 +34881,6 @@
           <cell r="A452" t="str">
             <v>S-2026-05-76</v>
           </cell>
-          <cell r="B452"/>
           <cell r="C452" t="str">
             <v>RPRO-260526-0394</v>
           </cell>
@@ -35414,7 +34949,6 @@
           <cell r="A453" t="str">
             <v>S-2026-05-77</v>
           </cell>
-          <cell r="B453"/>
           <cell r="C453" t="str">
             <v>RPRO-260526-0395</v>
           </cell>
@@ -35483,7 +35017,6 @@
           <cell r="A454" t="str">
             <v>S-2026-05-78</v>
           </cell>
-          <cell r="B454"/>
           <cell r="C454" t="str">
             <v>RPRO-260526-0396</v>
           </cell>
@@ -35552,7 +35085,6 @@
           <cell r="A455" t="str">
             <v>S-2026-05-79</v>
           </cell>
-          <cell r="B455"/>
           <cell r="C455" t="str">
             <v>RPRO-260526-0397</v>
           </cell>
@@ -35621,7 +35153,6 @@
           <cell r="A456" t="str">
             <v>S-2026-05-80</v>
           </cell>
-          <cell r="B456"/>
           <cell r="C456" t="str">
             <v>RPRO-260526-0398</v>
           </cell>
@@ -35690,7 +35221,6 @@
           <cell r="A457" t="str">
             <v>S-2026-05-81</v>
           </cell>
-          <cell r="B457"/>
           <cell r="C457" t="str">
             <v>RPRO-260526-0399</v>
           </cell>
@@ -35830,7 +35360,6 @@
           <cell r="A459" t="str">
             <v>S-2026-05-83</v>
           </cell>
-          <cell r="B459"/>
           <cell r="C459" t="str">
             <v>RPRO-260526-0401</v>
           </cell>
@@ -35970,7 +35499,6 @@
           <cell r="A461" t="str">
             <v>S-2026-05-85</v>
           </cell>
-          <cell r="B461"/>
           <cell r="C461" t="str">
             <v>RPRO-260526-0402</v>
           </cell>
@@ -36039,7 +35567,6 @@
           <cell r="A462" t="str">
             <v>S-2026-05-86</v>
           </cell>
-          <cell r="B462"/>
           <cell r="C462" t="str">
             <v>RPRO-260527-0578</v>
           </cell>
@@ -36108,7 +35635,6 @@
           <cell r="A463" t="str">
             <v>S-2026-05-87</v>
           </cell>
-          <cell r="B463"/>
           <cell r="C463" t="str">
             <v>RPRO-260527-0579</v>
           </cell>
@@ -36177,7 +35703,6 @@
           <cell r="A464" t="str">
             <v>S-2026-05-88</v>
           </cell>
-          <cell r="B464"/>
           <cell r="C464" t="str">
             <v>RPRO-260527-0580</v>
           </cell>
@@ -36246,7 +35771,6 @@
           <cell r="A465" t="str">
             <v>S-2026-05-89</v>
           </cell>
-          <cell r="B465"/>
           <cell r="C465" t="str">
             <v>RPRO-260527-0581</v>
           </cell>
@@ -36315,7 +35839,6 @@
           <cell r="A466" t="str">
             <v>S-2026-05-90</v>
           </cell>
-          <cell r="B466"/>
           <cell r="C466" t="str">
             <v>RPRO-260527-0582</v>
           </cell>
@@ -36384,7 +35907,6 @@
           <cell r="A467" t="str">
             <v>S-2026-05-91</v>
           </cell>
-          <cell r="B467"/>
           <cell r="C467" t="str">
             <v>RPRO-260527-0583</v>
           </cell>
@@ -36453,7 +35975,6 @@
           <cell r="A468" t="str">
             <v>S-2026-05-92</v>
           </cell>
-          <cell r="B468"/>
           <cell r="C468" t="str">
             <v>RPRO-260528-0001</v>
           </cell>
@@ -36522,7 +36043,6 @@
           <cell r="A469" t="str">
             <v>S-2026-05-93</v>
           </cell>
-          <cell r="B469"/>
           <cell r="C469" t="str">
             <v>RPRO-260529-0339</v>
           </cell>
@@ -36591,7 +36111,6 @@
           <cell r="A470" t="str">
             <v>S-2026-05-94</v>
           </cell>
-          <cell r="B470"/>
           <cell r="C470" t="str">
             <v>RPRO-260529-0340</v>
           </cell>
@@ -36731,7 +36250,6 @@
           <cell r="A472" t="str">
             <v>S-2026-05-96</v>
           </cell>
-          <cell r="B472"/>
           <cell r="C472" t="str">
             <v>RPRO-260529-0342</v>
           </cell>
@@ -36800,7 +36318,6 @@
           <cell r="A473" t="str">
             <v>S-2026-05-97</v>
           </cell>
-          <cell r="B473"/>
           <cell r="C473" t="str">
             <v>RPRO-260529-0343</v>
           </cell>
@@ -37011,7 +36528,6 @@
           <cell r="A476" t="str">
             <v>S-2026-05-100</v>
           </cell>
-          <cell r="B476"/>
           <cell r="C476" t="str">
             <v>RPRO-260529-0346</v>
           </cell>
@@ -37080,7 +36596,6 @@
           <cell r="A477" t="str">
             <v>S-2026-05-102</v>
           </cell>
-          <cell r="B477"/>
           <cell r="C477" t="str">
             <v>RPRO-260601-0847</v>
           </cell>
@@ -37149,7 +36664,6 @@
           <cell r="A478" t="str">
             <v>S-2026-05-103</v>
           </cell>
-          <cell r="B478"/>
           <cell r="C478" t="str">
             <v>RPRO-260601-0848</v>
           </cell>
@@ -37218,7 +36732,6 @@
           <cell r="A479" t="str">
             <v>S-2026-05-104</v>
           </cell>
-          <cell r="B479"/>
           <cell r="C479" t="str">
             <v>RPRO-260601-0849</v>
           </cell>
@@ -37287,7 +36800,6 @@
           <cell r="A480" t="str">
             <v>S-2026-05-105</v>
           </cell>
-          <cell r="B480"/>
           <cell r="C480" t="str">
             <v>RPRO-260601-0850</v>
           </cell>
@@ -37356,7 +36868,6 @@
           <cell r="A481" t="str">
             <v>S-2026-05-106</v>
           </cell>
-          <cell r="B481"/>
           <cell r="C481" t="str">
             <v>RPRO-260601-0851</v>
           </cell>
@@ -37425,7 +36936,6 @@
           <cell r="A482" t="str">
             <v>S-2026-06-01</v>
           </cell>
-          <cell r="B482"/>
           <cell r="C482" t="str">
             <v>RPRO-260602-0720</v>
           </cell>
@@ -37495,7 +37005,6 @@
           <cell r="A483" t="str">
             <v>S-2026-06-02</v>
           </cell>
-          <cell r="B483"/>
           <cell r="C483" t="str">
             <v>RPRO-260602-0721</v>
           </cell>
@@ -37564,7 +37073,6 @@
           <cell r="A484" t="str">
             <v>S-2026-06-03</v>
           </cell>
-          <cell r="B484"/>
           <cell r="C484" t="str">
             <v>RPRO-260602-0722</v>
           </cell>
@@ -37633,7 +37141,6 @@
           <cell r="A485" t="str">
             <v>S-2026-06-04</v>
           </cell>
-          <cell r="B485"/>
           <cell r="C485" t="str">
             <v>RPRO-260602-0723</v>
           </cell>
@@ -37702,7 +37209,6 @@
           <cell r="A486" t="str">
             <v>S-2026-06-05</v>
           </cell>
-          <cell r="B486"/>
           <cell r="C486" t="str">
             <v>RPRO-260602-0724</v>
           </cell>
@@ -37771,7 +37277,6 @@
           <cell r="A487" t="str">
             <v>S-2026-06-06</v>
           </cell>
-          <cell r="B487"/>
           <cell r="C487" t="str">
             <v>RPRO-260602-0725</v>
           </cell>
@@ -37840,7 +37345,6 @@
           <cell r="A488" t="str">
             <v>S-2026-06-07</v>
           </cell>
-          <cell r="B488"/>
           <cell r="C488" t="str">
             <v>RPRO-260602-0726</v>
           </cell>
@@ -37909,7 +37413,6 @@
           <cell r="A489" t="str">
             <v>S-2026-06-08</v>
           </cell>
-          <cell r="B489"/>
           <cell r="C489" t="str">
             <v>RPRO-260602-0727</v>
           </cell>
@@ -38049,7 +37552,6 @@
           <cell r="A491" t="str">
             <v>S-2026-06-10</v>
           </cell>
-          <cell r="B491"/>
           <cell r="C491" t="str">
             <v>RPRO-260603-0482</v>
           </cell>
@@ -38118,7 +37620,6 @@
           <cell r="A492" t="str">
             <v>S-2026-06-11</v>
           </cell>
-          <cell r="B492"/>
           <cell r="C492" t="str">
             <v>RPRO-260603-0483</v>
           </cell>
@@ -38187,7 +37688,6 @@
           <cell r="A493" t="str">
             <v>S-2026-06-12</v>
           </cell>
-          <cell r="B493"/>
           <cell r="C493" t="str">
             <v>RPRO-260603-0484</v>
           </cell>
@@ -38327,7 +37827,6 @@
           <cell r="A495" t="str">
             <v>S-2026-06-15</v>
           </cell>
-          <cell r="B495"/>
           <cell r="C495" t="str">
             <v>RPRO-260604-0522</v>
           </cell>
@@ -38396,7 +37895,6 @@
           <cell r="A496" t="str">
             <v>L-2026-06-01</v>
           </cell>
-          <cell r="B496"/>
           <cell r="C496" t="str">
             <v>RPRO-260604-0523</v>
           </cell>
@@ -38427,8 +37925,6 @@
           <cell r="L496" t="str">
             <v>NIKE-POU CHEN VÀ CONVERSE</v>
           </cell>
-          <cell r="M496"/>
-          <cell r="N496"/>
           <cell r="O496" t="str">
             <v>Lab test</v>
           </cell>
@@ -38461,7 +37957,6 @@
           <cell r="A497" t="str">
             <v>L-2026-06-02</v>
           </cell>
-          <cell r="B497"/>
           <cell r="C497" t="str">
             <v>RPRO-260604-0524</v>
           </cell>
@@ -38492,8 +37987,6 @@
           <cell r="L497" t="str">
             <v>NIKE-POU CHEN VÀ CONVERSE</v>
           </cell>
-          <cell r="M497"/>
-          <cell r="N497"/>
           <cell r="O497" t="str">
             <v>Lab test</v>
           </cell>
@@ -38526,7 +38019,6 @@
           <cell r="A498" t="str">
             <v>L-2026-06-03</v>
           </cell>
-          <cell r="B498"/>
           <cell r="C498" t="str">
             <v>RPRO-260604-0525</v>
           </cell>
@@ -38557,8 +38049,6 @@
           <cell r="L498" t="str">
             <v>NIKE-POU CHEN VÀ CONVERSE</v>
           </cell>
-          <cell r="M498"/>
-          <cell r="N498"/>
           <cell r="O498" t="str">
             <v>Lab test</v>
           </cell>
@@ -38591,7 +38081,6 @@
           <cell r="A499" t="str">
             <v>L-2026-06-04</v>
           </cell>
-          <cell r="B499"/>
           <cell r="C499" t="str">
             <v>RPRO-260604-0526</v>
           </cell>
@@ -38622,8 +38111,6 @@
           <cell r="L499" t="str">
             <v>NIKE-POU CHEN VÀ CONVERSE</v>
           </cell>
-          <cell r="M499"/>
-          <cell r="N499"/>
           <cell r="O499" t="str">
             <v>Lab test</v>
           </cell>
@@ -38656,7 +38143,6 @@
           <cell r="A500" t="str">
             <v>L-2026-06-05</v>
           </cell>
-          <cell r="B500"/>
           <cell r="C500" t="str">
             <v>RPRO-260604-0527</v>
           </cell>
@@ -38687,8 +38173,6 @@
           <cell r="L500" t="str">
             <v>NIKE-POU CHEN VÀ CONVERSE</v>
           </cell>
-          <cell r="M500"/>
-          <cell r="N500"/>
           <cell r="O500" t="str">
             <v>Lab test</v>
           </cell>
@@ -38721,7 +38205,6 @@
           <cell r="A501" t="str">
             <v>L-2026-06-06</v>
           </cell>
-          <cell r="B501"/>
           <cell r="C501" t="str">
             <v>RPRO-260604-0528</v>
           </cell>
@@ -38752,8 +38235,6 @@
           <cell r="L501" t="str">
             <v>NIKE-POU CHEN VÀ CONVERSE</v>
           </cell>
-          <cell r="M501"/>
-          <cell r="N501"/>
           <cell r="O501" t="str">
             <v>Lab test</v>
           </cell>
@@ -38786,7 +38267,6 @@
           <cell r="A502" t="str">
             <v>L-2026-06-07</v>
           </cell>
-          <cell r="B502"/>
           <cell r="C502" t="str">
             <v>RPRO-260604-0529</v>
           </cell>
@@ -38817,8 +38297,6 @@
           <cell r="L502" t="str">
             <v>SHYANG HUNG TAH</v>
           </cell>
-          <cell r="M502"/>
-          <cell r="N502"/>
           <cell r="O502" t="str">
             <v>Lab test</v>
           </cell>
@@ -38851,7 +38329,6 @@
           <cell r="A503" t="str">
             <v>S-2026-06-16</v>
           </cell>
-          <cell r="B503"/>
           <cell r="C503" t="str">
             <v>RPRO-260605-0678</v>
           </cell>
@@ -38920,7 +38397,6 @@
           <cell r="A504" t="str">
             <v>S-2026-06-17</v>
           </cell>
-          <cell r="B504"/>
           <cell r="C504" t="str">
             <v>RPRO-260605-0679</v>
           </cell>
@@ -38989,7 +38465,6 @@
           <cell r="A505" t="str">
             <v>S-2026-06-18</v>
           </cell>
-          <cell r="B505"/>
           <cell r="C505" t="str">
             <v>RPRO-260605-0680</v>
           </cell>
@@ -39058,7 +38533,6 @@
           <cell r="A506" t="str">
             <v>S-2026-06-19</v>
           </cell>
-          <cell r="B506"/>
           <cell r="C506" t="str">
             <v>RPRO-260605-0681</v>
           </cell>
@@ -39127,7 +38601,6 @@
           <cell r="A507" t="str">
             <v>S-2026-06-20</v>
           </cell>
-          <cell r="B507"/>
           <cell r="C507" t="str">
             <v>RPRO-260605-0682</v>
           </cell>
@@ -39196,7 +38669,6 @@
           <cell r="A508" t="str">
             <v>S-2026-06-21</v>
           </cell>
-          <cell r="B508"/>
           <cell r="C508" t="str">
             <v>RPRO-260605-0683</v>
           </cell>
@@ -39265,7 +38737,6 @@
           <cell r="A509" t="str">
             <v>S-2026-06-22</v>
           </cell>
-          <cell r="B509"/>
           <cell r="C509" t="str">
             <v>RPRO-260605-0684</v>
           </cell>
@@ -39334,7 +38805,6 @@
           <cell r="A510" t="str">
             <v>S-2026-06-23</v>
           </cell>
-          <cell r="B510"/>
           <cell r="C510" t="str">
             <v>RPRO-260605-0685</v>
           </cell>
@@ -39403,7 +38873,6 @@
           <cell r="A511" t="str">
             <v>S-2026-06-24</v>
           </cell>
-          <cell r="B511"/>
           <cell r="C511" t="str">
             <v>RPRO-260605-0686</v>
           </cell>
@@ -39472,7 +38941,6 @@
           <cell r="A512" t="str">
             <v>S-2026-06-25</v>
           </cell>
-          <cell r="B512"/>
           <cell r="C512" t="str">
             <v>RPRO-260606-0217</v>
           </cell>
@@ -39541,7 +39009,6 @@
           <cell r="A513" t="str">
             <v>S-2026-06-26</v>
           </cell>
-          <cell r="B513"/>
           <cell r="C513" t="str">
             <v>RPRO-260608-1016</v>
           </cell>
@@ -39610,7 +39077,6 @@
           <cell r="A514" t="str">
             <v>S-2026-06-27</v>
           </cell>
-          <cell r="B514"/>
           <cell r="C514" t="str">
             <v>RPRO-260608-1017</v>
           </cell>
@@ -39679,7 +39145,6 @@
           <cell r="A515" t="str">
             <v>S-2026-06-28</v>
           </cell>
-          <cell r="B515"/>
           <cell r="C515" t="str">
             <v>RPRO-260608-1018</v>
           </cell>
@@ -39748,7 +39213,6 @@
           <cell r="A516" t="str">
             <v>S-2026-06-29</v>
           </cell>
-          <cell r="B516"/>
           <cell r="C516" t="str">
             <v>RPRO-260608-1019</v>
           </cell>
@@ -39817,7 +39281,6 @@
           <cell r="A517" t="str">
             <v>S-2026-06-30</v>
           </cell>
-          <cell r="B517"/>
           <cell r="C517" t="str">
             <v>RPRO-260608-1020</v>
           </cell>
@@ -39883,95 +39346,30 @@
           </cell>
         </row>
         <row r="518">
-          <cell r="A518"/>
-          <cell r="B518"/>
-          <cell r="C518"/>
-          <cell r="D518"/>
-          <cell r="E518" t="str">
-            <v/>
-          </cell>
-          <cell r="F518"/>
-          <cell r="G518"/>
-          <cell r="H518"/>
-          <cell r="I518"/>
+          <cell r="E518"/>
           <cell r="J518">
             <v>0</v>
           </cell>
           <cell r="K518">
             <v>0</v>
           </cell>
-          <cell r="L518"/>
-          <cell r="M518"/>
-          <cell r="N518"/>
-          <cell r="O518"/>
-          <cell r="P518"/>
-          <cell r="Q518"/>
-          <cell r="R518"/>
-          <cell r="S518"/>
-          <cell r="T518"/>
-          <cell r="U518"/>
-          <cell r="V518"/>
-          <cell r="W518"/>
         </row>
         <row r="519">
-          <cell r="A519"/>
-          <cell r="B519"/>
-          <cell r="C519"/>
-          <cell r="D519"/>
-          <cell r="E519" t="str">
-            <v/>
-          </cell>
-          <cell r="F519"/>
-          <cell r="G519"/>
-          <cell r="H519"/>
-          <cell r="I519"/>
+          <cell r="E519"/>
           <cell r="J519">
             <v>0</v>
           </cell>
           <cell r="K519">
             <v>0</v>
           </cell>
-          <cell r="L519"/>
-          <cell r="M519"/>
-          <cell r="N519"/>
-          <cell r="O519"/>
-          <cell r="P519"/>
-          <cell r="Q519"/>
-          <cell r="R519"/>
-          <cell r="S519"/>
-          <cell r="T519"/>
-          <cell r="U519"/>
-          <cell r="V519"/>
-          <cell r="W519"/>
         </row>
         <row r="520">
-          <cell r="A520"/>
-          <cell r="B520"/>
-          <cell r="C520"/>
-          <cell r="D520"/>
-          <cell r="E520"/>
-          <cell r="F520"/>
-          <cell r="G520"/>
-          <cell r="H520"/>
-          <cell r="I520"/>
           <cell r="J520">
             <v>0</v>
           </cell>
           <cell r="K520">
             <v>0</v>
           </cell>
-          <cell r="L520"/>
-          <cell r="M520"/>
-          <cell r="N520"/>
-          <cell r="O520"/>
-          <cell r="P520"/>
-          <cell r="Q520"/>
-          <cell r="R520"/>
-          <cell r="S520"/>
-          <cell r="T520"/>
-          <cell r="U520"/>
-          <cell r="V520"/>
-          <cell r="W520"/>
         </row>
       </sheetData>
       <sheetData sheetId="4"/>
@@ -40078,7 +39476,13 @@
       <sheetData sheetId="105"/>
       <sheetData sheetId="106"/>
       <sheetData sheetId="107"/>
-      <sheetData sheetId="108"/>
+      <sheetData sheetId="108">
+        <row r="1">
+          <cell r="F1" t="str">
+            <v>No_Item</v>
+          </cell>
+        </row>
+      </sheetData>
       <sheetData sheetId="109"/>
       <sheetData sheetId="110"/>
       <sheetData sheetId="111"/>
@@ -41950,7 +41354,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46182.334269444444</v>
+        <v>46182.483680439815</v>
       </c>
       <c r="D1" s="83" t="s">
         <v>1</v>
@@ -43393,7 +42797,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46182.334269444444</v>
+        <v>46182.483680439815</v>
       </c>
       <c r="D1" s="83" t="s">
         <v>1</v>
@@ -44835,7 +44239,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46182.334269444444</v>
+        <v>46182.483680439815</v>
       </c>
       <c r="D1" s="83" t="s">
         <v>1</v>
@@ -46180,7 +45584,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46182.334269444444</v>
+        <v>46182.483680439815</v>
       </c>
       <c r="D1" s="83" t="s">
         <v>1</v>
@@ -47706,7 +47110,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46182.334269212966</v>
+        <v>46182.483680439815</v>
       </c>
       <c r="D1" s="83" t="s">
         <v>1</v>
@@ -48998,7 +48402,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46182.334269212966</v>
+        <v>46182.483680439815</v>
       </c>
       <c r="D1" s="83" t="s">
         <v>1</v>
@@ -50396,7 +49800,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46182.334269444444</v>
+        <v>46182.483680439815</v>
       </c>
       <c r="D1" s="83" t="s">
         <v>1</v>
@@ -51806,7 +51210,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46182.334269444444</v>
+        <v>46182.483680439815</v>
       </c>
       <c r="D1" s="83" t="s">
         <v>1</v>
@@ -53274,7 +52678,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46182.334269444444</v>
+        <v>46182.483680439815</v>
       </c>
       <c r="D1" s="83" t="s">
         <v>1</v>
@@ -54707,7 +54111,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46182.334269444444</v>
+        <v>46182.483680439815</v>
       </c>
       <c r="D1" s="83" t="s">
         <v>1</v>
@@ -55999,7 +55403,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46182.334269444444</v>
+        <v>46182.483680439815</v>
       </c>
       <c r="D1" s="83" t="s">
         <v>1</v>
@@ -57389,7 +56793,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46182.334269444444</v>
+        <v>46182.483680439815</v>
       </c>
       <c r="D1" s="83" t="s">
         <v>1</v>
@@ -58805,7 +58209,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46182.334269444444</v>
+        <v>46182.483680439815</v>
       </c>
       <c r="D1" s="83" t="s">
         <v>1</v>
@@ -60256,7 +59660,7 @@
       </c>
       <c r="B1" s="1">
         <f ca="1">NOW()</f>
-        <v>46182.334269444444</v>
+        <v>46182.483680439815</v>
       </c>
       <c r="D1" s="83" t="s">
         <v>1</v>

</xml_diff>